<commit_message>
mejora de la plantilla para la carga de usuarios
</commit_message>
<xml_diff>
--- a/public/plantilla_carga_usuarios.xlsx
+++ b/public/plantilla_carga_usuarios.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Usuarios" sheetId="1" r:id="Rb934f466f2bb44b1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="2" r:id="R94b6cc6a4d064a22"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Usuarios" sheetId="1" r:id="R61990382be5440a5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="2" r:id="R419950f374be4233"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -403,8 +403,9 @@
     <x:col min="11" max="11" width="20" hidden="0" customWidth="1"/>
     <x:col min="12" max="12" width="16" hidden="0" customWidth="1"/>
     <x:col min="13" max="13" width="15" hidden="0" customWidth="1"/>
-    <x:col min="14" max="14" width="22" hidden="0" customWidth="1"/>
-    <x:col min="15" max="15" width="23" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="24" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="22" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="23" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
@@ -448,9 +449,12 @@
         <x:v>rei</x:v>
       </x:c>
       <x:c r="N1" s="10" t="str">
+        <x:v>codigo_institucional</x:v>
+      </x:c>
+      <x:c r="O1" s="10" t="str">
         <x:v>rol</x:v>
       </x:c>
-      <x:c r="O1" s="11" t="str">
+      <x:c r="P1" s="11" t="str">
         <x:v>can_create_monitoreo</x:v>
       </x:c>
     </x:row>
@@ -468,8 +472,9 @@
       <x:c r="K2" s="13"/>
       <x:c r="L2" s="13"/>
       <x:c r="M2" s="13"/>
-      <x:c r="N2" s="13"/>
+      <x:c r="N2" s="16"/>
       <x:c r="O2" s="13"/>
+      <x:c r="P2" s="13"/>
     </x:row>
     <x:row r="3" ht="22" customHeight="1">
       <x:c r="A3" s="17"/>
@@ -485,8 +490,9 @@
       <x:c r="K3" s="14"/>
       <x:c r="L3" s="14"/>
       <x:c r="M3" s="14"/>
-      <x:c r="N3" s="14"/>
+      <x:c r="N3" s="17"/>
       <x:c r="O3" s="14"/>
+      <x:c r="P3" s="14"/>
     </x:row>
     <x:row r="4" ht="22" customHeight="1">
       <x:c r="A4" s="17"/>
@@ -502,8 +508,9 @@
       <x:c r="K4" s="14"/>
       <x:c r="L4" s="14"/>
       <x:c r="M4" s="14"/>
-      <x:c r="N4" s="14"/>
+      <x:c r="N4" s="17"/>
       <x:c r="O4" s="14"/>
+      <x:c r="P4" s="14"/>
     </x:row>
     <x:row r="5" ht="22" customHeight="1">
       <x:c r="A5" s="17"/>
@@ -519,8 +526,9 @@
       <x:c r="K5" s="14"/>
       <x:c r="L5" s="14"/>
       <x:c r="M5" s="14"/>
-      <x:c r="N5" s="14"/>
+      <x:c r="N5" s="17"/>
       <x:c r="O5" s="14"/>
+      <x:c r="P5" s="14"/>
     </x:row>
     <x:row r="6" ht="22" customHeight="1">
       <x:c r="A6" s="17"/>
@@ -536,8 +544,9 @@
       <x:c r="K6" s="14"/>
       <x:c r="L6" s="14"/>
       <x:c r="M6" s="14"/>
-      <x:c r="N6" s="14"/>
+      <x:c r="N6" s="17"/>
       <x:c r="O6" s="14"/>
+      <x:c r="P6" s="14"/>
     </x:row>
     <x:row r="7" ht="22" customHeight="1">
       <x:c r="A7" s="17"/>
@@ -553,8 +562,9 @@
       <x:c r="K7" s="14"/>
       <x:c r="L7" s="14"/>
       <x:c r="M7" s="14"/>
-      <x:c r="N7" s="14"/>
+      <x:c r="N7" s="17"/>
       <x:c r="O7" s="14"/>
+      <x:c r="P7" s="14"/>
     </x:row>
     <x:row r="8" ht="22" customHeight="1">
       <x:c r="A8" s="17"/>
@@ -570,8 +580,9 @@
       <x:c r="K8" s="14"/>
       <x:c r="L8" s="14"/>
       <x:c r="M8" s="14"/>
-      <x:c r="N8" s="14"/>
+      <x:c r="N8" s="17"/>
       <x:c r="O8" s="14"/>
+      <x:c r="P8" s="14"/>
     </x:row>
     <x:row r="9" ht="22" customHeight="1">
       <x:c r="A9" s="17"/>
@@ -587,8 +598,9 @@
       <x:c r="K9" s="14"/>
       <x:c r="L9" s="14"/>
       <x:c r="M9" s="14"/>
-      <x:c r="N9" s="14"/>
+      <x:c r="N9" s="17"/>
       <x:c r="O9" s="14"/>
+      <x:c r="P9" s="14"/>
     </x:row>
     <x:row r="10" ht="22" customHeight="1">
       <x:c r="A10" s="17"/>
@@ -604,8 +616,9 @@
       <x:c r="K10" s="14"/>
       <x:c r="L10" s="14"/>
       <x:c r="M10" s="14"/>
-      <x:c r="N10" s="14"/>
+      <x:c r="N10" s="17"/>
       <x:c r="O10" s="14"/>
+      <x:c r="P10" s="14"/>
     </x:row>
     <x:row r="11" ht="22" customHeight="1">
       <x:c r="A11" s="17"/>
@@ -621,8 +634,9 @@
       <x:c r="K11" s="14"/>
       <x:c r="L11" s="14"/>
       <x:c r="M11" s="14"/>
-      <x:c r="N11" s="14"/>
+      <x:c r="N11" s="17"/>
       <x:c r="O11" s="14"/>
+      <x:c r="P11" s="14"/>
     </x:row>
     <x:row r="12" ht="22" customHeight="1">
       <x:c r="A12" s="17"/>
@@ -638,8 +652,9 @@
       <x:c r="K12" s="14"/>
       <x:c r="L12" s="14"/>
       <x:c r="M12" s="14"/>
-      <x:c r="N12" s="14"/>
+      <x:c r="N12" s="17"/>
       <x:c r="O12" s="14"/>
+      <x:c r="P12" s="14"/>
     </x:row>
     <x:row r="13" ht="22" customHeight="1">
       <x:c r="A13" s="17"/>
@@ -655,8 +670,9 @@
       <x:c r="K13" s="14"/>
       <x:c r="L13" s="14"/>
       <x:c r="M13" s="14"/>
-      <x:c r="N13" s="14"/>
+      <x:c r="N13" s="17"/>
       <x:c r="O13" s="14"/>
+      <x:c r="P13" s="14"/>
     </x:row>
     <x:row r="14" ht="22" customHeight="1">
       <x:c r="A14" s="17"/>
@@ -672,8 +688,9 @@
       <x:c r="K14" s="14"/>
       <x:c r="L14" s="14"/>
       <x:c r="M14" s="14"/>
-      <x:c r="N14" s="14"/>
+      <x:c r="N14" s="17"/>
       <x:c r="O14" s="14"/>
+      <x:c r="P14" s="14"/>
     </x:row>
     <x:row r="15" ht="22" customHeight="1">
       <x:c r="A15" s="17"/>
@@ -689,8 +706,9 @@
       <x:c r="K15" s="14"/>
       <x:c r="L15" s="14"/>
       <x:c r="M15" s="14"/>
-      <x:c r="N15" s="14"/>
+      <x:c r="N15" s="17"/>
       <x:c r="O15" s="14"/>
+      <x:c r="P15" s="14"/>
     </x:row>
     <x:row r="16" ht="22" customHeight="1">
       <x:c r="A16" s="17"/>
@@ -706,8 +724,9 @@
       <x:c r="K16" s="14"/>
       <x:c r="L16" s="14"/>
       <x:c r="M16" s="14"/>
-      <x:c r="N16" s="14"/>
+      <x:c r="N16" s="17"/>
       <x:c r="O16" s="14"/>
+      <x:c r="P16" s="14"/>
     </x:row>
     <x:row r="17" ht="22" customHeight="1">
       <x:c r="A17" s="17"/>
@@ -723,8 +742,9 @@
       <x:c r="K17" s="14"/>
       <x:c r="L17" s="14"/>
       <x:c r="M17" s="14"/>
-      <x:c r="N17" s="14"/>
+      <x:c r="N17" s="17"/>
       <x:c r="O17" s="14"/>
+      <x:c r="P17" s="14"/>
     </x:row>
     <x:row r="18" ht="22" customHeight="1">
       <x:c r="A18" s="17"/>
@@ -740,8 +760,9 @@
       <x:c r="K18" s="14"/>
       <x:c r="L18" s="14"/>
       <x:c r="M18" s="14"/>
-      <x:c r="N18" s="14"/>
+      <x:c r="N18" s="17"/>
       <x:c r="O18" s="14"/>
+      <x:c r="P18" s="14"/>
     </x:row>
     <x:row r="19" ht="22" customHeight="1">
       <x:c r="A19" s="17"/>
@@ -757,8 +778,9 @@
       <x:c r="K19" s="14"/>
       <x:c r="L19" s="14"/>
       <x:c r="M19" s="14"/>
-      <x:c r="N19" s="14"/>
+      <x:c r="N19" s="17"/>
       <x:c r="O19" s="14"/>
+      <x:c r="P19" s="14"/>
     </x:row>
     <x:row r="20" ht="22" customHeight="1">
       <x:c r="A20" s="17"/>
@@ -774,8 +796,9 @@
       <x:c r="K20" s="14"/>
       <x:c r="L20" s="14"/>
       <x:c r="M20" s="14"/>
-      <x:c r="N20" s="14"/>
+      <x:c r="N20" s="17"/>
       <x:c r="O20" s="14"/>
+      <x:c r="P20" s="14"/>
     </x:row>
     <x:row r="21" ht="22" customHeight="1">
       <x:c r="A21" s="17"/>
@@ -791,8 +814,9 @@
       <x:c r="K21" s="14"/>
       <x:c r="L21" s="14"/>
       <x:c r="M21" s="14"/>
-      <x:c r="N21" s="14"/>
+      <x:c r="N21" s="17"/>
       <x:c r="O21" s="14"/>
+      <x:c r="P21" s="14"/>
     </x:row>
     <x:row r="22" ht="22" customHeight="1">
       <x:c r="A22" s="17"/>
@@ -808,8 +832,9 @@
       <x:c r="K22" s="14"/>
       <x:c r="L22" s="14"/>
       <x:c r="M22" s="14"/>
-      <x:c r="N22" s="14"/>
+      <x:c r="N22" s="17"/>
       <x:c r="O22" s="14"/>
+      <x:c r="P22" s="14"/>
     </x:row>
     <x:row r="23" ht="22" customHeight="1">
       <x:c r="A23" s="17"/>
@@ -825,8 +850,9 @@
       <x:c r="K23" s="14"/>
       <x:c r="L23" s="14"/>
       <x:c r="M23" s="14"/>
-      <x:c r="N23" s="14"/>
+      <x:c r="N23" s="17"/>
       <x:c r="O23" s="14"/>
+      <x:c r="P23" s="14"/>
     </x:row>
     <x:row r="24" ht="22" customHeight="1">
       <x:c r="A24" s="17"/>
@@ -842,8 +868,9 @@
       <x:c r="K24" s="14"/>
       <x:c r="L24" s="14"/>
       <x:c r="M24" s="14"/>
-      <x:c r="N24" s="14"/>
+      <x:c r="N24" s="17"/>
       <x:c r="O24" s="14"/>
+      <x:c r="P24" s="14"/>
     </x:row>
     <x:row r="25" ht="22" customHeight="1">
       <x:c r="A25" s="17"/>
@@ -859,8 +886,9 @@
       <x:c r="K25" s="14"/>
       <x:c r="L25" s="14"/>
       <x:c r="M25" s="14"/>
-      <x:c r="N25" s="14"/>
+      <x:c r="N25" s="17"/>
       <x:c r="O25" s="14"/>
+      <x:c r="P25" s="14"/>
     </x:row>
     <x:row r="26" ht="22" customHeight="1">
       <x:c r="A26" s="17"/>
@@ -876,8 +904,9 @@
       <x:c r="K26" s="14"/>
       <x:c r="L26" s="14"/>
       <x:c r="M26" s="14"/>
-      <x:c r="N26" s="14"/>
+      <x:c r="N26" s="17"/>
       <x:c r="O26" s="14"/>
+      <x:c r="P26" s="14"/>
     </x:row>
     <x:row r="27" ht="22" customHeight="1">
       <x:c r="A27" s="17"/>
@@ -893,8 +922,9 @@
       <x:c r="K27" s="14"/>
       <x:c r="L27" s="14"/>
       <x:c r="M27" s="14"/>
-      <x:c r="N27" s="14"/>
+      <x:c r="N27" s="17"/>
       <x:c r="O27" s="14"/>
+      <x:c r="P27" s="14"/>
     </x:row>
     <x:row r="28" ht="22" customHeight="1">
       <x:c r="A28" s="17"/>
@@ -910,8 +940,9 @@
       <x:c r="K28" s="14"/>
       <x:c r="L28" s="14"/>
       <x:c r="M28" s="14"/>
-      <x:c r="N28" s="14"/>
+      <x:c r="N28" s="17"/>
       <x:c r="O28" s="14"/>
+      <x:c r="P28" s="14"/>
     </x:row>
     <x:row r="29" ht="22" customHeight="1">
       <x:c r="A29" s="17"/>
@@ -927,8 +958,9 @@
       <x:c r="K29" s="14"/>
       <x:c r="L29" s="14"/>
       <x:c r="M29" s="14"/>
-      <x:c r="N29" s="14"/>
+      <x:c r="N29" s="17"/>
       <x:c r="O29" s="14"/>
+      <x:c r="P29" s="14"/>
     </x:row>
     <x:row r="30" ht="22" customHeight="1">
       <x:c r="A30" s="17"/>
@@ -944,8 +976,9 @@
       <x:c r="K30" s="14"/>
       <x:c r="L30" s="14"/>
       <x:c r="M30" s="14"/>
-      <x:c r="N30" s="14"/>
+      <x:c r="N30" s="17"/>
       <x:c r="O30" s="14"/>
+      <x:c r="P30" s="14"/>
     </x:row>
     <x:row r="31" ht="22" customHeight="1">
       <x:c r="A31" s="17"/>
@@ -961,8 +994,9 @@
       <x:c r="K31" s="14"/>
       <x:c r="L31" s="14"/>
       <x:c r="M31" s="14"/>
-      <x:c r="N31" s="14"/>
+      <x:c r="N31" s="17"/>
       <x:c r="O31" s="14"/>
+      <x:c r="P31" s="14"/>
     </x:row>
     <x:row r="32" ht="22" customHeight="1">
       <x:c r="A32" s="17"/>
@@ -978,8 +1012,9 @@
       <x:c r="K32" s="14"/>
       <x:c r="L32" s="14"/>
       <x:c r="M32" s="14"/>
-      <x:c r="N32" s="14"/>
+      <x:c r="N32" s="17"/>
       <x:c r="O32" s="14"/>
+      <x:c r="P32" s="14"/>
     </x:row>
     <x:row r="33" ht="22" customHeight="1">
       <x:c r="A33" s="17"/>
@@ -995,8 +1030,9 @@
       <x:c r="K33" s="14"/>
       <x:c r="L33" s="14"/>
       <x:c r="M33" s="14"/>
-      <x:c r="N33" s="14"/>
+      <x:c r="N33" s="17"/>
       <x:c r="O33" s="14"/>
+      <x:c r="P33" s="14"/>
     </x:row>
     <x:row r="34" ht="22" customHeight="1">
       <x:c r="A34" s="17"/>
@@ -1012,8 +1048,9 @@
       <x:c r="K34" s="14"/>
       <x:c r="L34" s="14"/>
       <x:c r="M34" s="14"/>
-      <x:c r="N34" s="14"/>
+      <x:c r="N34" s="17"/>
       <x:c r="O34" s="14"/>
+      <x:c r="P34" s="14"/>
     </x:row>
     <x:row r="35" ht="22" customHeight="1">
       <x:c r="A35" s="17"/>
@@ -1029,8 +1066,9 @@
       <x:c r="K35" s="14"/>
       <x:c r="L35" s="14"/>
       <x:c r="M35" s="14"/>
-      <x:c r="N35" s="14"/>
+      <x:c r="N35" s="17"/>
       <x:c r="O35" s="14"/>
+      <x:c r="P35" s="14"/>
     </x:row>
     <x:row r="36" ht="22" customHeight="1">
       <x:c r="A36" s="17"/>
@@ -1046,8 +1084,9 @@
       <x:c r="K36" s="14"/>
       <x:c r="L36" s="14"/>
       <x:c r="M36" s="14"/>
-      <x:c r="N36" s="14"/>
+      <x:c r="N36" s="17"/>
       <x:c r="O36" s="14"/>
+      <x:c r="P36" s="14"/>
     </x:row>
     <x:row r="37" ht="22" customHeight="1">
       <x:c r="A37" s="17"/>
@@ -1063,8 +1102,9 @@
       <x:c r="K37" s="14"/>
       <x:c r="L37" s="14"/>
       <x:c r="M37" s="14"/>
-      <x:c r="N37" s="14"/>
+      <x:c r="N37" s="17"/>
       <x:c r="O37" s="14"/>
+      <x:c r="P37" s="14"/>
     </x:row>
     <x:row r="38" ht="22" customHeight="1">
       <x:c r="A38" s="17"/>
@@ -1080,8 +1120,9 @@
       <x:c r="K38" s="14"/>
       <x:c r="L38" s="14"/>
       <x:c r="M38" s="14"/>
-      <x:c r="N38" s="14"/>
+      <x:c r="N38" s="17"/>
       <x:c r="O38" s="14"/>
+      <x:c r="P38" s="14"/>
     </x:row>
     <x:row r="39" ht="22" customHeight="1">
       <x:c r="A39" s="17"/>
@@ -1097,8 +1138,9 @@
       <x:c r="K39" s="14"/>
       <x:c r="L39" s="14"/>
       <x:c r="M39" s="14"/>
-      <x:c r="N39" s="14"/>
+      <x:c r="N39" s="17"/>
       <x:c r="O39" s="14"/>
+      <x:c r="P39" s="14"/>
     </x:row>
     <x:row r="40" ht="22" customHeight="1">
       <x:c r="A40" s="17"/>
@@ -1114,8 +1156,9 @@
       <x:c r="K40" s="14"/>
       <x:c r="L40" s="14"/>
       <x:c r="M40" s="14"/>
-      <x:c r="N40" s="14"/>
+      <x:c r="N40" s="17"/>
       <x:c r="O40" s="14"/>
+      <x:c r="P40" s="14"/>
     </x:row>
     <x:row r="41" ht="22" customHeight="1">
       <x:c r="A41" s="17"/>
@@ -1131,8 +1174,9 @@
       <x:c r="K41" s="14"/>
       <x:c r="L41" s="14"/>
       <x:c r="M41" s="14"/>
-      <x:c r="N41" s="14"/>
+      <x:c r="N41" s="17"/>
       <x:c r="O41" s="14"/>
+      <x:c r="P41" s="14"/>
     </x:row>
     <x:row r="42" ht="22" customHeight="1">
       <x:c r="A42" s="17"/>
@@ -1148,8 +1192,9 @@
       <x:c r="K42" s="14"/>
       <x:c r="L42" s="14"/>
       <x:c r="M42" s="14"/>
-      <x:c r="N42" s="14"/>
+      <x:c r="N42" s="17"/>
       <x:c r="O42" s="14"/>
+      <x:c r="P42" s="14"/>
     </x:row>
     <x:row r="43" ht="22" customHeight="1">
       <x:c r="A43" s="17"/>
@@ -1165,8 +1210,9 @@
       <x:c r="K43" s="14"/>
       <x:c r="L43" s="14"/>
       <x:c r="M43" s="14"/>
-      <x:c r="N43" s="14"/>
+      <x:c r="N43" s="17"/>
       <x:c r="O43" s="14"/>
+      <x:c r="P43" s="14"/>
     </x:row>
     <x:row r="44" ht="22" customHeight="1">
       <x:c r="A44" s="17"/>
@@ -1182,8 +1228,9 @@
       <x:c r="K44" s="14"/>
       <x:c r="L44" s="14"/>
       <x:c r="M44" s="14"/>
-      <x:c r="N44" s="14"/>
+      <x:c r="N44" s="17"/>
       <x:c r="O44" s="14"/>
+      <x:c r="P44" s="14"/>
     </x:row>
     <x:row r="45" ht="22" customHeight="1">
       <x:c r="A45" s="17"/>
@@ -1199,8 +1246,9 @@
       <x:c r="K45" s="14"/>
       <x:c r="L45" s="14"/>
       <x:c r="M45" s="14"/>
-      <x:c r="N45" s="14"/>
+      <x:c r="N45" s="17"/>
       <x:c r="O45" s="14"/>
+      <x:c r="P45" s="14"/>
     </x:row>
     <x:row r="46" ht="22" customHeight="1">
       <x:c r="A46" s="17"/>
@@ -1216,8 +1264,9 @@
       <x:c r="K46" s="14"/>
       <x:c r="L46" s="14"/>
       <x:c r="M46" s="14"/>
-      <x:c r="N46" s="14"/>
+      <x:c r="N46" s="17"/>
       <x:c r="O46" s="14"/>
+      <x:c r="P46" s="14"/>
     </x:row>
     <x:row r="47" ht="22" customHeight="1">
       <x:c r="A47" s="17"/>
@@ -1233,8 +1282,9 @@
       <x:c r="K47" s="14"/>
       <x:c r="L47" s="14"/>
       <x:c r="M47" s="14"/>
-      <x:c r="N47" s="14"/>
+      <x:c r="N47" s="17"/>
       <x:c r="O47" s="14"/>
+      <x:c r="P47" s="14"/>
     </x:row>
     <x:row r="48" ht="22" customHeight="1">
       <x:c r="A48" s="17"/>
@@ -1250,8 +1300,9 @@
       <x:c r="K48" s="14"/>
       <x:c r="L48" s="14"/>
       <x:c r="M48" s="14"/>
-      <x:c r="N48" s="14"/>
+      <x:c r="N48" s="17"/>
       <x:c r="O48" s="14"/>
+      <x:c r="P48" s="14"/>
     </x:row>
     <x:row r="49" ht="22" customHeight="1">
       <x:c r="A49" s="17"/>
@@ -1267,8 +1318,9 @@
       <x:c r="K49" s="14"/>
       <x:c r="L49" s="14"/>
       <x:c r="M49" s="14"/>
-      <x:c r="N49" s="14"/>
+      <x:c r="N49" s="17"/>
       <x:c r="O49" s="14"/>
+      <x:c r="P49" s="14"/>
     </x:row>
     <x:row r="50" ht="22" customHeight="1">
       <x:c r="A50" s="17"/>
@@ -1284,8 +1336,9 @@
       <x:c r="K50" s="14"/>
       <x:c r="L50" s="14"/>
       <x:c r="M50" s="14"/>
-      <x:c r="N50" s="14"/>
+      <x:c r="N50" s="17"/>
       <x:c r="O50" s="14"/>
+      <x:c r="P50" s="14"/>
     </x:row>
     <x:row r="51" ht="22" customHeight="1">
       <x:c r="A51" s="17"/>
@@ -1301,8 +1354,9 @@
       <x:c r="K51" s="14"/>
       <x:c r="L51" s="14"/>
       <x:c r="M51" s="14"/>
-      <x:c r="N51" s="14"/>
+      <x:c r="N51" s="17"/>
       <x:c r="O51" s="14"/>
+      <x:c r="P51" s="14"/>
     </x:row>
     <x:row r="52" ht="22" customHeight="1">
       <x:c r="A52" s="17"/>
@@ -1318,8 +1372,9 @@
       <x:c r="K52" s="14"/>
       <x:c r="L52" s="14"/>
       <x:c r="M52" s="14"/>
-      <x:c r="N52" s="14"/>
+      <x:c r="N52" s="17"/>
       <x:c r="O52" s="14"/>
+      <x:c r="P52" s="14"/>
     </x:row>
     <x:row r="53" ht="22" customHeight="1">
       <x:c r="A53" s="17"/>
@@ -1335,8 +1390,9 @@
       <x:c r="K53" s="14"/>
       <x:c r="L53" s="14"/>
       <x:c r="M53" s="14"/>
-      <x:c r="N53" s="14"/>
+      <x:c r="N53" s="17"/>
       <x:c r="O53" s="14"/>
+      <x:c r="P53" s="14"/>
     </x:row>
     <x:row r="54" ht="22" customHeight="1">
       <x:c r="A54" s="17"/>
@@ -1352,8 +1408,9 @@
       <x:c r="K54" s="14"/>
       <x:c r="L54" s="14"/>
       <x:c r="M54" s="14"/>
-      <x:c r="N54" s="14"/>
+      <x:c r="N54" s="17"/>
       <x:c r="O54" s="14"/>
+      <x:c r="P54" s="14"/>
     </x:row>
     <x:row r="55" ht="22" customHeight="1">
       <x:c r="A55" s="17"/>
@@ -1369,8 +1426,9 @@
       <x:c r="K55" s="14"/>
       <x:c r="L55" s="14"/>
       <x:c r="M55" s="14"/>
-      <x:c r="N55" s="14"/>
+      <x:c r="N55" s="17"/>
       <x:c r="O55" s="14"/>
+      <x:c r="P55" s="14"/>
     </x:row>
     <x:row r="56" ht="22" customHeight="1">
       <x:c r="A56" s="17"/>
@@ -1386,8 +1444,9 @@
       <x:c r="K56" s="14"/>
       <x:c r="L56" s="14"/>
       <x:c r="M56" s="14"/>
-      <x:c r="N56" s="14"/>
+      <x:c r="N56" s="17"/>
       <x:c r="O56" s="14"/>
+      <x:c r="P56" s="14"/>
     </x:row>
     <x:row r="57" ht="22" customHeight="1">
       <x:c r="A57" s="17"/>
@@ -1403,8 +1462,9 @@
       <x:c r="K57" s="14"/>
       <x:c r="L57" s="14"/>
       <x:c r="M57" s="14"/>
-      <x:c r="N57" s="14"/>
+      <x:c r="N57" s="17"/>
       <x:c r="O57" s="14"/>
+      <x:c r="P57" s="14"/>
     </x:row>
     <x:row r="58" ht="22" customHeight="1">
       <x:c r="A58" s="17"/>
@@ -1420,8 +1480,9 @@
       <x:c r="K58" s="14"/>
       <x:c r="L58" s="14"/>
       <x:c r="M58" s="14"/>
-      <x:c r="N58" s="14"/>
+      <x:c r="N58" s="17"/>
       <x:c r="O58" s="14"/>
+      <x:c r="P58" s="14"/>
     </x:row>
     <x:row r="59" ht="22" customHeight="1">
       <x:c r="A59" s="17"/>
@@ -1437,8 +1498,9 @@
       <x:c r="K59" s="14"/>
       <x:c r="L59" s="14"/>
       <x:c r="M59" s="14"/>
-      <x:c r="N59" s="14"/>
+      <x:c r="N59" s="17"/>
       <x:c r="O59" s="14"/>
+      <x:c r="P59" s="14"/>
     </x:row>
     <x:row r="60" ht="22" customHeight="1">
       <x:c r="A60" s="17"/>
@@ -1454,8 +1516,9 @@
       <x:c r="K60" s="14"/>
       <x:c r="L60" s="14"/>
       <x:c r="M60" s="14"/>
-      <x:c r="N60" s="14"/>
+      <x:c r="N60" s="17"/>
       <x:c r="O60" s="14"/>
+      <x:c r="P60" s="14"/>
     </x:row>
     <x:row r="61" ht="22" customHeight="1">
       <x:c r="A61" s="17"/>
@@ -1471,8 +1534,9 @@
       <x:c r="K61" s="14"/>
       <x:c r="L61" s="14"/>
       <x:c r="M61" s="14"/>
-      <x:c r="N61" s="14"/>
+      <x:c r="N61" s="17"/>
       <x:c r="O61" s="14"/>
+      <x:c r="P61" s="14"/>
     </x:row>
     <x:row r="62" ht="22" customHeight="1">
       <x:c r="A62" s="17"/>
@@ -1488,8 +1552,9 @@
       <x:c r="K62" s="14"/>
       <x:c r="L62" s="14"/>
       <x:c r="M62" s="14"/>
-      <x:c r="N62" s="14"/>
+      <x:c r="N62" s="17"/>
       <x:c r="O62" s="14"/>
+      <x:c r="P62" s="14"/>
     </x:row>
     <x:row r="63" ht="22" customHeight="1">
       <x:c r="A63" s="17"/>
@@ -1505,8 +1570,9 @@
       <x:c r="K63" s="14"/>
       <x:c r="L63" s="14"/>
       <x:c r="M63" s="14"/>
-      <x:c r="N63" s="14"/>
+      <x:c r="N63" s="17"/>
       <x:c r="O63" s="14"/>
+      <x:c r="P63" s="14"/>
     </x:row>
     <x:row r="64" ht="22" customHeight="1">
       <x:c r="A64" s="17"/>
@@ -1522,8 +1588,9 @@
       <x:c r="K64" s="14"/>
       <x:c r="L64" s="14"/>
       <x:c r="M64" s="14"/>
-      <x:c r="N64" s="14"/>
+      <x:c r="N64" s="17"/>
       <x:c r="O64" s="14"/>
+      <x:c r="P64" s="14"/>
     </x:row>
     <x:row r="65" ht="22" customHeight="1">
       <x:c r="A65" s="17"/>
@@ -1539,8 +1606,9 @@
       <x:c r="K65" s="14"/>
       <x:c r="L65" s="14"/>
       <x:c r="M65" s="14"/>
-      <x:c r="N65" s="14"/>
+      <x:c r="N65" s="17"/>
       <x:c r="O65" s="14"/>
+      <x:c r="P65" s="14"/>
     </x:row>
     <x:row r="66" ht="22" customHeight="1">
       <x:c r="A66" s="17"/>
@@ -1556,8 +1624,9 @@
       <x:c r="K66" s="14"/>
       <x:c r="L66" s="14"/>
       <x:c r="M66" s="14"/>
-      <x:c r="N66" s="14"/>
+      <x:c r="N66" s="17"/>
       <x:c r="O66" s="14"/>
+      <x:c r="P66" s="14"/>
     </x:row>
     <x:row r="67" ht="22" customHeight="1">
       <x:c r="A67" s="17"/>
@@ -1573,8 +1642,9 @@
       <x:c r="K67" s="14"/>
       <x:c r="L67" s="14"/>
       <x:c r="M67" s="14"/>
-      <x:c r="N67" s="14"/>
+      <x:c r="N67" s="17"/>
       <x:c r="O67" s="14"/>
+      <x:c r="P67" s="14"/>
     </x:row>
     <x:row r="68" ht="22" customHeight="1">
       <x:c r="A68" s="17"/>
@@ -1590,8 +1660,9 @@
       <x:c r="K68" s="14"/>
       <x:c r="L68" s="14"/>
       <x:c r="M68" s="14"/>
-      <x:c r="N68" s="14"/>
+      <x:c r="N68" s="17"/>
       <x:c r="O68" s="14"/>
+      <x:c r="P68" s="14"/>
     </x:row>
     <x:row r="69" ht="22" customHeight="1">
       <x:c r="A69" s="17"/>
@@ -1607,8 +1678,9 @@
       <x:c r="K69" s="14"/>
       <x:c r="L69" s="14"/>
       <x:c r="M69" s="14"/>
-      <x:c r="N69" s="14"/>
+      <x:c r="N69" s="17"/>
       <x:c r="O69" s="14"/>
+      <x:c r="P69" s="14"/>
     </x:row>
     <x:row r="70" ht="22" customHeight="1">
       <x:c r="A70" s="17"/>
@@ -1624,8 +1696,9 @@
       <x:c r="K70" s="14"/>
       <x:c r="L70" s="14"/>
       <x:c r="M70" s="14"/>
-      <x:c r="N70" s="14"/>
+      <x:c r="N70" s="17"/>
       <x:c r="O70" s="14"/>
+      <x:c r="P70" s="14"/>
     </x:row>
     <x:row r="71" ht="22" customHeight="1">
       <x:c r="A71" s="17"/>
@@ -1641,8 +1714,9 @@
       <x:c r="K71" s="14"/>
       <x:c r="L71" s="14"/>
       <x:c r="M71" s="14"/>
-      <x:c r="N71" s="14"/>
+      <x:c r="N71" s="17"/>
       <x:c r="O71" s="14"/>
+      <x:c r="P71" s="14"/>
     </x:row>
     <x:row r="72" ht="22" customHeight="1">
       <x:c r="A72" s="17"/>
@@ -1658,8 +1732,9 @@
       <x:c r="K72" s="14"/>
       <x:c r="L72" s="14"/>
       <x:c r="M72" s="14"/>
-      <x:c r="N72" s="14"/>
+      <x:c r="N72" s="17"/>
       <x:c r="O72" s="14"/>
+      <x:c r="P72" s="14"/>
     </x:row>
     <x:row r="73" ht="22" customHeight="1">
       <x:c r="A73" s="17"/>
@@ -1675,8 +1750,9 @@
       <x:c r="K73" s="14"/>
       <x:c r="L73" s="14"/>
       <x:c r="M73" s="14"/>
-      <x:c r="N73" s="14"/>
+      <x:c r="N73" s="17"/>
       <x:c r="O73" s="14"/>
+      <x:c r="P73" s="14"/>
     </x:row>
     <x:row r="74" ht="22" customHeight="1">
       <x:c r="A74" s="17"/>
@@ -1692,8 +1768,9 @@
       <x:c r="K74" s="14"/>
       <x:c r="L74" s="14"/>
       <x:c r="M74" s="14"/>
-      <x:c r="N74" s="14"/>
+      <x:c r="N74" s="17"/>
       <x:c r="O74" s="14"/>
+      <x:c r="P74" s="14"/>
     </x:row>
     <x:row r="75" ht="22" customHeight="1">
       <x:c r="A75" s="17"/>
@@ -1709,8 +1786,9 @@
       <x:c r="K75" s="14"/>
       <x:c r="L75" s="14"/>
       <x:c r="M75" s="14"/>
-      <x:c r="N75" s="14"/>
+      <x:c r="N75" s="17"/>
       <x:c r="O75" s="14"/>
+      <x:c r="P75" s="14"/>
     </x:row>
     <x:row r="76" ht="22" customHeight="1">
       <x:c r="A76" s="17"/>
@@ -1726,8 +1804,9 @@
       <x:c r="K76" s="14"/>
       <x:c r="L76" s="14"/>
       <x:c r="M76" s="14"/>
-      <x:c r="N76" s="14"/>
+      <x:c r="N76" s="17"/>
       <x:c r="O76" s="14"/>
+      <x:c r="P76" s="14"/>
     </x:row>
     <x:row r="77" ht="22" customHeight="1">
       <x:c r="A77" s="17"/>
@@ -1743,8 +1822,9 @@
       <x:c r="K77" s="14"/>
       <x:c r="L77" s="14"/>
       <x:c r="M77" s="14"/>
-      <x:c r="N77" s="14"/>
+      <x:c r="N77" s="17"/>
       <x:c r="O77" s="14"/>
+      <x:c r="P77" s="14"/>
     </x:row>
     <x:row r="78" ht="22" customHeight="1">
       <x:c r="A78" s="17"/>
@@ -1760,8 +1840,9 @@
       <x:c r="K78" s="14"/>
       <x:c r="L78" s="14"/>
       <x:c r="M78" s="14"/>
-      <x:c r="N78" s="14"/>
+      <x:c r="N78" s="17"/>
       <x:c r="O78" s="14"/>
+      <x:c r="P78" s="14"/>
     </x:row>
     <x:row r="79" ht="22" customHeight="1">
       <x:c r="A79" s="17"/>
@@ -1777,8 +1858,9 @@
       <x:c r="K79" s="14"/>
       <x:c r="L79" s="14"/>
       <x:c r="M79" s="14"/>
-      <x:c r="N79" s="14"/>
+      <x:c r="N79" s="17"/>
       <x:c r="O79" s="14"/>
+      <x:c r="P79" s="14"/>
     </x:row>
     <x:row r="80" ht="22" customHeight="1">
       <x:c r="A80" s="17"/>
@@ -1794,8 +1876,9 @@
       <x:c r="K80" s="14"/>
       <x:c r="L80" s="14"/>
       <x:c r="M80" s="14"/>
-      <x:c r="N80" s="14"/>
+      <x:c r="N80" s="17"/>
       <x:c r="O80" s="14"/>
+      <x:c r="P80" s="14"/>
     </x:row>
     <x:row r="81" ht="22" customHeight="1">
       <x:c r="A81" s="17"/>
@@ -1811,8 +1894,9 @@
       <x:c r="K81" s="14"/>
       <x:c r="L81" s="14"/>
       <x:c r="M81" s="14"/>
-      <x:c r="N81" s="14"/>
+      <x:c r="N81" s="17"/>
       <x:c r="O81" s="14"/>
+      <x:c r="P81" s="14"/>
     </x:row>
     <x:row r="82" ht="22" customHeight="1">
       <x:c r="A82" s="17"/>
@@ -1828,8 +1912,9 @@
       <x:c r="K82" s="14"/>
       <x:c r="L82" s="14"/>
       <x:c r="M82" s="14"/>
-      <x:c r="N82" s="14"/>
+      <x:c r="N82" s="17"/>
       <x:c r="O82" s="14"/>
+      <x:c r="P82" s="14"/>
     </x:row>
     <x:row r="83" ht="22" customHeight="1">
       <x:c r="A83" s="17"/>
@@ -1845,8 +1930,9 @@
       <x:c r="K83" s="14"/>
       <x:c r="L83" s="14"/>
       <x:c r="M83" s="14"/>
-      <x:c r="N83" s="14"/>
+      <x:c r="N83" s="17"/>
       <x:c r="O83" s="14"/>
+      <x:c r="P83" s="14"/>
     </x:row>
     <x:row r="84" ht="22" customHeight="1">
       <x:c r="A84" s="17"/>
@@ -1862,8 +1948,9 @@
       <x:c r="K84" s="14"/>
       <x:c r="L84" s="14"/>
       <x:c r="M84" s="14"/>
-      <x:c r="N84" s="14"/>
+      <x:c r="N84" s="17"/>
       <x:c r="O84" s="14"/>
+      <x:c r="P84" s="14"/>
     </x:row>
     <x:row r="85" ht="22" customHeight="1">
       <x:c r="A85" s="17"/>
@@ -1879,8 +1966,9 @@
       <x:c r="K85" s="14"/>
       <x:c r="L85" s="14"/>
       <x:c r="M85" s="14"/>
-      <x:c r="N85" s="14"/>
+      <x:c r="N85" s="17"/>
       <x:c r="O85" s="14"/>
+      <x:c r="P85" s="14"/>
     </x:row>
     <x:row r="86" ht="22" customHeight="1">
       <x:c r="A86" s="17"/>
@@ -1896,8 +1984,9 @@
       <x:c r="K86" s="14"/>
       <x:c r="L86" s="14"/>
       <x:c r="M86" s="14"/>
-      <x:c r="N86" s="14"/>
+      <x:c r="N86" s="17"/>
       <x:c r="O86" s="14"/>
+      <x:c r="P86" s="14"/>
     </x:row>
     <x:row r="87" ht="22" customHeight="1">
       <x:c r="A87" s="17"/>
@@ -1913,8 +2002,9 @@
       <x:c r="K87" s="14"/>
       <x:c r="L87" s="14"/>
       <x:c r="M87" s="14"/>
-      <x:c r="N87" s="14"/>
+      <x:c r="N87" s="17"/>
       <x:c r="O87" s="14"/>
+      <x:c r="P87" s="14"/>
     </x:row>
     <x:row r="88" ht="22" customHeight="1">
       <x:c r="A88" s="17"/>
@@ -1930,8 +2020,9 @@
       <x:c r="K88" s="14"/>
       <x:c r="L88" s="14"/>
       <x:c r="M88" s="14"/>
-      <x:c r="N88" s="14"/>
+      <x:c r="N88" s="17"/>
       <x:c r="O88" s="14"/>
+      <x:c r="P88" s="14"/>
     </x:row>
     <x:row r="89" ht="22" customHeight="1">
       <x:c r="A89" s="17"/>
@@ -1947,8 +2038,9 @@
       <x:c r="K89" s="14"/>
       <x:c r="L89" s="14"/>
       <x:c r="M89" s="14"/>
-      <x:c r="N89" s="14"/>
+      <x:c r="N89" s="17"/>
       <x:c r="O89" s="14"/>
+      <x:c r="P89" s="14"/>
     </x:row>
     <x:row r="90" ht="22" customHeight="1">
       <x:c r="A90" s="17"/>
@@ -1964,8 +2056,9 @@
       <x:c r="K90" s="14"/>
       <x:c r="L90" s="14"/>
       <x:c r="M90" s="14"/>
-      <x:c r="N90" s="14"/>
+      <x:c r="N90" s="17"/>
       <x:c r="O90" s="14"/>
+      <x:c r="P90" s="14"/>
     </x:row>
     <x:row r="91" ht="22" customHeight="1">
       <x:c r="A91" s="17"/>
@@ -1981,8 +2074,9 @@
       <x:c r="K91" s="14"/>
       <x:c r="L91" s="14"/>
       <x:c r="M91" s="14"/>
-      <x:c r="N91" s="14"/>
+      <x:c r="N91" s="17"/>
       <x:c r="O91" s="14"/>
+      <x:c r="P91" s="14"/>
     </x:row>
     <x:row r="92" ht="22" customHeight="1">
       <x:c r="A92" s="17"/>
@@ -1998,8 +2092,9 @@
       <x:c r="K92" s="14"/>
       <x:c r="L92" s="14"/>
       <x:c r="M92" s="14"/>
-      <x:c r="N92" s="14"/>
+      <x:c r="N92" s="17"/>
       <x:c r="O92" s="14"/>
+      <x:c r="P92" s="14"/>
     </x:row>
     <x:row r="93" ht="22" customHeight="1">
       <x:c r="A93" s="17"/>
@@ -2015,8 +2110,9 @@
       <x:c r="K93" s="14"/>
       <x:c r="L93" s="14"/>
       <x:c r="M93" s="14"/>
-      <x:c r="N93" s="14"/>
+      <x:c r="N93" s="17"/>
       <x:c r="O93" s="14"/>
+      <x:c r="P93" s="14"/>
     </x:row>
     <x:row r="94" ht="22" customHeight="1">
       <x:c r="A94" s="17"/>
@@ -2032,8 +2128,9 @@
       <x:c r="K94" s="14"/>
       <x:c r="L94" s="14"/>
       <x:c r="M94" s="14"/>
-      <x:c r="N94" s="14"/>
+      <x:c r="N94" s="17"/>
       <x:c r="O94" s="14"/>
+      <x:c r="P94" s="14"/>
     </x:row>
     <x:row r="95" ht="22" customHeight="1">
       <x:c r="A95" s="17"/>
@@ -2049,8 +2146,9 @@
       <x:c r="K95" s="14"/>
       <x:c r="L95" s="14"/>
       <x:c r="M95" s="14"/>
-      <x:c r="N95" s="14"/>
+      <x:c r="N95" s="17"/>
       <x:c r="O95" s="14"/>
+      <x:c r="P95" s="14"/>
     </x:row>
     <x:row r="96" ht="22" customHeight="1">
       <x:c r="A96" s="17"/>
@@ -2066,8 +2164,9 @@
       <x:c r="K96" s="14"/>
       <x:c r="L96" s="14"/>
       <x:c r="M96" s="14"/>
-      <x:c r="N96" s="14"/>
+      <x:c r="N96" s="17"/>
       <x:c r="O96" s="14"/>
+      <x:c r="P96" s="14"/>
     </x:row>
     <x:row r="97" ht="22" customHeight="1">
       <x:c r="A97" s="17"/>
@@ -2083,8 +2182,9 @@
       <x:c r="K97" s="14"/>
       <x:c r="L97" s="14"/>
       <x:c r="M97" s="14"/>
-      <x:c r="N97" s="14"/>
+      <x:c r="N97" s="17"/>
       <x:c r="O97" s="14"/>
+      <x:c r="P97" s="14"/>
     </x:row>
     <x:row r="98" ht="22" customHeight="1">
       <x:c r="A98" s="17"/>
@@ -2100,8 +2200,9 @@
       <x:c r="K98" s="14"/>
       <x:c r="L98" s="14"/>
       <x:c r="M98" s="14"/>
-      <x:c r="N98" s="14"/>
+      <x:c r="N98" s="17"/>
       <x:c r="O98" s="14"/>
+      <x:c r="P98" s="14"/>
     </x:row>
     <x:row r="99" ht="22" customHeight="1">
       <x:c r="A99" s="17"/>
@@ -2117,8 +2218,9 @@
       <x:c r="K99" s="14"/>
       <x:c r="L99" s="14"/>
       <x:c r="M99" s="14"/>
-      <x:c r="N99" s="14"/>
+      <x:c r="N99" s="17"/>
       <x:c r="O99" s="14"/>
+      <x:c r="P99" s="14"/>
     </x:row>
     <x:row r="100" ht="22" customHeight="1">
       <x:c r="A100" s="17"/>
@@ -2134,8 +2236,9 @@
       <x:c r="K100" s="14"/>
       <x:c r="L100" s="14"/>
       <x:c r="M100" s="14"/>
-      <x:c r="N100" s="14"/>
+      <x:c r="N100" s="17"/>
       <x:c r="O100" s="14"/>
+      <x:c r="P100" s="14"/>
     </x:row>
     <x:row r="101" ht="22" customHeight="1">
       <x:c r="A101" s="17"/>
@@ -2151,8 +2254,9 @@
       <x:c r="K101" s="14"/>
       <x:c r="L101" s="14"/>
       <x:c r="M101" s="14"/>
-      <x:c r="N101" s="14"/>
+      <x:c r="N101" s="17"/>
       <x:c r="O101" s="14"/>
+      <x:c r="P101" s="14"/>
     </x:row>
     <x:row r="102" ht="22" customHeight="1">
       <x:c r="A102" s="17"/>
@@ -2168,8 +2272,9 @@
       <x:c r="K102" s="14"/>
       <x:c r="L102" s="14"/>
       <x:c r="M102" s="14"/>
-      <x:c r="N102" s="14"/>
+      <x:c r="N102" s="17"/>
       <x:c r="O102" s="14"/>
+      <x:c r="P102" s="14"/>
     </x:row>
     <x:row r="103" ht="22" customHeight="1">
       <x:c r="A103" s="17"/>
@@ -2185,8 +2290,9 @@
       <x:c r="K103" s="14"/>
       <x:c r="L103" s="14"/>
       <x:c r="M103" s="14"/>
-      <x:c r="N103" s="14"/>
+      <x:c r="N103" s="17"/>
       <x:c r="O103" s="14"/>
+      <x:c r="P103" s="14"/>
     </x:row>
     <x:row r="104" ht="22" customHeight="1">
       <x:c r="A104" s="17"/>
@@ -2202,8 +2308,9 @@
       <x:c r="K104" s="14"/>
       <x:c r="L104" s="14"/>
       <x:c r="M104" s="14"/>
-      <x:c r="N104" s="14"/>
+      <x:c r="N104" s="17"/>
       <x:c r="O104" s="14"/>
+      <x:c r="P104" s="14"/>
     </x:row>
     <x:row r="105" ht="22" customHeight="1">
       <x:c r="A105" s="17"/>
@@ -2219,8 +2326,9 @@
       <x:c r="K105" s="14"/>
       <x:c r="L105" s="14"/>
       <x:c r="M105" s="14"/>
-      <x:c r="N105" s="14"/>
+      <x:c r="N105" s="17"/>
       <x:c r="O105" s="14"/>
+      <x:c r="P105" s="14"/>
     </x:row>
     <x:row r="106" ht="22" customHeight="1">
       <x:c r="A106" s="17"/>
@@ -2236,8 +2344,9 @@
       <x:c r="K106" s="14"/>
       <x:c r="L106" s="14"/>
       <x:c r="M106" s="14"/>
-      <x:c r="N106" s="14"/>
+      <x:c r="N106" s="17"/>
       <x:c r="O106" s="14"/>
+      <x:c r="P106" s="14"/>
     </x:row>
     <x:row r="107" ht="22" customHeight="1">
       <x:c r="A107" s="17"/>
@@ -2253,8 +2362,9 @@
       <x:c r="K107" s="14"/>
       <x:c r="L107" s="14"/>
       <x:c r="M107" s="14"/>
-      <x:c r="N107" s="14"/>
+      <x:c r="N107" s="17"/>
       <x:c r="O107" s="14"/>
+      <x:c r="P107" s="14"/>
     </x:row>
     <x:row r="108" ht="22" customHeight="1">
       <x:c r="A108" s="17"/>
@@ -2270,8 +2380,9 @@
       <x:c r="K108" s="14"/>
       <x:c r="L108" s="14"/>
       <x:c r="M108" s="14"/>
-      <x:c r="N108" s="14"/>
+      <x:c r="N108" s="17"/>
       <x:c r="O108" s="14"/>
+      <x:c r="P108" s="14"/>
     </x:row>
     <x:row r="109" ht="22" customHeight="1">
       <x:c r="A109" s="17"/>
@@ -2287,8 +2398,9 @@
       <x:c r="K109" s="14"/>
       <x:c r="L109" s="14"/>
       <x:c r="M109" s="14"/>
-      <x:c r="N109" s="14"/>
+      <x:c r="N109" s="17"/>
       <x:c r="O109" s="14"/>
+      <x:c r="P109" s="14"/>
     </x:row>
     <x:row r="110" ht="22" customHeight="1">
       <x:c r="A110" s="17"/>
@@ -2304,8 +2416,9 @@
       <x:c r="K110" s="14"/>
       <x:c r="L110" s="14"/>
       <x:c r="M110" s="14"/>
-      <x:c r="N110" s="14"/>
+      <x:c r="N110" s="17"/>
       <x:c r="O110" s="14"/>
+      <x:c r="P110" s="14"/>
     </x:row>
     <x:row r="111" ht="22" customHeight="1">
       <x:c r="A111" s="17"/>
@@ -2321,8 +2434,9 @@
       <x:c r="K111" s="14"/>
       <x:c r="L111" s="14"/>
       <x:c r="M111" s="14"/>
-      <x:c r="N111" s="14"/>
+      <x:c r="N111" s="17"/>
       <x:c r="O111" s="14"/>
+      <x:c r="P111" s="14"/>
     </x:row>
     <x:row r="112" ht="22" customHeight="1">
       <x:c r="A112" s="17"/>
@@ -2338,8 +2452,9 @@
       <x:c r="K112" s="14"/>
       <x:c r="L112" s="14"/>
       <x:c r="M112" s="14"/>
-      <x:c r="N112" s="14"/>
+      <x:c r="N112" s="17"/>
       <x:c r="O112" s="14"/>
+      <x:c r="P112" s="14"/>
     </x:row>
     <x:row r="113" ht="22" customHeight="1">
       <x:c r="A113" s="17"/>
@@ -2355,8 +2470,9 @@
       <x:c r="K113" s="14"/>
       <x:c r="L113" s="14"/>
       <x:c r="M113" s="14"/>
-      <x:c r="N113" s="14"/>
+      <x:c r="N113" s="17"/>
       <x:c r="O113" s="14"/>
+      <x:c r="P113" s="14"/>
     </x:row>
     <x:row r="114" ht="22" customHeight="1">
       <x:c r="A114" s="17"/>
@@ -2372,8 +2488,9 @@
       <x:c r="K114" s="14"/>
       <x:c r="L114" s="14"/>
       <x:c r="M114" s="14"/>
-      <x:c r="N114" s="14"/>
+      <x:c r="N114" s="17"/>
       <x:c r="O114" s="14"/>
+      <x:c r="P114" s="14"/>
     </x:row>
     <x:row r="115" ht="22" customHeight="1">
       <x:c r="A115" s="17"/>
@@ -2389,8 +2506,9 @@
       <x:c r="K115" s="14"/>
       <x:c r="L115" s="14"/>
       <x:c r="M115" s="14"/>
-      <x:c r="N115" s="14"/>
+      <x:c r="N115" s="17"/>
       <x:c r="O115" s="14"/>
+      <x:c r="P115" s="14"/>
     </x:row>
     <x:row r="116" ht="22" customHeight="1">
       <x:c r="A116" s="17"/>
@@ -2406,8 +2524,9 @@
       <x:c r="K116" s="14"/>
       <x:c r="L116" s="14"/>
       <x:c r="M116" s="14"/>
-      <x:c r="N116" s="14"/>
+      <x:c r="N116" s="17"/>
       <x:c r="O116" s="14"/>
+      <x:c r="P116" s="14"/>
     </x:row>
     <x:row r="117" ht="22" customHeight="1">
       <x:c r="A117" s="17"/>
@@ -2423,8 +2542,9 @@
       <x:c r="K117" s="14"/>
       <x:c r="L117" s="14"/>
       <x:c r="M117" s="14"/>
-      <x:c r="N117" s="14"/>
+      <x:c r="N117" s="17"/>
       <x:c r="O117" s="14"/>
+      <x:c r="P117" s="14"/>
     </x:row>
     <x:row r="118" ht="22" customHeight="1">
       <x:c r="A118" s="17"/>
@@ -2440,8 +2560,9 @@
       <x:c r="K118" s="14"/>
       <x:c r="L118" s="14"/>
       <x:c r="M118" s="14"/>
-      <x:c r="N118" s="14"/>
+      <x:c r="N118" s="17"/>
       <x:c r="O118" s="14"/>
+      <x:c r="P118" s="14"/>
     </x:row>
     <x:row r="119" ht="22" customHeight="1">
       <x:c r="A119" s="17"/>
@@ -2457,8 +2578,9 @@
       <x:c r="K119" s="14"/>
       <x:c r="L119" s="14"/>
       <x:c r="M119" s="14"/>
-      <x:c r="N119" s="14"/>
+      <x:c r="N119" s="17"/>
       <x:c r="O119" s="14"/>
+      <x:c r="P119" s="14"/>
     </x:row>
     <x:row r="120" ht="22" customHeight="1">
       <x:c r="A120" s="17"/>
@@ -2474,8 +2596,9 @@
       <x:c r="K120" s="14"/>
       <x:c r="L120" s="14"/>
       <x:c r="M120" s="14"/>
-      <x:c r="N120" s="14"/>
+      <x:c r="N120" s="17"/>
       <x:c r="O120" s="14"/>
+      <x:c r="P120" s="14"/>
     </x:row>
     <x:row r="121" ht="22" customHeight="1">
       <x:c r="A121" s="17"/>
@@ -2491,8 +2614,9 @@
       <x:c r="K121" s="14"/>
       <x:c r="L121" s="14"/>
       <x:c r="M121" s="14"/>
-      <x:c r="N121" s="14"/>
+      <x:c r="N121" s="17"/>
       <x:c r="O121" s="14"/>
+      <x:c r="P121" s="14"/>
     </x:row>
     <x:row r="122" ht="22" customHeight="1">
       <x:c r="A122" s="17"/>
@@ -2508,8 +2632,9 @@
       <x:c r="K122" s="14"/>
       <x:c r="L122" s="14"/>
       <x:c r="M122" s="14"/>
-      <x:c r="N122" s="14"/>
+      <x:c r="N122" s="17"/>
       <x:c r="O122" s="14"/>
+      <x:c r="P122" s="14"/>
     </x:row>
     <x:row r="123" ht="22" customHeight="1">
       <x:c r="A123" s="17"/>
@@ -2525,8 +2650,9 @@
       <x:c r="K123" s="14"/>
       <x:c r="L123" s="14"/>
       <x:c r="M123" s="14"/>
-      <x:c r="N123" s="14"/>
+      <x:c r="N123" s="17"/>
       <x:c r="O123" s="14"/>
+      <x:c r="P123" s="14"/>
     </x:row>
     <x:row r="124" ht="22" customHeight="1">
       <x:c r="A124" s="17"/>
@@ -2542,8 +2668,9 @@
       <x:c r="K124" s="14"/>
       <x:c r="L124" s="14"/>
       <x:c r="M124" s="14"/>
-      <x:c r="N124" s="14"/>
+      <x:c r="N124" s="17"/>
       <x:c r="O124" s="14"/>
+      <x:c r="P124" s="14"/>
     </x:row>
     <x:row r="125" ht="22" customHeight="1">
       <x:c r="A125" s="17"/>
@@ -2559,8 +2686,9 @@
       <x:c r="K125" s="14"/>
       <x:c r="L125" s="14"/>
       <x:c r="M125" s="14"/>
-      <x:c r="N125" s="14"/>
+      <x:c r="N125" s="17"/>
       <x:c r="O125" s="14"/>
+      <x:c r="P125" s="14"/>
     </x:row>
     <x:row r="126" ht="22" customHeight="1">
       <x:c r="A126" s="17"/>
@@ -2576,8 +2704,9 @@
       <x:c r="K126" s="14"/>
       <x:c r="L126" s="14"/>
       <x:c r="M126" s="14"/>
-      <x:c r="N126" s="14"/>
+      <x:c r="N126" s="17"/>
       <x:c r="O126" s="14"/>
+      <x:c r="P126" s="14"/>
     </x:row>
     <x:row r="127" ht="22" customHeight="1">
       <x:c r="A127" s="17"/>
@@ -2593,8 +2722,9 @@
       <x:c r="K127" s="14"/>
       <x:c r="L127" s="14"/>
       <x:c r="M127" s="14"/>
-      <x:c r="N127" s="14"/>
+      <x:c r="N127" s="17"/>
       <x:c r="O127" s="14"/>
+      <x:c r="P127" s="14"/>
     </x:row>
     <x:row r="128" ht="22" customHeight="1">
       <x:c r="A128" s="17"/>
@@ -2610,8 +2740,9 @@
       <x:c r="K128" s="14"/>
       <x:c r="L128" s="14"/>
       <x:c r="M128" s="14"/>
-      <x:c r="N128" s="14"/>
+      <x:c r="N128" s="17"/>
       <x:c r="O128" s="14"/>
+      <x:c r="P128" s="14"/>
     </x:row>
     <x:row r="129" ht="22" customHeight="1">
       <x:c r="A129" s="17"/>
@@ -2627,8 +2758,9 @@
       <x:c r="K129" s="14"/>
       <x:c r="L129" s="14"/>
       <x:c r="M129" s="14"/>
-      <x:c r="N129" s="14"/>
+      <x:c r="N129" s="17"/>
       <x:c r="O129" s="14"/>
+      <x:c r="P129" s="14"/>
     </x:row>
     <x:row r="130" ht="22" customHeight="1">
       <x:c r="A130" s="17"/>
@@ -2644,8 +2776,9 @@
       <x:c r="K130" s="14"/>
       <x:c r="L130" s="14"/>
       <x:c r="M130" s="14"/>
-      <x:c r="N130" s="14"/>
+      <x:c r="N130" s="17"/>
       <x:c r="O130" s="14"/>
+      <x:c r="P130" s="14"/>
     </x:row>
     <x:row r="131" ht="22" customHeight="1">
       <x:c r="A131" s="17"/>
@@ -2661,8 +2794,9 @@
       <x:c r="K131" s="14"/>
       <x:c r="L131" s="14"/>
       <x:c r="M131" s="14"/>
-      <x:c r="N131" s="14"/>
+      <x:c r="N131" s="17"/>
       <x:c r="O131" s="14"/>
+      <x:c r="P131" s="14"/>
     </x:row>
     <x:row r="132" ht="22" customHeight="1">
       <x:c r="A132" s="17"/>
@@ -2678,8 +2812,9 @@
       <x:c r="K132" s="14"/>
       <x:c r="L132" s="14"/>
       <x:c r="M132" s="14"/>
-      <x:c r="N132" s="14"/>
+      <x:c r="N132" s="17"/>
       <x:c r="O132" s="14"/>
+      <x:c r="P132" s="14"/>
     </x:row>
     <x:row r="133" ht="22" customHeight="1">
       <x:c r="A133" s="17"/>
@@ -2695,8 +2830,9 @@
       <x:c r="K133" s="14"/>
       <x:c r="L133" s="14"/>
       <x:c r="M133" s="14"/>
-      <x:c r="N133" s="14"/>
+      <x:c r="N133" s="17"/>
       <x:c r="O133" s="14"/>
+      <x:c r="P133" s="14"/>
     </x:row>
     <x:row r="134" ht="22" customHeight="1">
       <x:c r="A134" s="17"/>
@@ -2712,8 +2848,9 @@
       <x:c r="K134" s="14"/>
       <x:c r="L134" s="14"/>
       <x:c r="M134" s="14"/>
-      <x:c r="N134" s="14"/>
+      <x:c r="N134" s="17"/>
       <x:c r="O134" s="14"/>
+      <x:c r="P134" s="14"/>
     </x:row>
     <x:row r="135" ht="22" customHeight="1">
       <x:c r="A135" s="17"/>
@@ -2729,8 +2866,9 @@
       <x:c r="K135" s="14"/>
       <x:c r="L135" s="14"/>
       <x:c r="M135" s="14"/>
-      <x:c r="N135" s="14"/>
+      <x:c r="N135" s="17"/>
       <x:c r="O135" s="14"/>
+      <x:c r="P135" s="14"/>
     </x:row>
     <x:row r="136" ht="22" customHeight="1">
       <x:c r="A136" s="17"/>
@@ -2746,8 +2884,9 @@
       <x:c r="K136" s="14"/>
       <x:c r="L136" s="14"/>
       <x:c r="M136" s="14"/>
-      <x:c r="N136" s="14"/>
+      <x:c r="N136" s="17"/>
       <x:c r="O136" s="14"/>
+      <x:c r="P136" s="14"/>
     </x:row>
     <x:row r="137" ht="22" customHeight="1">
       <x:c r="A137" s="17"/>
@@ -2763,8 +2902,9 @@
       <x:c r="K137" s="14"/>
       <x:c r="L137" s="14"/>
       <x:c r="M137" s="14"/>
-      <x:c r="N137" s="14"/>
+      <x:c r="N137" s="17"/>
       <x:c r="O137" s="14"/>
+      <x:c r="P137" s="14"/>
     </x:row>
     <x:row r="138" ht="22" customHeight="1">
       <x:c r="A138" s="17"/>
@@ -2780,8 +2920,9 @@
       <x:c r="K138" s="14"/>
       <x:c r="L138" s="14"/>
       <x:c r="M138" s="14"/>
-      <x:c r="N138" s="14"/>
+      <x:c r="N138" s="17"/>
       <x:c r="O138" s="14"/>
+      <x:c r="P138" s="14"/>
     </x:row>
     <x:row r="139" ht="22" customHeight="1">
       <x:c r="A139" s="17"/>
@@ -2797,8 +2938,9 @@
       <x:c r="K139" s="14"/>
       <x:c r="L139" s="14"/>
       <x:c r="M139" s="14"/>
-      <x:c r="N139" s="14"/>
+      <x:c r="N139" s="17"/>
       <x:c r="O139" s="14"/>
+      <x:c r="P139" s="14"/>
     </x:row>
     <x:row r="140" ht="22" customHeight="1">
       <x:c r="A140" s="17"/>
@@ -2814,8 +2956,9 @@
       <x:c r="K140" s="14"/>
       <x:c r="L140" s="14"/>
       <x:c r="M140" s="14"/>
-      <x:c r="N140" s="14"/>
+      <x:c r="N140" s="17"/>
       <x:c r="O140" s="14"/>
+      <x:c r="P140" s="14"/>
     </x:row>
     <x:row r="141" ht="22" customHeight="1">
       <x:c r="A141" s="17"/>
@@ -2831,8 +2974,9 @@
       <x:c r="K141" s="14"/>
       <x:c r="L141" s="14"/>
       <x:c r="M141" s="14"/>
-      <x:c r="N141" s="14"/>
+      <x:c r="N141" s="17"/>
       <x:c r="O141" s="14"/>
+      <x:c r="P141" s="14"/>
     </x:row>
     <x:row r="142" ht="22" customHeight="1">
       <x:c r="A142" s="17"/>
@@ -2848,8 +2992,9 @@
       <x:c r="K142" s="14"/>
       <x:c r="L142" s="14"/>
       <x:c r="M142" s="14"/>
-      <x:c r="N142" s="14"/>
+      <x:c r="N142" s="17"/>
       <x:c r="O142" s="14"/>
+      <x:c r="P142" s="14"/>
     </x:row>
     <x:row r="143" ht="22" customHeight="1">
       <x:c r="A143" s="17"/>
@@ -2865,8 +3010,9 @@
       <x:c r="K143" s="14"/>
       <x:c r="L143" s="14"/>
       <x:c r="M143" s="14"/>
-      <x:c r="N143" s="14"/>
+      <x:c r="N143" s="17"/>
       <x:c r="O143" s="14"/>
+      <x:c r="P143" s="14"/>
     </x:row>
     <x:row r="144" ht="22" customHeight="1">
       <x:c r="A144" s="17"/>
@@ -2882,8 +3028,9 @@
       <x:c r="K144" s="14"/>
       <x:c r="L144" s="14"/>
       <x:c r="M144" s="14"/>
-      <x:c r="N144" s="14"/>
+      <x:c r="N144" s="17"/>
       <x:c r="O144" s="14"/>
+      <x:c r="P144" s="14"/>
     </x:row>
     <x:row r="145" ht="22" customHeight="1">
       <x:c r="A145" s="17"/>
@@ -2899,8 +3046,9 @@
       <x:c r="K145" s="14"/>
       <x:c r="L145" s="14"/>
       <x:c r="M145" s="14"/>
-      <x:c r="N145" s="14"/>
+      <x:c r="N145" s="17"/>
       <x:c r="O145" s="14"/>
+      <x:c r="P145" s="14"/>
     </x:row>
     <x:row r="146" ht="22" customHeight="1">
       <x:c r="A146" s="17"/>
@@ -2916,8 +3064,9 @@
       <x:c r="K146" s="14"/>
       <x:c r="L146" s="14"/>
       <x:c r="M146" s="14"/>
-      <x:c r="N146" s="14"/>
+      <x:c r="N146" s="17"/>
       <x:c r="O146" s="14"/>
+      <x:c r="P146" s="14"/>
     </x:row>
     <x:row r="147" ht="22" customHeight="1">
       <x:c r="A147" s="17"/>
@@ -2933,8 +3082,9 @@
       <x:c r="K147" s="14"/>
       <x:c r="L147" s="14"/>
       <x:c r="M147" s="14"/>
-      <x:c r="N147" s="14"/>
+      <x:c r="N147" s="17"/>
       <x:c r="O147" s="14"/>
+      <x:c r="P147" s="14"/>
     </x:row>
     <x:row r="148" ht="22" customHeight="1">
       <x:c r="A148" s="17"/>
@@ -2950,8 +3100,9 @@
       <x:c r="K148" s="14"/>
       <x:c r="L148" s="14"/>
       <x:c r="M148" s="14"/>
-      <x:c r="N148" s="14"/>
+      <x:c r="N148" s="17"/>
       <x:c r="O148" s="14"/>
+      <x:c r="P148" s="14"/>
     </x:row>
     <x:row r="149" ht="22" customHeight="1">
       <x:c r="A149" s="17"/>
@@ -2967,8 +3118,9 @@
       <x:c r="K149" s="14"/>
       <x:c r="L149" s="14"/>
       <x:c r="M149" s="14"/>
-      <x:c r="N149" s="14"/>
+      <x:c r="N149" s="17"/>
       <x:c r="O149" s="14"/>
+      <x:c r="P149" s="14"/>
     </x:row>
     <x:row r="150" ht="22" customHeight="1">
       <x:c r="A150" s="17"/>
@@ -2984,8 +3136,9 @@
       <x:c r="K150" s="14"/>
       <x:c r="L150" s="14"/>
       <x:c r="M150" s="14"/>
-      <x:c r="N150" s="14"/>
+      <x:c r="N150" s="17"/>
       <x:c r="O150" s="14"/>
+      <x:c r="P150" s="14"/>
     </x:row>
     <x:row r="151" ht="22" customHeight="1">
       <x:c r="A151" s="17"/>
@@ -3001,8 +3154,9 @@
       <x:c r="K151" s="14"/>
       <x:c r="L151" s="14"/>
       <x:c r="M151" s="14"/>
-      <x:c r="N151" s="14"/>
+      <x:c r="N151" s="17"/>
       <x:c r="O151" s="14"/>
+      <x:c r="P151" s="14"/>
     </x:row>
     <x:row r="152" ht="22" customHeight="1">
       <x:c r="A152" s="17"/>
@@ -3018,8 +3172,9 @@
       <x:c r="K152" s="14"/>
       <x:c r="L152" s="14"/>
       <x:c r="M152" s="14"/>
-      <x:c r="N152" s="14"/>
+      <x:c r="N152" s="17"/>
       <x:c r="O152" s="14"/>
+      <x:c r="P152" s="14"/>
     </x:row>
     <x:row r="153" ht="22" customHeight="1">
       <x:c r="A153" s="17"/>
@@ -3035,8 +3190,9 @@
       <x:c r="K153" s="14"/>
       <x:c r="L153" s="14"/>
       <x:c r="M153" s="14"/>
-      <x:c r="N153" s="14"/>
+      <x:c r="N153" s="17"/>
       <x:c r="O153" s="14"/>
+      <x:c r="P153" s="14"/>
     </x:row>
     <x:row r="154" ht="22" customHeight="1">
       <x:c r="A154" s="17"/>
@@ -3052,8 +3208,9 @@
       <x:c r="K154" s="14"/>
       <x:c r="L154" s="14"/>
       <x:c r="M154" s="14"/>
-      <x:c r="N154" s="14"/>
+      <x:c r="N154" s="17"/>
       <x:c r="O154" s="14"/>
+      <x:c r="P154" s="14"/>
     </x:row>
     <x:row r="155" ht="22" customHeight="1">
       <x:c r="A155" s="17"/>
@@ -3069,8 +3226,9 @@
       <x:c r="K155" s="14"/>
       <x:c r="L155" s="14"/>
       <x:c r="M155" s="14"/>
-      <x:c r="N155" s="14"/>
+      <x:c r="N155" s="17"/>
       <x:c r="O155" s="14"/>
+      <x:c r="P155" s="14"/>
     </x:row>
     <x:row r="156" ht="22" customHeight="1">
       <x:c r="A156" s="17"/>
@@ -3086,8 +3244,9 @@
       <x:c r="K156" s="14"/>
       <x:c r="L156" s="14"/>
       <x:c r="M156" s="14"/>
-      <x:c r="N156" s="14"/>
+      <x:c r="N156" s="17"/>
       <x:c r="O156" s="14"/>
+      <x:c r="P156" s="14"/>
     </x:row>
     <x:row r="157" ht="22" customHeight="1">
       <x:c r="A157" s="17"/>
@@ -3103,8 +3262,9 @@
       <x:c r="K157" s="14"/>
       <x:c r="L157" s="14"/>
       <x:c r="M157" s="14"/>
-      <x:c r="N157" s="14"/>
+      <x:c r="N157" s="17"/>
       <x:c r="O157" s="14"/>
+      <x:c r="P157" s="14"/>
     </x:row>
     <x:row r="158" ht="22" customHeight="1">
       <x:c r="A158" s="17"/>
@@ -3120,8 +3280,9 @@
       <x:c r="K158" s="14"/>
       <x:c r="L158" s="14"/>
       <x:c r="M158" s="14"/>
-      <x:c r="N158" s="14"/>
+      <x:c r="N158" s="17"/>
       <x:c r="O158" s="14"/>
+      <x:c r="P158" s="14"/>
     </x:row>
     <x:row r="159" ht="22" customHeight="1">
       <x:c r="A159" s="17"/>
@@ -3137,8 +3298,9 @@
       <x:c r="K159" s="14"/>
       <x:c r="L159" s="14"/>
       <x:c r="M159" s="14"/>
-      <x:c r="N159" s="14"/>
+      <x:c r="N159" s="17"/>
       <x:c r="O159" s="14"/>
+      <x:c r="P159" s="14"/>
     </x:row>
     <x:row r="160" ht="22" customHeight="1">
       <x:c r="A160" s="17"/>
@@ -3154,8 +3316,9 @@
       <x:c r="K160" s="14"/>
       <x:c r="L160" s="14"/>
       <x:c r="M160" s="14"/>
-      <x:c r="N160" s="14"/>
+      <x:c r="N160" s="17"/>
       <x:c r="O160" s="14"/>
+      <x:c r="P160" s="14"/>
     </x:row>
     <x:row r="161" ht="22" customHeight="1">
       <x:c r="A161" s="17"/>
@@ -3171,8 +3334,9 @@
       <x:c r="K161" s="14"/>
       <x:c r="L161" s="14"/>
       <x:c r="M161" s="14"/>
-      <x:c r="N161" s="14"/>
+      <x:c r="N161" s="17"/>
       <x:c r="O161" s="14"/>
+      <x:c r="P161" s="14"/>
     </x:row>
     <x:row r="162" ht="22" customHeight="1">
       <x:c r="A162" s="17"/>
@@ -3188,8 +3352,9 @@
       <x:c r="K162" s="14"/>
       <x:c r="L162" s="14"/>
       <x:c r="M162" s="14"/>
-      <x:c r="N162" s="14"/>
+      <x:c r="N162" s="17"/>
       <x:c r="O162" s="14"/>
+      <x:c r="P162" s="14"/>
     </x:row>
     <x:row r="163" ht="22" customHeight="1">
       <x:c r="A163" s="17"/>
@@ -3205,8 +3370,9 @@
       <x:c r="K163" s="14"/>
       <x:c r="L163" s="14"/>
       <x:c r="M163" s="14"/>
-      <x:c r="N163" s="14"/>
+      <x:c r="N163" s="17"/>
       <x:c r="O163" s="14"/>
+      <x:c r="P163" s="14"/>
     </x:row>
     <x:row r="164" ht="22" customHeight="1">
       <x:c r="A164" s="17"/>
@@ -3222,8 +3388,9 @@
       <x:c r="K164" s="14"/>
       <x:c r="L164" s="14"/>
       <x:c r="M164" s="14"/>
-      <x:c r="N164" s="14"/>
+      <x:c r="N164" s="17"/>
       <x:c r="O164" s="14"/>
+      <x:c r="P164" s="14"/>
     </x:row>
     <x:row r="165" ht="22" customHeight="1">
       <x:c r="A165" s="17"/>
@@ -3239,8 +3406,9 @@
       <x:c r="K165" s="14"/>
       <x:c r="L165" s="14"/>
       <x:c r="M165" s="14"/>
-      <x:c r="N165" s="14"/>
+      <x:c r="N165" s="17"/>
       <x:c r="O165" s="14"/>
+      <x:c r="P165" s="14"/>
     </x:row>
     <x:row r="166" ht="22" customHeight="1">
       <x:c r="A166" s="17"/>
@@ -3256,8 +3424,9 @@
       <x:c r="K166" s="14"/>
       <x:c r="L166" s="14"/>
       <x:c r="M166" s="14"/>
-      <x:c r="N166" s="14"/>
+      <x:c r="N166" s="17"/>
       <x:c r="O166" s="14"/>
+      <x:c r="P166" s="14"/>
     </x:row>
     <x:row r="167" ht="22" customHeight="1">
       <x:c r="A167" s="17"/>
@@ -3273,8 +3442,9 @@
       <x:c r="K167" s="14"/>
       <x:c r="L167" s="14"/>
       <x:c r="M167" s="14"/>
-      <x:c r="N167" s="14"/>
+      <x:c r="N167" s="17"/>
       <x:c r="O167" s="14"/>
+      <x:c r="P167" s="14"/>
     </x:row>
     <x:row r="168" ht="22" customHeight="1">
       <x:c r="A168" s="17"/>
@@ -3290,8 +3460,9 @@
       <x:c r="K168" s="14"/>
       <x:c r="L168" s="14"/>
       <x:c r="M168" s="14"/>
-      <x:c r="N168" s="14"/>
+      <x:c r="N168" s="17"/>
       <x:c r="O168" s="14"/>
+      <x:c r="P168" s="14"/>
     </x:row>
     <x:row r="169" ht="22" customHeight="1">
       <x:c r="A169" s="17"/>
@@ -3307,8 +3478,9 @@
       <x:c r="K169" s="14"/>
       <x:c r="L169" s="14"/>
       <x:c r="M169" s="14"/>
-      <x:c r="N169" s="14"/>
+      <x:c r="N169" s="17"/>
       <x:c r="O169" s="14"/>
+      <x:c r="P169" s="14"/>
     </x:row>
     <x:row r="170" ht="22" customHeight="1">
       <x:c r="A170" s="17"/>
@@ -3324,8 +3496,9 @@
       <x:c r="K170" s="14"/>
       <x:c r="L170" s="14"/>
       <x:c r="M170" s="14"/>
-      <x:c r="N170" s="14"/>
+      <x:c r="N170" s="17"/>
       <x:c r="O170" s="14"/>
+      <x:c r="P170" s="14"/>
     </x:row>
     <x:row r="171" ht="22" customHeight="1">
       <x:c r="A171" s="17"/>
@@ -3341,8 +3514,9 @@
       <x:c r="K171" s="14"/>
       <x:c r="L171" s="14"/>
       <x:c r="M171" s="14"/>
-      <x:c r="N171" s="14"/>
+      <x:c r="N171" s="17"/>
       <x:c r="O171" s="14"/>
+      <x:c r="P171" s="14"/>
     </x:row>
     <x:row r="172" ht="22" customHeight="1">
       <x:c r="A172" s="17"/>
@@ -3358,8 +3532,9 @@
       <x:c r="K172" s="14"/>
       <x:c r="L172" s="14"/>
       <x:c r="M172" s="14"/>
-      <x:c r="N172" s="14"/>
+      <x:c r="N172" s="17"/>
       <x:c r="O172" s="14"/>
+      <x:c r="P172" s="14"/>
     </x:row>
     <x:row r="173" ht="22" customHeight="1">
       <x:c r="A173" s="17"/>
@@ -3375,8 +3550,9 @@
       <x:c r="K173" s="14"/>
       <x:c r="L173" s="14"/>
       <x:c r="M173" s="14"/>
-      <x:c r="N173" s="14"/>
+      <x:c r="N173" s="17"/>
       <x:c r="O173" s="14"/>
+      <x:c r="P173" s="14"/>
     </x:row>
     <x:row r="174" ht="22" customHeight="1">
       <x:c r="A174" s="17"/>
@@ -3392,8 +3568,9 @@
       <x:c r="K174" s="14"/>
       <x:c r="L174" s="14"/>
       <x:c r="M174" s="14"/>
-      <x:c r="N174" s="14"/>
+      <x:c r="N174" s="17"/>
       <x:c r="O174" s="14"/>
+      <x:c r="P174" s="14"/>
     </x:row>
     <x:row r="175" ht="22" customHeight="1">
       <x:c r="A175" s="17"/>
@@ -3409,8 +3586,9 @@
       <x:c r="K175" s="14"/>
       <x:c r="L175" s="14"/>
       <x:c r="M175" s="14"/>
-      <x:c r="N175" s="14"/>
+      <x:c r="N175" s="17"/>
       <x:c r="O175" s="14"/>
+      <x:c r="P175" s="14"/>
     </x:row>
     <x:row r="176" ht="22" customHeight="1">
       <x:c r="A176" s="17"/>
@@ -3426,8 +3604,9 @@
       <x:c r="K176" s="14"/>
       <x:c r="L176" s="14"/>
       <x:c r="M176" s="14"/>
-      <x:c r="N176" s="14"/>
+      <x:c r="N176" s="17"/>
       <x:c r="O176" s="14"/>
+      <x:c r="P176" s="14"/>
     </x:row>
     <x:row r="177" ht="22" customHeight="1">
       <x:c r="A177" s="17"/>
@@ -3443,8 +3622,9 @@
       <x:c r="K177" s="14"/>
       <x:c r="L177" s="14"/>
       <x:c r="M177" s="14"/>
-      <x:c r="N177" s="14"/>
+      <x:c r="N177" s="17"/>
       <x:c r="O177" s="14"/>
+      <x:c r="P177" s="14"/>
     </x:row>
     <x:row r="178" ht="22" customHeight="1">
       <x:c r="A178" s="17"/>
@@ -3460,8 +3640,9 @@
       <x:c r="K178" s="14"/>
       <x:c r="L178" s="14"/>
       <x:c r="M178" s="14"/>
-      <x:c r="N178" s="14"/>
+      <x:c r="N178" s="17"/>
       <x:c r="O178" s="14"/>
+      <x:c r="P178" s="14"/>
     </x:row>
     <x:row r="179" ht="22" customHeight="1">
       <x:c r="A179" s="17"/>
@@ -3477,8 +3658,9 @@
       <x:c r="K179" s="14"/>
       <x:c r="L179" s="14"/>
       <x:c r="M179" s="14"/>
-      <x:c r="N179" s="14"/>
+      <x:c r="N179" s="17"/>
       <x:c r="O179" s="14"/>
+      <x:c r="P179" s="14"/>
     </x:row>
     <x:row r="180" ht="22" customHeight="1">
       <x:c r="A180" s="17"/>
@@ -3494,8 +3676,9 @@
       <x:c r="K180" s="14"/>
       <x:c r="L180" s="14"/>
       <x:c r="M180" s="14"/>
-      <x:c r="N180" s="14"/>
+      <x:c r="N180" s="17"/>
       <x:c r="O180" s="14"/>
+      <x:c r="P180" s="14"/>
     </x:row>
     <x:row r="181" ht="22" customHeight="1">
       <x:c r="A181" s="17"/>
@@ -3511,8 +3694,9 @@
       <x:c r="K181" s="14"/>
       <x:c r="L181" s="14"/>
       <x:c r="M181" s="14"/>
-      <x:c r="N181" s="14"/>
+      <x:c r="N181" s="17"/>
       <x:c r="O181" s="14"/>
+      <x:c r="P181" s="14"/>
     </x:row>
     <x:row r="182" ht="22" customHeight="1">
       <x:c r="A182" s="17"/>
@@ -3528,8 +3712,9 @@
       <x:c r="K182" s="14"/>
       <x:c r="L182" s="14"/>
       <x:c r="M182" s="14"/>
-      <x:c r="N182" s="14"/>
+      <x:c r="N182" s="17"/>
       <x:c r="O182" s="14"/>
+      <x:c r="P182" s="14"/>
     </x:row>
     <x:row r="183" ht="22" customHeight="1">
       <x:c r="A183" s="17"/>
@@ -3545,8 +3730,9 @@
       <x:c r="K183" s="14"/>
       <x:c r="L183" s="14"/>
       <x:c r="M183" s="14"/>
-      <x:c r="N183" s="14"/>
+      <x:c r="N183" s="17"/>
       <x:c r="O183" s="14"/>
+      <x:c r="P183" s="14"/>
     </x:row>
     <x:row r="184" ht="22" customHeight="1">
       <x:c r="A184" s="17"/>
@@ -3562,8 +3748,9 @@
       <x:c r="K184" s="14"/>
       <x:c r="L184" s="14"/>
       <x:c r="M184" s="14"/>
-      <x:c r="N184" s="14"/>
+      <x:c r="N184" s="17"/>
       <x:c r="O184" s="14"/>
+      <x:c r="P184" s="14"/>
     </x:row>
     <x:row r="185" ht="22" customHeight="1">
       <x:c r="A185" s="17"/>
@@ -3579,8 +3766,9 @@
       <x:c r="K185" s="14"/>
       <x:c r="L185" s="14"/>
       <x:c r="M185" s="14"/>
-      <x:c r="N185" s="14"/>
+      <x:c r="N185" s="17"/>
       <x:c r="O185" s="14"/>
+      <x:c r="P185" s="14"/>
     </x:row>
     <x:row r="186" ht="22" customHeight="1">
       <x:c r="A186" s="17"/>
@@ -3596,8 +3784,9 @@
       <x:c r="K186" s="14"/>
       <x:c r="L186" s="14"/>
       <x:c r="M186" s="14"/>
-      <x:c r="N186" s="14"/>
+      <x:c r="N186" s="17"/>
       <x:c r="O186" s="14"/>
+      <x:c r="P186" s="14"/>
     </x:row>
     <x:row r="187" ht="22" customHeight="1">
       <x:c r="A187" s="17"/>
@@ -3613,8 +3802,9 @@
       <x:c r="K187" s="14"/>
       <x:c r="L187" s="14"/>
       <x:c r="M187" s="14"/>
-      <x:c r="N187" s="14"/>
+      <x:c r="N187" s="17"/>
       <x:c r="O187" s="14"/>
+      <x:c r="P187" s="14"/>
     </x:row>
     <x:row r="188" ht="22" customHeight="1">
       <x:c r="A188" s="17"/>
@@ -3630,8 +3820,9 @@
       <x:c r="K188" s="14"/>
       <x:c r="L188" s="14"/>
       <x:c r="M188" s="14"/>
-      <x:c r="N188" s="14"/>
+      <x:c r="N188" s="17"/>
       <x:c r="O188" s="14"/>
+      <x:c r="P188" s="14"/>
     </x:row>
     <x:row r="189" ht="22" customHeight="1">
       <x:c r="A189" s="17"/>
@@ -3647,8 +3838,9 @@
       <x:c r="K189" s="14"/>
       <x:c r="L189" s="14"/>
       <x:c r="M189" s="14"/>
-      <x:c r="N189" s="14"/>
+      <x:c r="N189" s="17"/>
       <x:c r="O189" s="14"/>
+      <x:c r="P189" s="14"/>
     </x:row>
     <x:row r="190" ht="22" customHeight="1">
       <x:c r="A190" s="17"/>
@@ -3664,8 +3856,9 @@
       <x:c r="K190" s="14"/>
       <x:c r="L190" s="14"/>
       <x:c r="M190" s="14"/>
-      <x:c r="N190" s="14"/>
+      <x:c r="N190" s="17"/>
       <x:c r="O190" s="14"/>
+      <x:c r="P190" s="14"/>
     </x:row>
     <x:row r="191" ht="22" customHeight="1">
       <x:c r="A191" s="17"/>
@@ -3681,8 +3874,9 @@
       <x:c r="K191" s="14"/>
       <x:c r="L191" s="14"/>
       <x:c r="M191" s="14"/>
-      <x:c r="N191" s="14"/>
+      <x:c r="N191" s="17"/>
       <x:c r="O191" s="14"/>
+      <x:c r="P191" s="14"/>
     </x:row>
     <x:row r="192" ht="22" customHeight="1">
       <x:c r="A192" s="17"/>
@@ -3698,8 +3892,9 @@
       <x:c r="K192" s="14"/>
       <x:c r="L192" s="14"/>
       <x:c r="M192" s="14"/>
-      <x:c r="N192" s="14"/>
+      <x:c r="N192" s="17"/>
       <x:c r="O192" s="14"/>
+      <x:c r="P192" s="14"/>
     </x:row>
     <x:row r="193" ht="22" customHeight="1">
       <x:c r="A193" s="17"/>
@@ -3715,8 +3910,9 @@
       <x:c r="K193" s="14"/>
       <x:c r="L193" s="14"/>
       <x:c r="M193" s="14"/>
-      <x:c r="N193" s="14"/>
+      <x:c r="N193" s="17"/>
       <x:c r="O193" s="14"/>
+      <x:c r="P193" s="14"/>
     </x:row>
     <x:row r="194" ht="22" customHeight="1">
       <x:c r="A194" s="17"/>
@@ -3732,8 +3928,9 @@
       <x:c r="K194" s="14"/>
       <x:c r="L194" s="14"/>
       <x:c r="M194" s="14"/>
-      <x:c r="N194" s="14"/>
+      <x:c r="N194" s="17"/>
       <x:c r="O194" s="14"/>
+      <x:c r="P194" s="14"/>
     </x:row>
     <x:row r="195" ht="22" customHeight="1">
       <x:c r="A195" s="17"/>
@@ -3749,8 +3946,9 @@
       <x:c r="K195" s="14"/>
       <x:c r="L195" s="14"/>
       <x:c r="M195" s="14"/>
-      <x:c r="N195" s="14"/>
+      <x:c r="N195" s="17"/>
       <x:c r="O195" s="14"/>
+      <x:c r="P195" s="14"/>
     </x:row>
     <x:row r="196" ht="22" customHeight="1">
       <x:c r="A196" s="17"/>
@@ -3766,8 +3964,9 @@
       <x:c r="K196" s="14"/>
       <x:c r="L196" s="14"/>
       <x:c r="M196" s="14"/>
-      <x:c r="N196" s="14"/>
+      <x:c r="N196" s="17"/>
       <x:c r="O196" s="14"/>
+      <x:c r="P196" s="14"/>
     </x:row>
     <x:row r="197" ht="22" customHeight="1">
       <x:c r="A197" s="17"/>
@@ -3783,8 +3982,9 @@
       <x:c r="K197" s="14"/>
       <x:c r="L197" s="14"/>
       <x:c r="M197" s="14"/>
-      <x:c r="N197" s="14"/>
+      <x:c r="N197" s="17"/>
       <x:c r="O197" s="14"/>
+      <x:c r="P197" s="14"/>
     </x:row>
     <x:row r="198" ht="22" customHeight="1">
       <x:c r="A198" s="17"/>
@@ -3800,8 +4000,9 @@
       <x:c r="K198" s="14"/>
       <x:c r="L198" s="14"/>
       <x:c r="M198" s="14"/>
-      <x:c r="N198" s="14"/>
+      <x:c r="N198" s="17"/>
       <x:c r="O198" s="14"/>
+      <x:c r="P198" s="14"/>
     </x:row>
     <x:row r="199" ht="22" customHeight="1">
       <x:c r="A199" s="17"/>
@@ -3817,8 +4018,9 @@
       <x:c r="K199" s="14"/>
       <x:c r="L199" s="14"/>
       <x:c r="M199" s="14"/>
-      <x:c r="N199" s="14"/>
+      <x:c r="N199" s="17"/>
       <x:c r="O199" s="14"/>
+      <x:c r="P199" s="14"/>
     </x:row>
     <x:row r="200" ht="22" customHeight="1">
       <x:c r="A200" s="17"/>
@@ -3834,8 +4036,9 @@
       <x:c r="K200" s="14"/>
       <x:c r="L200" s="14"/>
       <x:c r="M200" s="14"/>
-      <x:c r="N200" s="14"/>
+      <x:c r="N200" s="17"/>
       <x:c r="O200" s="14"/>
+      <x:c r="P200" s="14"/>
     </x:row>
     <x:row r="201" ht="22" customHeight="1">
       <x:c r="A201" s="17"/>
@@ -3851,8 +4054,9 @@
       <x:c r="K201" s="14"/>
       <x:c r="L201" s="14"/>
       <x:c r="M201" s="14"/>
-      <x:c r="N201" s="14"/>
+      <x:c r="N201" s="17"/>
       <x:c r="O201" s="14"/>
+      <x:c r="P201" s="14"/>
     </x:row>
     <x:row r="202" ht="22" customHeight="1">
       <x:c r="A202" s="17"/>
@@ -3868,8 +4072,9 @@
       <x:c r="K202" s="14"/>
       <x:c r="L202" s="14"/>
       <x:c r="M202" s="14"/>
-      <x:c r="N202" s="14"/>
+      <x:c r="N202" s="17"/>
       <x:c r="O202" s="14"/>
+      <x:c r="P202" s="14"/>
     </x:row>
     <x:row r="203" ht="22" customHeight="1">
       <x:c r="A203" s="17"/>
@@ -3885,8 +4090,9 @@
       <x:c r="K203" s="14"/>
       <x:c r="L203" s="14"/>
       <x:c r="M203" s="14"/>
-      <x:c r="N203" s="14"/>
+      <x:c r="N203" s="17"/>
       <x:c r="O203" s="14"/>
+      <x:c r="P203" s="14"/>
     </x:row>
     <x:row r="204" ht="22" customHeight="1">
       <x:c r="A204" s="17"/>
@@ -3902,8 +4108,9 @@
       <x:c r="K204" s="14"/>
       <x:c r="L204" s="14"/>
       <x:c r="M204" s="14"/>
-      <x:c r="N204" s="14"/>
+      <x:c r="N204" s="17"/>
       <x:c r="O204" s="14"/>
+      <x:c r="P204" s="14"/>
     </x:row>
     <x:row r="205" ht="22" customHeight="1">
       <x:c r="A205" s="17"/>
@@ -3919,8 +4126,9 @@
       <x:c r="K205" s="14"/>
       <x:c r="L205" s="14"/>
       <x:c r="M205" s="14"/>
-      <x:c r="N205" s="14"/>
+      <x:c r="N205" s="17"/>
       <x:c r="O205" s="14"/>
+      <x:c r="P205" s="14"/>
     </x:row>
     <x:row r="206" ht="22" customHeight="1">
       <x:c r="A206" s="17"/>
@@ -3936,8 +4144,9 @@
       <x:c r="K206" s="14"/>
       <x:c r="L206" s="14"/>
       <x:c r="M206" s="14"/>
-      <x:c r="N206" s="14"/>
+      <x:c r="N206" s="17"/>
       <x:c r="O206" s="14"/>
+      <x:c r="P206" s="14"/>
     </x:row>
     <x:row r="207" ht="22" customHeight="1">
       <x:c r="A207" s="17"/>
@@ -3953,8 +4162,9 @@
       <x:c r="K207" s="14"/>
       <x:c r="L207" s="14"/>
       <x:c r="M207" s="14"/>
-      <x:c r="N207" s="14"/>
+      <x:c r="N207" s="17"/>
       <x:c r="O207" s="14"/>
+      <x:c r="P207" s="14"/>
     </x:row>
     <x:row r="208" ht="22" customHeight="1">
       <x:c r="A208" s="17"/>
@@ -3970,8 +4180,9 @@
       <x:c r="K208" s="14"/>
       <x:c r="L208" s="14"/>
       <x:c r="M208" s="14"/>
-      <x:c r="N208" s="14"/>
+      <x:c r="N208" s="17"/>
       <x:c r="O208" s="14"/>
+      <x:c r="P208" s="14"/>
     </x:row>
     <x:row r="209" ht="22" customHeight="1">
       <x:c r="A209" s="17"/>
@@ -3987,8 +4198,9 @@
       <x:c r="K209" s="14"/>
       <x:c r="L209" s="14"/>
       <x:c r="M209" s="14"/>
-      <x:c r="N209" s="14"/>
+      <x:c r="N209" s="17"/>
       <x:c r="O209" s="14"/>
+      <x:c r="P209" s="14"/>
     </x:row>
     <x:row r="210" ht="22" customHeight="1">
       <x:c r="A210" s="17"/>
@@ -4004,8 +4216,9 @@
       <x:c r="K210" s="14"/>
       <x:c r="L210" s="14"/>
       <x:c r="M210" s="14"/>
-      <x:c r="N210" s="14"/>
+      <x:c r="N210" s="17"/>
       <x:c r="O210" s="14"/>
+      <x:c r="P210" s="14"/>
     </x:row>
     <x:row r="211" ht="22" customHeight="1">
       <x:c r="A211" s="17"/>
@@ -4021,8 +4234,9 @@
       <x:c r="K211" s="14"/>
       <x:c r="L211" s="14"/>
       <x:c r="M211" s="14"/>
-      <x:c r="N211" s="14"/>
+      <x:c r="N211" s="17"/>
       <x:c r="O211" s="14"/>
+      <x:c r="P211" s="14"/>
     </x:row>
     <x:row r="212" ht="22" customHeight="1">
       <x:c r="A212" s="17"/>
@@ -4038,8 +4252,9 @@
       <x:c r="K212" s="14"/>
       <x:c r="L212" s="14"/>
       <x:c r="M212" s="14"/>
-      <x:c r="N212" s="14"/>
+      <x:c r="N212" s="17"/>
       <x:c r="O212" s="14"/>
+      <x:c r="P212" s="14"/>
     </x:row>
     <x:row r="213" ht="22" customHeight="1">
       <x:c r="A213" s="17"/>
@@ -4055,8 +4270,9 @@
       <x:c r="K213" s="14"/>
       <x:c r="L213" s="14"/>
       <x:c r="M213" s="14"/>
-      <x:c r="N213" s="14"/>
+      <x:c r="N213" s="17"/>
       <x:c r="O213" s="14"/>
+      <x:c r="P213" s="14"/>
     </x:row>
     <x:row r="214" ht="22" customHeight="1">
       <x:c r="A214" s="17"/>
@@ -4072,8 +4288,9 @@
       <x:c r="K214" s="14"/>
       <x:c r="L214" s="14"/>
       <x:c r="M214" s="14"/>
-      <x:c r="N214" s="14"/>
+      <x:c r="N214" s="17"/>
       <x:c r="O214" s="14"/>
+      <x:c r="P214" s="14"/>
     </x:row>
     <x:row r="215" ht="22" customHeight="1">
       <x:c r="A215" s="17"/>
@@ -4089,8 +4306,9 @@
       <x:c r="K215" s="14"/>
       <x:c r="L215" s="14"/>
       <x:c r="M215" s="14"/>
-      <x:c r="N215" s="14"/>
+      <x:c r="N215" s="17"/>
       <x:c r="O215" s="14"/>
+      <x:c r="P215" s="14"/>
     </x:row>
     <x:row r="216" ht="22" customHeight="1">
       <x:c r="A216" s="17"/>
@@ -4106,8 +4324,9 @@
       <x:c r="K216" s="14"/>
       <x:c r="L216" s="14"/>
       <x:c r="M216" s="14"/>
-      <x:c r="N216" s="14"/>
+      <x:c r="N216" s="17"/>
       <x:c r="O216" s="14"/>
+      <x:c r="P216" s="14"/>
     </x:row>
     <x:row r="217" ht="22" customHeight="1">
       <x:c r="A217" s="17"/>
@@ -4123,8 +4342,9 @@
       <x:c r="K217" s="14"/>
       <x:c r="L217" s="14"/>
       <x:c r="M217" s="14"/>
-      <x:c r="N217" s="14"/>
+      <x:c r="N217" s="17"/>
       <x:c r="O217" s="14"/>
+      <x:c r="P217" s="14"/>
     </x:row>
     <x:row r="218" ht="22" customHeight="1">
       <x:c r="A218" s="17"/>
@@ -4140,8 +4360,9 @@
       <x:c r="K218" s="14"/>
       <x:c r="L218" s="14"/>
       <x:c r="M218" s="14"/>
-      <x:c r="N218" s="14"/>
+      <x:c r="N218" s="17"/>
       <x:c r="O218" s="14"/>
+      <x:c r="P218" s="14"/>
     </x:row>
     <x:row r="219" ht="22" customHeight="1">
       <x:c r="A219" s="17"/>
@@ -4157,8 +4378,9 @@
       <x:c r="K219" s="14"/>
       <x:c r="L219" s="14"/>
       <x:c r="M219" s="14"/>
-      <x:c r="N219" s="14"/>
+      <x:c r="N219" s="17"/>
       <x:c r="O219" s="14"/>
+      <x:c r="P219" s="14"/>
     </x:row>
     <x:row r="220" ht="22" customHeight="1">
       <x:c r="A220" s="17"/>
@@ -4174,8 +4396,9 @@
       <x:c r="K220" s="14"/>
       <x:c r="L220" s="14"/>
       <x:c r="M220" s="14"/>
-      <x:c r="N220" s="14"/>
+      <x:c r="N220" s="17"/>
       <x:c r="O220" s="14"/>
+      <x:c r="P220" s="14"/>
     </x:row>
     <x:row r="221" ht="22" customHeight="1">
       <x:c r="A221" s="17"/>
@@ -4191,8 +4414,9 @@
       <x:c r="K221" s="14"/>
       <x:c r="L221" s="14"/>
       <x:c r="M221" s="14"/>
-      <x:c r="N221" s="14"/>
+      <x:c r="N221" s="17"/>
       <x:c r="O221" s="14"/>
+      <x:c r="P221" s="14"/>
     </x:row>
     <x:row r="222" ht="22" customHeight="1">
       <x:c r="A222" s="17"/>
@@ -4208,8 +4432,9 @@
       <x:c r="K222" s="14"/>
       <x:c r="L222" s="14"/>
       <x:c r="M222" s="14"/>
-      <x:c r="N222" s="14"/>
+      <x:c r="N222" s="17"/>
       <x:c r="O222" s="14"/>
+      <x:c r="P222" s="14"/>
     </x:row>
     <x:row r="223" ht="22" customHeight="1">
       <x:c r="A223" s="17"/>
@@ -4225,8 +4450,9 @@
       <x:c r="K223" s="14"/>
       <x:c r="L223" s="14"/>
       <x:c r="M223" s="14"/>
-      <x:c r="N223" s="14"/>
+      <x:c r="N223" s="17"/>
       <x:c r="O223" s="14"/>
+      <x:c r="P223" s="14"/>
     </x:row>
     <x:row r="224" ht="22" customHeight="1">
       <x:c r="A224" s="17"/>
@@ -4242,8 +4468,9 @@
       <x:c r="K224" s="14"/>
       <x:c r="L224" s="14"/>
       <x:c r="M224" s="14"/>
-      <x:c r="N224" s="14"/>
+      <x:c r="N224" s="17"/>
       <x:c r="O224" s="14"/>
+      <x:c r="P224" s="14"/>
     </x:row>
     <x:row r="225" ht="22" customHeight="1">
       <x:c r="A225" s="17"/>
@@ -4259,8 +4486,9 @@
       <x:c r="K225" s="14"/>
       <x:c r="L225" s="14"/>
       <x:c r="M225" s="14"/>
-      <x:c r="N225" s="14"/>
+      <x:c r="N225" s="17"/>
       <x:c r="O225" s="14"/>
+      <x:c r="P225" s="14"/>
     </x:row>
     <x:row r="226" ht="22" customHeight="1">
       <x:c r="A226" s="17"/>
@@ -4276,8 +4504,9 @@
       <x:c r="K226" s="14"/>
       <x:c r="L226" s="14"/>
       <x:c r="M226" s="14"/>
-      <x:c r="N226" s="14"/>
+      <x:c r="N226" s="17"/>
       <x:c r="O226" s="14"/>
+      <x:c r="P226" s="14"/>
     </x:row>
     <x:row r="227" ht="22" customHeight="1">
       <x:c r="A227" s="17"/>
@@ -4293,8 +4522,9 @@
       <x:c r="K227" s="14"/>
       <x:c r="L227" s="14"/>
       <x:c r="M227" s="14"/>
-      <x:c r="N227" s="14"/>
+      <x:c r="N227" s="17"/>
       <x:c r="O227" s="14"/>
+      <x:c r="P227" s="14"/>
     </x:row>
     <x:row r="228" ht="22" customHeight="1">
       <x:c r="A228" s="17"/>
@@ -4310,8 +4540,9 @@
       <x:c r="K228" s="14"/>
       <x:c r="L228" s="14"/>
       <x:c r="M228" s="14"/>
-      <x:c r="N228" s="14"/>
+      <x:c r="N228" s="17"/>
       <x:c r="O228" s="14"/>
+      <x:c r="P228" s="14"/>
     </x:row>
     <x:row r="229" ht="22" customHeight="1">
       <x:c r="A229" s="17"/>
@@ -4327,8 +4558,9 @@
       <x:c r="K229" s="14"/>
       <x:c r="L229" s="14"/>
       <x:c r="M229" s="14"/>
-      <x:c r="N229" s="14"/>
+      <x:c r="N229" s="17"/>
       <x:c r="O229" s="14"/>
+      <x:c r="P229" s="14"/>
     </x:row>
     <x:row r="230" ht="22" customHeight="1">
       <x:c r="A230" s="17"/>
@@ -4344,8 +4576,9 @@
       <x:c r="K230" s="14"/>
       <x:c r="L230" s="14"/>
       <x:c r="M230" s="14"/>
-      <x:c r="N230" s="14"/>
+      <x:c r="N230" s="17"/>
       <x:c r="O230" s="14"/>
+      <x:c r="P230" s="14"/>
     </x:row>
     <x:row r="231" ht="22" customHeight="1">
       <x:c r="A231" s="17"/>
@@ -4361,8 +4594,9 @@
       <x:c r="K231" s="14"/>
       <x:c r="L231" s="14"/>
       <x:c r="M231" s="14"/>
-      <x:c r="N231" s="14"/>
+      <x:c r="N231" s="17"/>
       <x:c r="O231" s="14"/>
+      <x:c r="P231" s="14"/>
     </x:row>
     <x:row r="232" ht="22" customHeight="1">
       <x:c r="A232" s="17"/>
@@ -4378,8 +4612,9 @@
       <x:c r="K232" s="14"/>
       <x:c r="L232" s="14"/>
       <x:c r="M232" s="14"/>
-      <x:c r="N232" s="14"/>
+      <x:c r="N232" s="17"/>
       <x:c r="O232" s="14"/>
+      <x:c r="P232" s="14"/>
     </x:row>
     <x:row r="233" ht="22" customHeight="1">
       <x:c r="A233" s="17"/>
@@ -4395,8 +4630,9 @@
       <x:c r="K233" s="14"/>
       <x:c r="L233" s="14"/>
       <x:c r="M233" s="14"/>
-      <x:c r="N233" s="14"/>
+      <x:c r="N233" s="17"/>
       <x:c r="O233" s="14"/>
+      <x:c r="P233" s="14"/>
     </x:row>
     <x:row r="234" ht="22" customHeight="1">
       <x:c r="A234" s="17"/>
@@ -4412,8 +4648,9 @@
       <x:c r="K234" s="14"/>
       <x:c r="L234" s="14"/>
       <x:c r="M234" s="14"/>
-      <x:c r="N234" s="14"/>
+      <x:c r="N234" s="17"/>
       <x:c r="O234" s="14"/>
+      <x:c r="P234" s="14"/>
     </x:row>
     <x:row r="235" ht="22" customHeight="1">
       <x:c r="A235" s="17"/>
@@ -4429,8 +4666,9 @@
       <x:c r="K235" s="14"/>
       <x:c r="L235" s="14"/>
       <x:c r="M235" s="14"/>
-      <x:c r="N235" s="14"/>
+      <x:c r="N235" s="17"/>
       <x:c r="O235" s="14"/>
+      <x:c r="P235" s="14"/>
     </x:row>
     <x:row r="236" ht="22" customHeight="1">
       <x:c r="A236" s="17"/>
@@ -4446,8 +4684,9 @@
       <x:c r="K236" s="14"/>
       <x:c r="L236" s="14"/>
       <x:c r="M236" s="14"/>
-      <x:c r="N236" s="14"/>
+      <x:c r="N236" s="17"/>
       <x:c r="O236" s="14"/>
+      <x:c r="P236" s="14"/>
     </x:row>
     <x:row r="237" ht="22" customHeight="1">
       <x:c r="A237" s="17"/>
@@ -4463,8 +4702,9 @@
       <x:c r="K237" s="14"/>
       <x:c r="L237" s="14"/>
       <x:c r="M237" s="14"/>
-      <x:c r="N237" s="14"/>
+      <x:c r="N237" s="17"/>
       <x:c r="O237" s="14"/>
+      <x:c r="P237" s="14"/>
     </x:row>
     <x:row r="238" ht="22" customHeight="1">
       <x:c r="A238" s="17"/>
@@ -4480,8 +4720,9 @@
       <x:c r="K238" s="14"/>
       <x:c r="L238" s="14"/>
       <x:c r="M238" s="14"/>
-      <x:c r="N238" s="14"/>
+      <x:c r="N238" s="17"/>
       <x:c r="O238" s="14"/>
+      <x:c r="P238" s="14"/>
     </x:row>
     <x:row r="239" ht="22" customHeight="1">
       <x:c r="A239" s="17"/>
@@ -4497,8 +4738,9 @@
       <x:c r="K239" s="14"/>
       <x:c r="L239" s="14"/>
       <x:c r="M239" s="14"/>
-      <x:c r="N239" s="14"/>
+      <x:c r="N239" s="17"/>
       <x:c r="O239" s="14"/>
+      <x:c r="P239" s="14"/>
     </x:row>
     <x:row r="240" ht="22" customHeight="1">
       <x:c r="A240" s="17"/>
@@ -4514,8 +4756,9 @@
       <x:c r="K240" s="14"/>
       <x:c r="L240" s="14"/>
       <x:c r="M240" s="14"/>
-      <x:c r="N240" s="14"/>
+      <x:c r="N240" s="17"/>
       <x:c r="O240" s="14"/>
+      <x:c r="P240" s="14"/>
     </x:row>
     <x:row r="241" ht="22" customHeight="1">
       <x:c r="A241" s="17"/>
@@ -4531,8 +4774,9 @@
       <x:c r="K241" s="14"/>
       <x:c r="L241" s="14"/>
       <x:c r="M241" s="14"/>
-      <x:c r="N241" s="14"/>
+      <x:c r="N241" s="17"/>
       <x:c r="O241" s="14"/>
+      <x:c r="P241" s="14"/>
     </x:row>
     <x:row r="242" ht="22" customHeight="1">
       <x:c r="A242" s="17"/>
@@ -4548,8 +4792,9 @@
       <x:c r="K242" s="14"/>
       <x:c r="L242" s="14"/>
       <x:c r="M242" s="14"/>
-      <x:c r="N242" s="14"/>
+      <x:c r="N242" s="17"/>
       <x:c r="O242" s="14"/>
+      <x:c r="P242" s="14"/>
     </x:row>
     <x:row r="243" ht="22" customHeight="1">
       <x:c r="A243" s="17"/>
@@ -4565,8 +4810,9 @@
       <x:c r="K243" s="14"/>
       <x:c r="L243" s="14"/>
       <x:c r="M243" s="14"/>
-      <x:c r="N243" s="14"/>
+      <x:c r="N243" s="17"/>
       <x:c r="O243" s="14"/>
+      <x:c r="P243" s="14"/>
     </x:row>
     <x:row r="244" ht="22" customHeight="1">
       <x:c r="A244" s="17"/>
@@ -4582,8 +4828,9 @@
       <x:c r="K244" s="14"/>
       <x:c r="L244" s="14"/>
       <x:c r="M244" s="14"/>
-      <x:c r="N244" s="14"/>
+      <x:c r="N244" s="17"/>
       <x:c r="O244" s="14"/>
+      <x:c r="P244" s="14"/>
     </x:row>
     <x:row r="245" ht="22" customHeight="1">
       <x:c r="A245" s="17"/>
@@ -4599,8 +4846,9 @@
       <x:c r="K245" s="14"/>
       <x:c r="L245" s="14"/>
       <x:c r="M245" s="14"/>
-      <x:c r="N245" s="14"/>
+      <x:c r="N245" s="17"/>
       <x:c r="O245" s="14"/>
+      <x:c r="P245" s="14"/>
     </x:row>
     <x:row r="246" ht="22" customHeight="1">
       <x:c r="A246" s="17"/>
@@ -4616,8 +4864,9 @@
       <x:c r="K246" s="14"/>
       <x:c r="L246" s="14"/>
       <x:c r="M246" s="14"/>
-      <x:c r="N246" s="14"/>
+      <x:c r="N246" s="17"/>
       <x:c r="O246" s="14"/>
+      <x:c r="P246" s="14"/>
     </x:row>
     <x:row r="247" ht="22" customHeight="1">
       <x:c r="A247" s="17"/>
@@ -4633,8 +4882,9 @@
       <x:c r="K247" s="14"/>
       <x:c r="L247" s="14"/>
       <x:c r="M247" s="14"/>
-      <x:c r="N247" s="14"/>
+      <x:c r="N247" s="17"/>
       <x:c r="O247" s="14"/>
+      <x:c r="P247" s="14"/>
     </x:row>
     <x:row r="248" ht="22" customHeight="1">
       <x:c r="A248" s="17"/>
@@ -4650,8 +4900,9 @@
       <x:c r="K248" s="14"/>
       <x:c r="L248" s="14"/>
       <x:c r="M248" s="14"/>
-      <x:c r="N248" s="14"/>
+      <x:c r="N248" s="17"/>
       <x:c r="O248" s="14"/>
+      <x:c r="P248" s="14"/>
     </x:row>
     <x:row r="249" ht="22" customHeight="1">
       <x:c r="A249" s="17"/>
@@ -4667,8 +4918,9 @@
       <x:c r="K249" s="14"/>
       <x:c r="L249" s="14"/>
       <x:c r="M249" s="14"/>
-      <x:c r="N249" s="14"/>
+      <x:c r="N249" s="17"/>
       <x:c r="O249" s="14"/>
+      <x:c r="P249" s="14"/>
     </x:row>
     <x:row r="250" ht="22" customHeight="1">
       <x:c r="A250" s="17"/>
@@ -4684,8 +4936,9 @@
       <x:c r="K250" s="14"/>
       <x:c r="L250" s="14"/>
       <x:c r="M250" s="14"/>
-      <x:c r="N250" s="14"/>
+      <x:c r="N250" s="17"/>
       <x:c r="O250" s="14"/>
+      <x:c r="P250" s="14"/>
     </x:row>
     <x:row r="251" ht="22" customHeight="1">
       <x:c r="A251" s="17"/>
@@ -4701,8 +4954,9 @@
       <x:c r="K251" s="14"/>
       <x:c r="L251" s="14"/>
       <x:c r="M251" s="14"/>
-      <x:c r="N251" s="14"/>
+      <x:c r="N251" s="17"/>
       <x:c r="O251" s="14"/>
+      <x:c r="P251" s="14"/>
     </x:row>
     <x:row r="252" ht="22" customHeight="1">
       <x:c r="A252" s="17"/>
@@ -4718,8 +4972,9 @@
       <x:c r="K252" s="14"/>
       <x:c r="L252" s="14"/>
       <x:c r="M252" s="14"/>
-      <x:c r="N252" s="14"/>
+      <x:c r="N252" s="17"/>
       <x:c r="O252" s="14"/>
+      <x:c r="P252" s="14"/>
     </x:row>
     <x:row r="253" ht="22" customHeight="1">
       <x:c r="A253" s="17"/>
@@ -4735,8 +4990,9 @@
       <x:c r="K253" s="14"/>
       <x:c r="L253" s="14"/>
       <x:c r="M253" s="14"/>
-      <x:c r="N253" s="14"/>
+      <x:c r="N253" s="17"/>
       <x:c r="O253" s="14"/>
+      <x:c r="P253" s="14"/>
     </x:row>
     <x:row r="254" ht="22" customHeight="1">
       <x:c r="A254" s="17"/>
@@ -4752,8 +5008,9 @@
       <x:c r="K254" s="14"/>
       <x:c r="L254" s="14"/>
       <x:c r="M254" s="14"/>
-      <x:c r="N254" s="14"/>
+      <x:c r="N254" s="17"/>
       <x:c r="O254" s="14"/>
+      <x:c r="P254" s="14"/>
     </x:row>
     <x:row r="255" ht="22" customHeight="1">
       <x:c r="A255" s="17"/>
@@ -4769,8 +5026,9 @@
       <x:c r="K255" s="14"/>
       <x:c r="L255" s="14"/>
       <x:c r="M255" s="14"/>
-      <x:c r="N255" s="14"/>
+      <x:c r="N255" s="17"/>
       <x:c r="O255" s="14"/>
+      <x:c r="P255" s="14"/>
     </x:row>
     <x:row r="256" ht="22" customHeight="1">
       <x:c r="A256" s="17"/>
@@ -4786,8 +5044,9 @@
       <x:c r="K256" s="14"/>
       <x:c r="L256" s="14"/>
       <x:c r="M256" s="14"/>
-      <x:c r="N256" s="14"/>
+      <x:c r="N256" s="17"/>
       <x:c r="O256" s="14"/>
+      <x:c r="P256" s="14"/>
     </x:row>
     <x:row r="257" ht="22" customHeight="1">
       <x:c r="A257" s="17"/>
@@ -4803,8 +5062,9 @@
       <x:c r="K257" s="14"/>
       <x:c r="L257" s="14"/>
       <x:c r="M257" s="14"/>
-      <x:c r="N257" s="14"/>
+      <x:c r="N257" s="17"/>
       <x:c r="O257" s="14"/>
+      <x:c r="P257" s="14"/>
     </x:row>
     <x:row r="258" ht="22" customHeight="1">
       <x:c r="A258" s="17"/>
@@ -4820,8 +5080,9 @@
       <x:c r="K258" s="14"/>
       <x:c r="L258" s="14"/>
       <x:c r="M258" s="14"/>
-      <x:c r="N258" s="14"/>
+      <x:c r="N258" s="17"/>
       <x:c r="O258" s="14"/>
+      <x:c r="P258" s="14"/>
     </x:row>
     <x:row r="259" ht="22" customHeight="1">
       <x:c r="A259" s="17"/>
@@ -4837,8 +5098,9 @@
       <x:c r="K259" s="14"/>
       <x:c r="L259" s="14"/>
       <x:c r="M259" s="14"/>
-      <x:c r="N259" s="14"/>
+      <x:c r="N259" s="17"/>
       <x:c r="O259" s="14"/>
+      <x:c r="P259" s="14"/>
     </x:row>
     <x:row r="260" ht="22" customHeight="1">
       <x:c r="A260" s="17"/>
@@ -4854,8 +5116,9 @@
       <x:c r="K260" s="14"/>
       <x:c r="L260" s="14"/>
       <x:c r="M260" s="14"/>
-      <x:c r="N260" s="14"/>
+      <x:c r="N260" s="17"/>
       <x:c r="O260" s="14"/>
+      <x:c r="P260" s="14"/>
     </x:row>
     <x:row r="261" ht="22" customHeight="1">
       <x:c r="A261" s="17"/>
@@ -4871,8 +5134,9 @@
       <x:c r="K261" s="14"/>
       <x:c r="L261" s="14"/>
       <x:c r="M261" s="14"/>
-      <x:c r="N261" s="14"/>
+      <x:c r="N261" s="17"/>
       <x:c r="O261" s="14"/>
+      <x:c r="P261" s="14"/>
     </x:row>
     <x:row r="262" ht="22" customHeight="1">
       <x:c r="A262" s="17"/>
@@ -4888,8 +5152,9 @@
       <x:c r="K262" s="14"/>
       <x:c r="L262" s="14"/>
       <x:c r="M262" s="14"/>
-      <x:c r="N262" s="14"/>
+      <x:c r="N262" s="17"/>
       <x:c r="O262" s="14"/>
+      <x:c r="P262" s="14"/>
     </x:row>
     <x:row r="263" ht="22" customHeight="1">
       <x:c r="A263" s="17"/>
@@ -4905,8 +5170,9 @@
       <x:c r="K263" s="14"/>
       <x:c r="L263" s="14"/>
       <x:c r="M263" s="14"/>
-      <x:c r="N263" s="14"/>
+      <x:c r="N263" s="17"/>
       <x:c r="O263" s="14"/>
+      <x:c r="P263" s="14"/>
     </x:row>
     <x:row r="264" ht="22" customHeight="1">
       <x:c r="A264" s="17"/>
@@ -4922,8 +5188,9 @@
       <x:c r="K264" s="14"/>
       <x:c r="L264" s="14"/>
       <x:c r="M264" s="14"/>
-      <x:c r="N264" s="14"/>
+      <x:c r="N264" s="17"/>
       <x:c r="O264" s="14"/>
+      <x:c r="P264" s="14"/>
     </x:row>
     <x:row r="265" ht="22" customHeight="1">
       <x:c r="A265" s="17"/>
@@ -4939,8 +5206,9 @@
       <x:c r="K265" s="14"/>
       <x:c r="L265" s="14"/>
       <x:c r="M265" s="14"/>
-      <x:c r="N265" s="14"/>
+      <x:c r="N265" s="17"/>
       <x:c r="O265" s="14"/>
+      <x:c r="P265" s="14"/>
     </x:row>
     <x:row r="266" ht="22" customHeight="1">
       <x:c r="A266" s="17"/>
@@ -4956,8 +5224,9 @@
       <x:c r="K266" s="14"/>
       <x:c r="L266" s="14"/>
       <x:c r="M266" s="14"/>
-      <x:c r="N266" s="14"/>
+      <x:c r="N266" s="17"/>
       <x:c r="O266" s="14"/>
+      <x:c r="P266" s="14"/>
     </x:row>
     <x:row r="267" ht="22" customHeight="1">
       <x:c r="A267" s="17"/>
@@ -4973,8 +5242,9 @@
       <x:c r="K267" s="14"/>
       <x:c r="L267" s="14"/>
       <x:c r="M267" s="14"/>
-      <x:c r="N267" s="14"/>
+      <x:c r="N267" s="17"/>
       <x:c r="O267" s="14"/>
+      <x:c r="P267" s="14"/>
     </x:row>
     <x:row r="268" ht="22" customHeight="1">
       <x:c r="A268" s="17"/>
@@ -4990,8 +5260,9 @@
       <x:c r="K268" s="14"/>
       <x:c r="L268" s="14"/>
       <x:c r="M268" s="14"/>
-      <x:c r="N268" s="14"/>
+      <x:c r="N268" s="17"/>
       <x:c r="O268" s="14"/>
+      <x:c r="P268" s="14"/>
     </x:row>
     <x:row r="269" ht="22" customHeight="1">
       <x:c r="A269" s="17"/>
@@ -5007,8 +5278,9 @@
       <x:c r="K269" s="14"/>
       <x:c r="L269" s="14"/>
       <x:c r="M269" s="14"/>
-      <x:c r="N269" s="14"/>
+      <x:c r="N269" s="17"/>
       <x:c r="O269" s="14"/>
+      <x:c r="P269" s="14"/>
     </x:row>
     <x:row r="270" ht="22" customHeight="1">
       <x:c r="A270" s="17"/>
@@ -5024,8 +5296,9 @@
       <x:c r="K270" s="14"/>
       <x:c r="L270" s="14"/>
       <x:c r="M270" s="14"/>
-      <x:c r="N270" s="14"/>
+      <x:c r="N270" s="17"/>
       <x:c r="O270" s="14"/>
+      <x:c r="P270" s="14"/>
     </x:row>
     <x:row r="271" ht="22" customHeight="1">
       <x:c r="A271" s="17"/>
@@ -5041,8 +5314,9 @@
       <x:c r="K271" s="14"/>
       <x:c r="L271" s="14"/>
       <x:c r="M271" s="14"/>
-      <x:c r="N271" s="14"/>
+      <x:c r="N271" s="17"/>
       <x:c r="O271" s="14"/>
+      <x:c r="P271" s="14"/>
     </x:row>
     <x:row r="272" ht="22" customHeight="1">
       <x:c r="A272" s="17"/>
@@ -5058,8 +5332,9 @@
       <x:c r="K272" s="14"/>
       <x:c r="L272" s="14"/>
       <x:c r="M272" s="14"/>
-      <x:c r="N272" s="14"/>
+      <x:c r="N272" s="17"/>
       <x:c r="O272" s="14"/>
+      <x:c r="P272" s="14"/>
     </x:row>
     <x:row r="273" ht="22" customHeight="1">
       <x:c r="A273" s="17"/>
@@ -5075,8 +5350,9 @@
       <x:c r="K273" s="14"/>
       <x:c r="L273" s="14"/>
       <x:c r="M273" s="14"/>
-      <x:c r="N273" s="14"/>
+      <x:c r="N273" s="17"/>
       <x:c r="O273" s="14"/>
+      <x:c r="P273" s="14"/>
     </x:row>
     <x:row r="274" ht="22" customHeight="1">
       <x:c r="A274" s="17"/>
@@ -5092,8 +5368,9 @@
       <x:c r="K274" s="14"/>
       <x:c r="L274" s="14"/>
       <x:c r="M274" s="14"/>
-      <x:c r="N274" s="14"/>
+      <x:c r="N274" s="17"/>
       <x:c r="O274" s="14"/>
+      <x:c r="P274" s="14"/>
     </x:row>
     <x:row r="275" ht="22" customHeight="1">
       <x:c r="A275" s="17"/>
@@ -5109,8 +5386,9 @@
       <x:c r="K275" s="14"/>
       <x:c r="L275" s="14"/>
       <x:c r="M275" s="14"/>
-      <x:c r="N275" s="14"/>
+      <x:c r="N275" s="17"/>
       <x:c r="O275" s="14"/>
+      <x:c r="P275" s="14"/>
     </x:row>
     <x:row r="276" ht="22" customHeight="1">
       <x:c r="A276" s="17"/>
@@ -5126,8 +5404,9 @@
       <x:c r="K276" s="14"/>
       <x:c r="L276" s="14"/>
       <x:c r="M276" s="14"/>
-      <x:c r="N276" s="14"/>
+      <x:c r="N276" s="17"/>
       <x:c r="O276" s="14"/>
+      <x:c r="P276" s="14"/>
     </x:row>
     <x:row r="277" ht="22" customHeight="1">
       <x:c r="A277" s="17"/>
@@ -5143,8 +5422,9 @@
       <x:c r="K277" s="14"/>
       <x:c r="L277" s="14"/>
       <x:c r="M277" s="14"/>
-      <x:c r="N277" s="14"/>
+      <x:c r="N277" s="17"/>
       <x:c r="O277" s="14"/>
+      <x:c r="P277" s="14"/>
     </x:row>
     <x:row r="278" ht="22" customHeight="1">
       <x:c r="A278" s="17"/>
@@ -5160,8 +5440,9 @@
       <x:c r="K278" s="14"/>
       <x:c r="L278" s="14"/>
       <x:c r="M278" s="14"/>
-      <x:c r="N278" s="14"/>
+      <x:c r="N278" s="17"/>
       <x:c r="O278" s="14"/>
+      <x:c r="P278" s="14"/>
     </x:row>
     <x:row r="279" ht="22" customHeight="1">
       <x:c r="A279" s="17"/>
@@ -5177,8 +5458,9 @@
       <x:c r="K279" s="14"/>
       <x:c r="L279" s="14"/>
       <x:c r="M279" s="14"/>
-      <x:c r="N279" s="14"/>
+      <x:c r="N279" s="17"/>
       <x:c r="O279" s="14"/>
+      <x:c r="P279" s="14"/>
     </x:row>
     <x:row r="280" ht="22" customHeight="1">
       <x:c r="A280" s="17"/>
@@ -5194,8 +5476,9 @@
       <x:c r="K280" s="14"/>
       <x:c r="L280" s="14"/>
       <x:c r="M280" s="14"/>
-      <x:c r="N280" s="14"/>
+      <x:c r="N280" s="17"/>
       <x:c r="O280" s="14"/>
+      <x:c r="P280" s="14"/>
     </x:row>
     <x:row r="281" ht="22" customHeight="1">
       <x:c r="A281" s="17"/>
@@ -5211,8 +5494,9 @@
       <x:c r="K281" s="14"/>
       <x:c r="L281" s="14"/>
       <x:c r="M281" s="14"/>
-      <x:c r="N281" s="14"/>
+      <x:c r="N281" s="17"/>
       <x:c r="O281" s="14"/>
+      <x:c r="P281" s="14"/>
     </x:row>
     <x:row r="282" ht="22" customHeight="1">
       <x:c r="A282" s="17"/>
@@ -5228,8 +5512,9 @@
       <x:c r="K282" s="14"/>
       <x:c r="L282" s="14"/>
       <x:c r="M282" s="14"/>
-      <x:c r="N282" s="14"/>
+      <x:c r="N282" s="17"/>
       <x:c r="O282" s="14"/>
+      <x:c r="P282" s="14"/>
     </x:row>
     <x:row r="283" ht="22" customHeight="1">
       <x:c r="A283" s="17"/>
@@ -5245,8 +5530,9 @@
       <x:c r="K283" s="14"/>
       <x:c r="L283" s="14"/>
       <x:c r="M283" s="14"/>
-      <x:c r="N283" s="14"/>
+      <x:c r="N283" s="17"/>
       <x:c r="O283" s="14"/>
+      <x:c r="P283" s="14"/>
     </x:row>
     <x:row r="284" ht="22" customHeight="1">
       <x:c r="A284" s="17"/>
@@ -5262,8 +5548,9 @@
       <x:c r="K284" s="14"/>
       <x:c r="L284" s="14"/>
       <x:c r="M284" s="14"/>
-      <x:c r="N284" s="14"/>
+      <x:c r="N284" s="17"/>
       <x:c r="O284" s="14"/>
+      <x:c r="P284" s="14"/>
     </x:row>
     <x:row r="285" ht="22" customHeight="1">
       <x:c r="A285" s="17"/>
@@ -5279,8 +5566,9 @@
       <x:c r="K285" s="14"/>
       <x:c r="L285" s="14"/>
       <x:c r="M285" s="14"/>
-      <x:c r="N285" s="14"/>
+      <x:c r="N285" s="17"/>
       <x:c r="O285" s="14"/>
+      <x:c r="P285" s="14"/>
     </x:row>
     <x:row r="286" ht="22" customHeight="1">
       <x:c r="A286" s="17"/>
@@ -5296,8 +5584,9 @@
       <x:c r="K286" s="14"/>
       <x:c r="L286" s="14"/>
       <x:c r="M286" s="14"/>
-      <x:c r="N286" s="14"/>
+      <x:c r="N286" s="17"/>
       <x:c r="O286" s="14"/>
+      <x:c r="P286" s="14"/>
     </x:row>
     <x:row r="287" ht="22" customHeight="1">
       <x:c r="A287" s="17"/>
@@ -5313,8 +5602,9 @@
       <x:c r="K287" s="14"/>
       <x:c r="L287" s="14"/>
       <x:c r="M287" s="14"/>
-      <x:c r="N287" s="14"/>
+      <x:c r="N287" s="17"/>
       <x:c r="O287" s="14"/>
+      <x:c r="P287" s="14"/>
     </x:row>
     <x:row r="288" ht="22" customHeight="1">
       <x:c r="A288" s="17"/>
@@ -5330,8 +5620,9 @@
       <x:c r="K288" s="14"/>
       <x:c r="L288" s="14"/>
       <x:c r="M288" s="14"/>
-      <x:c r="N288" s="14"/>
+      <x:c r="N288" s="17"/>
       <x:c r="O288" s="14"/>
+      <x:c r="P288" s="14"/>
     </x:row>
     <x:row r="289" ht="22" customHeight="1">
       <x:c r="A289" s="17"/>
@@ -5347,8 +5638,9 @@
       <x:c r="K289" s="14"/>
       <x:c r="L289" s="14"/>
       <x:c r="M289" s="14"/>
-      <x:c r="N289" s="14"/>
+      <x:c r="N289" s="17"/>
       <x:c r="O289" s="14"/>
+      <x:c r="P289" s="14"/>
     </x:row>
     <x:row r="290" ht="22" customHeight="1">
       <x:c r="A290" s="17"/>
@@ -5364,8 +5656,9 @@
       <x:c r="K290" s="14"/>
       <x:c r="L290" s="14"/>
       <x:c r="M290" s="14"/>
-      <x:c r="N290" s="14"/>
+      <x:c r="N290" s="17"/>
       <x:c r="O290" s="14"/>
+      <x:c r="P290" s="14"/>
     </x:row>
     <x:row r="291" ht="22" customHeight="1">
       <x:c r="A291" s="17"/>
@@ -5381,8 +5674,9 @@
       <x:c r="K291" s="14"/>
       <x:c r="L291" s="14"/>
       <x:c r="M291" s="14"/>
-      <x:c r="N291" s="14"/>
+      <x:c r="N291" s="17"/>
       <x:c r="O291" s="14"/>
+      <x:c r="P291" s="14"/>
     </x:row>
     <x:row r="292" ht="22" customHeight="1">
       <x:c r="A292" s="17"/>
@@ -5398,8 +5692,9 @@
       <x:c r="K292" s="14"/>
       <x:c r="L292" s="14"/>
       <x:c r="M292" s="14"/>
-      <x:c r="N292" s="14"/>
+      <x:c r="N292" s="17"/>
       <x:c r="O292" s="14"/>
+      <x:c r="P292" s="14"/>
     </x:row>
     <x:row r="293" ht="22" customHeight="1">
       <x:c r="A293" s="17"/>
@@ -5415,8 +5710,9 @@
       <x:c r="K293" s="14"/>
       <x:c r="L293" s="14"/>
       <x:c r="M293" s="14"/>
-      <x:c r="N293" s="14"/>
+      <x:c r="N293" s="17"/>
       <x:c r="O293" s="14"/>
+      <x:c r="P293" s="14"/>
     </x:row>
     <x:row r="294" ht="22" customHeight="1">
       <x:c r="A294" s="17"/>
@@ -5432,8 +5728,9 @@
       <x:c r="K294" s="14"/>
       <x:c r="L294" s="14"/>
       <x:c r="M294" s="14"/>
-      <x:c r="N294" s="14"/>
+      <x:c r="N294" s="17"/>
       <x:c r="O294" s="14"/>
+      <x:c r="P294" s="14"/>
     </x:row>
     <x:row r="295" ht="22" customHeight="1">
       <x:c r="A295" s="17"/>
@@ -5449,8 +5746,9 @@
       <x:c r="K295" s="14"/>
       <x:c r="L295" s="14"/>
       <x:c r="M295" s="14"/>
-      <x:c r="N295" s="14"/>
+      <x:c r="N295" s="17"/>
       <x:c r="O295" s="14"/>
+      <x:c r="P295" s="14"/>
     </x:row>
     <x:row r="296" ht="22" customHeight="1">
       <x:c r="A296" s="17"/>
@@ -5466,8 +5764,9 @@
       <x:c r="K296" s="14"/>
       <x:c r="L296" s="14"/>
       <x:c r="M296" s="14"/>
-      <x:c r="N296" s="14"/>
+      <x:c r="N296" s="17"/>
       <x:c r="O296" s="14"/>
+      <x:c r="P296" s="14"/>
     </x:row>
     <x:row r="297" ht="22" customHeight="1">
       <x:c r="A297" s="17"/>
@@ -5483,8 +5782,9 @@
       <x:c r="K297" s="14"/>
       <x:c r="L297" s="14"/>
       <x:c r="M297" s="14"/>
-      <x:c r="N297" s="14"/>
+      <x:c r="N297" s="17"/>
       <x:c r="O297" s="14"/>
+      <x:c r="P297" s="14"/>
     </x:row>
     <x:row r="298" ht="22" customHeight="1">
       <x:c r="A298" s="17"/>
@@ -5500,8 +5800,9 @@
       <x:c r="K298" s="14"/>
       <x:c r="L298" s="14"/>
       <x:c r="M298" s="14"/>
-      <x:c r="N298" s="14"/>
+      <x:c r="N298" s="17"/>
       <x:c r="O298" s="14"/>
+      <x:c r="P298" s="14"/>
     </x:row>
     <x:row r="299" ht="22" customHeight="1">
       <x:c r="A299" s="17"/>
@@ -5517,8 +5818,9 @@
       <x:c r="K299" s="14"/>
       <x:c r="L299" s="14"/>
       <x:c r="M299" s="14"/>
-      <x:c r="N299" s="14"/>
+      <x:c r="N299" s="17"/>
       <x:c r="O299" s="14"/>
+      <x:c r="P299" s="14"/>
     </x:row>
     <x:row r="300" ht="22" customHeight="1">
       <x:c r="A300" s="17"/>
@@ -5534,8 +5836,9 @@
       <x:c r="K300" s="14"/>
       <x:c r="L300" s="14"/>
       <x:c r="M300" s="14"/>
-      <x:c r="N300" s="14"/>
+      <x:c r="N300" s="17"/>
       <x:c r="O300" s="14"/>
+      <x:c r="P300" s="14"/>
     </x:row>
     <x:row r="301" ht="22" customHeight="1">
       <x:c r="A301" s="18"/>
@@ -5551,15 +5854,19 @@
       <x:c r="K301" s="15"/>
       <x:c r="L301" s="15"/>
       <x:c r="M301" s="15"/>
-      <x:c r="N301" s="15"/>
+      <x:c r="N301" s="18"/>
       <x:c r="O301" s="15"/>
+      <x:c r="P301" s="15"/>
     </x:row>
   </x:sheetData>
-  <x:dataValidations count="2">
+  <x:dataValidations count="3">
     <x:dataValidation type="list" sqref="A2:A301">
       <x:formula1>"DNI,CE"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="O2:O301">
+    <x:dataValidation type="list" sqref="M2:M301">
+      <x:formula1>"SIN REI,01,02,03,04,05,06,07,08,09,10,11,12,13,14,15,16,17,18,19"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="P2:P301">
       <x:formula1>"SI,NO"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -5639,7 +5946,7 @@
         <x:v>Cómo completar la plantilla</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="31" customHeight="1">
+    <x:row r="5" ht="34" customHeight="1">
       <x:c r="A5" s="28" t="str">
         <x:v>1</x:v>
       </x:c>
@@ -5651,7 +5958,7 @@
       <x:c r="E5" s="31"/>
       <x:c r="F5" s="31"/>
     </x:row>
-    <x:row r="6" ht="31" customHeight="1">
+    <x:row r="6" ht="34" customHeight="1">
       <x:c r="A6" s="28" t="str">
         <x:v>2</x:v>
       </x:c>
@@ -5663,7 +5970,7 @@
       <x:c r="E6" s="31"/>
       <x:c r="F6" s="31"/>
     </x:row>
-    <x:row r="7" ht="31" customHeight="1">
+    <x:row r="7" ht="34" customHeight="1">
       <x:c r="A7" s="28" t="str">
         <x:v>3</x:v>
       </x:c>
@@ -5675,7 +5982,7 @@
       <x:c r="E7" s="31"/>
       <x:c r="F7" s="31"/>
     </x:row>
-    <x:row r="8" ht="31" customHeight="1">
+    <x:row r="8" ht="34" customHeight="1">
       <x:c r="A8" s="28" t="str">
         <x:v>4</x:v>
       </x:c>
@@ -5687,7 +5994,7 @@
       <x:c r="E8" s="31"/>
       <x:c r="F8" s="31"/>
     </x:row>
-    <x:row r="9" ht="31" customHeight="1">
+    <x:row r="9" ht="34" customHeight="1">
       <x:c r="A9" s="28" t="str">
         <x:v>5</x:v>
       </x:c>
@@ -5699,7 +6006,7 @@
       <x:c r="E9" s="31"/>
       <x:c r="F9" s="31"/>
     </x:row>
-    <x:row r="10" ht="31" customHeight="1">
+    <x:row r="10" ht="34" customHeight="1">
       <x:c r="A10" s="28" t="str">
         <x:v>6</x:v>
       </x:c>
@@ -5711,69 +6018,81 @@
       <x:c r="E10" s="31"/>
       <x:c r="F10" s="31"/>
     </x:row>
-    <x:row r="11" ht="31" customHeight="1">
+    <x:row r="11" ht="34" customHeight="1">
       <x:c r="A11" s="28" t="str">
         <x:v>7</x:v>
       </x:c>
       <x:c r="B11" s="31" t="str">
-        <x:v>can_create_monitoreo: escribe SI o NO.</x:v>
+        <x:v>Código institucional: exactamente 8 dígitos, por ejemplo 25642929. Es obligatorio solo para director_iiee y se conserva como texto si inicia con 0.</x:v>
       </x:c>
       <x:c r="C11" s="31"/>
       <x:c r="D11" s="31"/>
       <x:c r="E11" s="31"/>
       <x:c r="F11" s="31"/>
     </x:row>
-    <x:row r="12" ht="31" customHeight="1">
+    <x:row r="12" ht="34" customHeight="1">
       <x:c r="A12" s="28" t="str">
         <x:v>8</x:v>
       </x:c>
       <x:c r="B12" s="31" t="str">
-        <x:v>No agregues una columna de contraseña. El sistema la genera desde el apellido paterno (QUISPE → Quispe123@@) y exige cambiarla en el primer ingreso.</x:v>
+        <x:v>REI: usa 01, 02, 03... hasta 19, o SIN REI. can_create_monitoreo: escribe SI o NO.</x:v>
       </x:c>
       <x:c r="C12" s="31"/>
       <x:c r="D12" s="31"/>
       <x:c r="E12" s="31"/>
       <x:c r="F12" s="31"/>
     </x:row>
-    <x:row r="14">
-      <x:c r="A14" s="25" t="str">
+    <x:row r="13" ht="34" customHeight="1">
+      <x:c r="A13" s="28" t="str">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B13" s="31" t="str">
+        <x:v>No agregues una columna de contraseña. El sistema la genera desde el apellido paterno (QUISPE → Quispe123@@) y exige cambiarla en el primer ingreso.</x:v>
+      </x:c>
+      <x:c r="C13" s="31"/>
+      <x:c r="D13" s="31"/>
+      <x:c r="E13" s="31"/>
+      <x:c r="F13" s="31"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="25" t="str">
         <x:v>Campos obligatorios</x:v>
       </x:c>
-      <x:c r="B14" s="25" t="str">
+      <x:c r="B15" s="25" t="str">
         <x:v>Campos obligatorios</x:v>
       </x:c>
-      <x:c r="C14" s="25" t="str">
+      <x:c r="C15" s="25" t="str">
         <x:v>Campos obligatorios</x:v>
       </x:c>
-      <x:c r="D14" s="25" t="str">
+      <x:c r="D15" s="25" t="str">
         <x:v>Campos obligatorios</x:v>
       </x:c>
-      <x:c r="E14" s="25" t="str">
+      <x:c r="E15" s="25" t="str">
         <x:v>Campos obligatorios</x:v>
       </x:c>
-      <x:c r="F14" s="25" t="str">
+      <x:c r="F15" s="25" t="str">
         <x:v>Campos obligatorios</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" ht="28" customHeight="1">
-      <x:c r="A15" s="30" t="str">
+    <x:row r="16" ht="32" customHeight="1">
+      <x:c r="A16" s="30" t="str">
         <x:v>tipo_documento, numero_documento, apellido_paterno, apellido_materno, nombres, correo y rol</x:v>
-      </x:c>
-      <x:c r="B15" s="30"/>
-      <x:c r="C15" s="30"/>
-      <x:c r="D15" s="30"/>
-      <x:c r="E15" s="30"/>
-      <x:c r="F15" s="30"/>
-    </x:row>
-    <x:row r="16" ht="28" customHeight="1">
-      <x:c r="A16" s="30" t="str">
-        <x:v>Los demás campos son opcionales. UGEL se completa como UGEL 06 y REI como SIN REI cuando se dejan vacíos.</x:v>
       </x:c>
       <x:c r="B16" s="30"/>
       <x:c r="C16" s="30"/>
       <x:c r="D16" s="30"/>
       <x:c r="E16" s="30"/>
       <x:c r="F16" s="30"/>
+    </x:row>
+    <x:row r="17" ht="32" customHeight="1">
+      <x:c r="A17" s="30" t="str">
+        <x:v>codigo_institucional es obligatorio únicamente para director_iiee. Los demás campos son opcionales; UGEL se completa como UGEL 06 y REI como SIN REI.</x:v>
+      </x:c>
+      <x:c r="B17" s="30"/>
+      <x:c r="C17" s="30"/>
+      <x:c r="D17" s="30"/>
+      <x:c r="E17" s="30"/>
+      <x:c r="F17" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -5787,9 +6106,10 @@
     <x:mergeCell ref="B10:F10"/>
     <x:mergeCell ref="B11:F11"/>
     <x:mergeCell ref="B12:F12"/>
-    <x:mergeCell ref="A14:F14"/>
+    <x:mergeCell ref="B13:F13"/>
     <x:mergeCell ref="A15:F15"/>
     <x:mergeCell ref="A16:F16"/>
+    <x:mergeCell ref="A17:F17"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
implementación de plazas y correcion de plantillas de carga de usuarios
</commit_message>
<xml_diff>
--- a/public/plantilla_carga_usuarios.xlsx
+++ b/public/plantilla_carga_usuarios.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Usuarios" sheetId="1" r:id="R61990382be5440a5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="2" r:id="R419950f374be4233"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Usuarios" sheetId="1" r:id="R68657ac4009f45d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="2" r:id="Rd4f8a2a682c94648"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -404,8 +404,10 @@
     <x:col min="12" max="12" width="16" hidden="0" customWidth="1"/>
     <x:col min="13" max="13" width="15" hidden="0" customWidth="1"/>
     <x:col min="14" max="14" width="24" hidden="0" customWidth="1"/>
-    <x:col min="15" max="15" width="22" hidden="0" customWidth="1"/>
-    <x:col min="16" max="16" width="23" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="34" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="16" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="22" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="23" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
@@ -452,9 +454,15 @@
         <x:v>codigo_institucional</x:v>
       </x:c>
       <x:c r="O1" s="10" t="str">
+        <x:v>nombre_colegio_referencia</x:v>
+      </x:c>
+      <x:c r="P1" s="10" t="str">
+        <x:v>modalidad</x:v>
+      </x:c>
+      <x:c r="Q1" s="10" t="str">
         <x:v>rol</x:v>
       </x:c>
-      <x:c r="P1" s="11" t="str">
+      <x:c r="R1" s="11" t="str">
         <x:v>can_create_monitoreo</x:v>
       </x:c>
     </x:row>
@@ -473,8 +481,10 @@
       <x:c r="L2" s="13"/>
       <x:c r="M2" s="13"/>
       <x:c r="N2" s="16"/>
-      <x:c r="O2" s="13"/>
-      <x:c r="P2" s="13"/>
+      <x:c r="O2" s="16"/>
+      <x:c r="P2" s="16"/>
+      <x:c r="Q2" s="13"/>
+      <x:c r="R2" s="13"/>
     </x:row>
     <x:row r="3" ht="22" customHeight="1">
       <x:c r="A3" s="17"/>
@@ -491,8 +501,10 @@
       <x:c r="L3" s="14"/>
       <x:c r="M3" s="14"/>
       <x:c r="N3" s="17"/>
-      <x:c r="O3" s="14"/>
-      <x:c r="P3" s="14"/>
+      <x:c r="O3" s="17"/>
+      <x:c r="P3" s="17"/>
+      <x:c r="Q3" s="14"/>
+      <x:c r="R3" s="14"/>
     </x:row>
     <x:row r="4" ht="22" customHeight="1">
       <x:c r="A4" s="17"/>
@@ -509,8 +521,10 @@
       <x:c r="L4" s="14"/>
       <x:c r="M4" s="14"/>
       <x:c r="N4" s="17"/>
-      <x:c r="O4" s="14"/>
-      <x:c r="P4" s="14"/>
+      <x:c r="O4" s="17"/>
+      <x:c r="P4" s="17"/>
+      <x:c r="Q4" s="14"/>
+      <x:c r="R4" s="14"/>
     </x:row>
     <x:row r="5" ht="22" customHeight="1">
       <x:c r="A5" s="17"/>
@@ -527,8 +541,10 @@
       <x:c r="L5" s="14"/>
       <x:c r="M5" s="14"/>
       <x:c r="N5" s="17"/>
-      <x:c r="O5" s="14"/>
-      <x:c r="P5" s="14"/>
+      <x:c r="O5" s="17"/>
+      <x:c r="P5" s="17"/>
+      <x:c r="Q5" s="14"/>
+      <x:c r="R5" s="14"/>
     </x:row>
     <x:row r="6" ht="22" customHeight="1">
       <x:c r="A6" s="17"/>
@@ -545,8 +561,10 @@
       <x:c r="L6" s="14"/>
       <x:c r="M6" s="14"/>
       <x:c r="N6" s="17"/>
-      <x:c r="O6" s="14"/>
-      <x:c r="P6" s="14"/>
+      <x:c r="O6" s="17"/>
+      <x:c r="P6" s="17"/>
+      <x:c r="Q6" s="14"/>
+      <x:c r="R6" s="14"/>
     </x:row>
     <x:row r="7" ht="22" customHeight="1">
       <x:c r="A7" s="17"/>
@@ -563,8 +581,10 @@
       <x:c r="L7" s="14"/>
       <x:c r="M7" s="14"/>
       <x:c r="N7" s="17"/>
-      <x:c r="O7" s="14"/>
-      <x:c r="P7" s="14"/>
+      <x:c r="O7" s="17"/>
+      <x:c r="P7" s="17"/>
+      <x:c r="Q7" s="14"/>
+      <x:c r="R7" s="14"/>
     </x:row>
     <x:row r="8" ht="22" customHeight="1">
       <x:c r="A8" s="17"/>
@@ -581,8 +601,10 @@
       <x:c r="L8" s="14"/>
       <x:c r="M8" s="14"/>
       <x:c r="N8" s="17"/>
-      <x:c r="O8" s="14"/>
-      <x:c r="P8" s="14"/>
+      <x:c r="O8" s="17"/>
+      <x:c r="P8" s="17"/>
+      <x:c r="Q8" s="14"/>
+      <x:c r="R8" s="14"/>
     </x:row>
     <x:row r="9" ht="22" customHeight="1">
       <x:c r="A9" s="17"/>
@@ -599,8 +621,10 @@
       <x:c r="L9" s="14"/>
       <x:c r="M9" s="14"/>
       <x:c r="N9" s="17"/>
-      <x:c r="O9" s="14"/>
-      <x:c r="P9" s="14"/>
+      <x:c r="O9" s="17"/>
+      <x:c r="P9" s="17"/>
+      <x:c r="Q9" s="14"/>
+      <x:c r="R9" s="14"/>
     </x:row>
     <x:row r="10" ht="22" customHeight="1">
       <x:c r="A10" s="17"/>
@@ -617,8 +641,10 @@
       <x:c r="L10" s="14"/>
       <x:c r="M10" s="14"/>
       <x:c r="N10" s="17"/>
-      <x:c r="O10" s="14"/>
-      <x:c r="P10" s="14"/>
+      <x:c r="O10" s="17"/>
+      <x:c r="P10" s="17"/>
+      <x:c r="Q10" s="14"/>
+      <x:c r="R10" s="14"/>
     </x:row>
     <x:row r="11" ht="22" customHeight="1">
       <x:c r="A11" s="17"/>
@@ -635,8 +661,10 @@
       <x:c r="L11" s="14"/>
       <x:c r="M11" s="14"/>
       <x:c r="N11" s="17"/>
-      <x:c r="O11" s="14"/>
-      <x:c r="P11" s="14"/>
+      <x:c r="O11" s="17"/>
+      <x:c r="P11" s="17"/>
+      <x:c r="Q11" s="14"/>
+      <x:c r="R11" s="14"/>
     </x:row>
     <x:row r="12" ht="22" customHeight="1">
       <x:c r="A12" s="17"/>
@@ -653,8 +681,10 @@
       <x:c r="L12" s="14"/>
       <x:c r="M12" s="14"/>
       <x:c r="N12" s="17"/>
-      <x:c r="O12" s="14"/>
-      <x:c r="P12" s="14"/>
+      <x:c r="O12" s="17"/>
+      <x:c r="P12" s="17"/>
+      <x:c r="Q12" s="14"/>
+      <x:c r="R12" s="14"/>
     </x:row>
     <x:row r="13" ht="22" customHeight="1">
       <x:c r="A13" s="17"/>
@@ -671,8 +701,10 @@
       <x:c r="L13" s="14"/>
       <x:c r="M13" s="14"/>
       <x:c r="N13" s="17"/>
-      <x:c r="O13" s="14"/>
-      <x:c r="P13" s="14"/>
+      <x:c r="O13" s="17"/>
+      <x:c r="P13" s="17"/>
+      <x:c r="Q13" s="14"/>
+      <x:c r="R13" s="14"/>
     </x:row>
     <x:row r="14" ht="22" customHeight="1">
       <x:c r="A14" s="17"/>
@@ -689,8 +721,10 @@
       <x:c r="L14" s="14"/>
       <x:c r="M14" s="14"/>
       <x:c r="N14" s="17"/>
-      <x:c r="O14" s="14"/>
-      <x:c r="P14" s="14"/>
+      <x:c r="O14" s="17"/>
+      <x:c r="P14" s="17"/>
+      <x:c r="Q14" s="14"/>
+      <x:c r="R14" s="14"/>
     </x:row>
     <x:row r="15" ht="22" customHeight="1">
       <x:c r="A15" s="17"/>
@@ -707,8 +741,10 @@
       <x:c r="L15" s="14"/>
       <x:c r="M15" s="14"/>
       <x:c r="N15" s="17"/>
-      <x:c r="O15" s="14"/>
-      <x:c r="P15" s="14"/>
+      <x:c r="O15" s="17"/>
+      <x:c r="P15" s="17"/>
+      <x:c r="Q15" s="14"/>
+      <x:c r="R15" s="14"/>
     </x:row>
     <x:row r="16" ht="22" customHeight="1">
       <x:c r="A16" s="17"/>
@@ -725,8 +761,10 @@
       <x:c r="L16" s="14"/>
       <x:c r="M16" s="14"/>
       <x:c r="N16" s="17"/>
-      <x:c r="O16" s="14"/>
-      <x:c r="P16" s="14"/>
+      <x:c r="O16" s="17"/>
+      <x:c r="P16" s="17"/>
+      <x:c r="Q16" s="14"/>
+      <x:c r="R16" s="14"/>
     </x:row>
     <x:row r="17" ht="22" customHeight="1">
       <x:c r="A17" s="17"/>
@@ -743,8 +781,10 @@
       <x:c r="L17" s="14"/>
       <x:c r="M17" s="14"/>
       <x:c r="N17" s="17"/>
-      <x:c r="O17" s="14"/>
-      <x:c r="P17" s="14"/>
+      <x:c r="O17" s="17"/>
+      <x:c r="P17" s="17"/>
+      <x:c r="Q17" s="14"/>
+      <x:c r="R17" s="14"/>
     </x:row>
     <x:row r="18" ht="22" customHeight="1">
       <x:c r="A18" s="17"/>
@@ -761,8 +801,10 @@
       <x:c r="L18" s="14"/>
       <x:c r="M18" s="14"/>
       <x:c r="N18" s="17"/>
-      <x:c r="O18" s="14"/>
-      <x:c r="P18" s="14"/>
+      <x:c r="O18" s="17"/>
+      <x:c r="P18" s="17"/>
+      <x:c r="Q18" s="14"/>
+      <x:c r="R18" s="14"/>
     </x:row>
     <x:row r="19" ht="22" customHeight="1">
       <x:c r="A19" s="17"/>
@@ -779,8 +821,10 @@
       <x:c r="L19" s="14"/>
       <x:c r="M19" s="14"/>
       <x:c r="N19" s="17"/>
-      <x:c r="O19" s="14"/>
-      <x:c r="P19" s="14"/>
+      <x:c r="O19" s="17"/>
+      <x:c r="P19" s="17"/>
+      <x:c r="Q19" s="14"/>
+      <x:c r="R19" s="14"/>
     </x:row>
     <x:row r="20" ht="22" customHeight="1">
       <x:c r="A20" s="17"/>
@@ -797,8 +841,10 @@
       <x:c r="L20" s="14"/>
       <x:c r="M20" s="14"/>
       <x:c r="N20" s="17"/>
-      <x:c r="O20" s="14"/>
-      <x:c r="P20" s="14"/>
+      <x:c r="O20" s="17"/>
+      <x:c r="P20" s="17"/>
+      <x:c r="Q20" s="14"/>
+      <x:c r="R20" s="14"/>
     </x:row>
     <x:row r="21" ht="22" customHeight="1">
       <x:c r="A21" s="17"/>
@@ -815,8 +861,10 @@
       <x:c r="L21" s="14"/>
       <x:c r="M21" s="14"/>
       <x:c r="N21" s="17"/>
-      <x:c r="O21" s="14"/>
-      <x:c r="P21" s="14"/>
+      <x:c r="O21" s="17"/>
+      <x:c r="P21" s="17"/>
+      <x:c r="Q21" s="14"/>
+      <x:c r="R21" s="14"/>
     </x:row>
     <x:row r="22" ht="22" customHeight="1">
       <x:c r="A22" s="17"/>
@@ -833,8 +881,10 @@
       <x:c r="L22" s="14"/>
       <x:c r="M22" s="14"/>
       <x:c r="N22" s="17"/>
-      <x:c r="O22" s="14"/>
-      <x:c r="P22" s="14"/>
+      <x:c r="O22" s="17"/>
+      <x:c r="P22" s="17"/>
+      <x:c r="Q22" s="14"/>
+      <x:c r="R22" s="14"/>
     </x:row>
     <x:row r="23" ht="22" customHeight="1">
       <x:c r="A23" s="17"/>
@@ -851,8 +901,10 @@
       <x:c r="L23" s="14"/>
       <x:c r="M23" s="14"/>
       <x:c r="N23" s="17"/>
-      <x:c r="O23" s="14"/>
-      <x:c r="P23" s="14"/>
+      <x:c r="O23" s="17"/>
+      <x:c r="P23" s="17"/>
+      <x:c r="Q23" s="14"/>
+      <x:c r="R23" s="14"/>
     </x:row>
     <x:row r="24" ht="22" customHeight="1">
       <x:c r="A24" s="17"/>
@@ -869,8 +921,10 @@
       <x:c r="L24" s="14"/>
       <x:c r="M24" s="14"/>
       <x:c r="N24" s="17"/>
-      <x:c r="O24" s="14"/>
-      <x:c r="P24" s="14"/>
+      <x:c r="O24" s="17"/>
+      <x:c r="P24" s="17"/>
+      <x:c r="Q24" s="14"/>
+      <x:c r="R24" s="14"/>
     </x:row>
     <x:row r="25" ht="22" customHeight="1">
       <x:c r="A25" s="17"/>
@@ -887,8 +941,10 @@
       <x:c r="L25" s="14"/>
       <x:c r="M25" s="14"/>
       <x:c r="N25" s="17"/>
-      <x:c r="O25" s="14"/>
-      <x:c r="P25" s="14"/>
+      <x:c r="O25" s="17"/>
+      <x:c r="P25" s="17"/>
+      <x:c r="Q25" s="14"/>
+      <x:c r="R25" s="14"/>
     </x:row>
     <x:row r="26" ht="22" customHeight="1">
       <x:c r="A26" s="17"/>
@@ -905,8 +961,10 @@
       <x:c r="L26" s="14"/>
       <x:c r="M26" s="14"/>
       <x:c r="N26" s="17"/>
-      <x:c r="O26" s="14"/>
-      <x:c r="P26" s="14"/>
+      <x:c r="O26" s="17"/>
+      <x:c r="P26" s="17"/>
+      <x:c r="Q26" s="14"/>
+      <x:c r="R26" s="14"/>
     </x:row>
     <x:row r="27" ht="22" customHeight="1">
       <x:c r="A27" s="17"/>
@@ -923,8 +981,10 @@
       <x:c r="L27" s="14"/>
       <x:c r="M27" s="14"/>
       <x:c r="N27" s="17"/>
-      <x:c r="O27" s="14"/>
-      <x:c r="P27" s="14"/>
+      <x:c r="O27" s="17"/>
+      <x:c r="P27" s="17"/>
+      <x:c r="Q27" s="14"/>
+      <x:c r="R27" s="14"/>
     </x:row>
     <x:row r="28" ht="22" customHeight="1">
       <x:c r="A28" s="17"/>
@@ -941,8 +1001,10 @@
       <x:c r="L28" s="14"/>
       <x:c r="M28" s="14"/>
       <x:c r="N28" s="17"/>
-      <x:c r="O28" s="14"/>
-      <x:c r="P28" s="14"/>
+      <x:c r="O28" s="17"/>
+      <x:c r="P28" s="17"/>
+      <x:c r="Q28" s="14"/>
+      <x:c r="R28" s="14"/>
     </x:row>
     <x:row r="29" ht="22" customHeight="1">
       <x:c r="A29" s="17"/>
@@ -959,8 +1021,10 @@
       <x:c r="L29" s="14"/>
       <x:c r="M29" s="14"/>
       <x:c r="N29" s="17"/>
-      <x:c r="O29" s="14"/>
-      <x:c r="P29" s="14"/>
+      <x:c r="O29" s="17"/>
+      <x:c r="P29" s="17"/>
+      <x:c r="Q29" s="14"/>
+      <x:c r="R29" s="14"/>
     </x:row>
     <x:row r="30" ht="22" customHeight="1">
       <x:c r="A30" s="17"/>
@@ -977,8 +1041,10 @@
       <x:c r="L30" s="14"/>
       <x:c r="M30" s="14"/>
       <x:c r="N30" s="17"/>
-      <x:c r="O30" s="14"/>
-      <x:c r="P30" s="14"/>
+      <x:c r="O30" s="17"/>
+      <x:c r="P30" s="17"/>
+      <x:c r="Q30" s="14"/>
+      <x:c r="R30" s="14"/>
     </x:row>
     <x:row r="31" ht="22" customHeight="1">
       <x:c r="A31" s="17"/>
@@ -995,8 +1061,10 @@
       <x:c r="L31" s="14"/>
       <x:c r="M31" s="14"/>
       <x:c r="N31" s="17"/>
-      <x:c r="O31" s="14"/>
-      <x:c r="P31" s="14"/>
+      <x:c r="O31" s="17"/>
+      <x:c r="P31" s="17"/>
+      <x:c r="Q31" s="14"/>
+      <x:c r="R31" s="14"/>
     </x:row>
     <x:row r="32" ht="22" customHeight="1">
       <x:c r="A32" s="17"/>
@@ -1013,8 +1081,10 @@
       <x:c r="L32" s="14"/>
       <x:c r="M32" s="14"/>
       <x:c r="N32" s="17"/>
-      <x:c r="O32" s="14"/>
-      <x:c r="P32" s="14"/>
+      <x:c r="O32" s="17"/>
+      <x:c r="P32" s="17"/>
+      <x:c r="Q32" s="14"/>
+      <x:c r="R32" s="14"/>
     </x:row>
     <x:row r="33" ht="22" customHeight="1">
       <x:c r="A33" s="17"/>
@@ -1031,8 +1101,10 @@
       <x:c r="L33" s="14"/>
       <x:c r="M33" s="14"/>
       <x:c r="N33" s="17"/>
-      <x:c r="O33" s="14"/>
-      <x:c r="P33" s="14"/>
+      <x:c r="O33" s="17"/>
+      <x:c r="P33" s="17"/>
+      <x:c r="Q33" s="14"/>
+      <x:c r="R33" s="14"/>
     </x:row>
     <x:row r="34" ht="22" customHeight="1">
       <x:c r="A34" s="17"/>
@@ -1049,8 +1121,10 @@
       <x:c r="L34" s="14"/>
       <x:c r="M34" s="14"/>
       <x:c r="N34" s="17"/>
-      <x:c r="O34" s="14"/>
-      <x:c r="P34" s="14"/>
+      <x:c r="O34" s="17"/>
+      <x:c r="P34" s="17"/>
+      <x:c r="Q34" s="14"/>
+      <x:c r="R34" s="14"/>
     </x:row>
     <x:row r="35" ht="22" customHeight="1">
       <x:c r="A35" s="17"/>
@@ -1067,8 +1141,10 @@
       <x:c r="L35" s="14"/>
       <x:c r="M35" s="14"/>
       <x:c r="N35" s="17"/>
-      <x:c r="O35" s="14"/>
-      <x:c r="P35" s="14"/>
+      <x:c r="O35" s="17"/>
+      <x:c r="P35" s="17"/>
+      <x:c r="Q35" s="14"/>
+      <x:c r="R35" s="14"/>
     </x:row>
     <x:row r="36" ht="22" customHeight="1">
       <x:c r="A36" s="17"/>
@@ -1085,8 +1161,10 @@
       <x:c r="L36" s="14"/>
       <x:c r="M36" s="14"/>
       <x:c r="N36" s="17"/>
-      <x:c r="O36" s="14"/>
-      <x:c r="P36" s="14"/>
+      <x:c r="O36" s="17"/>
+      <x:c r="P36" s="17"/>
+      <x:c r="Q36" s="14"/>
+      <x:c r="R36" s="14"/>
     </x:row>
     <x:row r="37" ht="22" customHeight="1">
       <x:c r="A37" s="17"/>
@@ -1103,8 +1181,10 @@
       <x:c r="L37" s="14"/>
       <x:c r="M37" s="14"/>
       <x:c r="N37" s="17"/>
-      <x:c r="O37" s="14"/>
-      <x:c r="P37" s="14"/>
+      <x:c r="O37" s="17"/>
+      <x:c r="P37" s="17"/>
+      <x:c r="Q37" s="14"/>
+      <x:c r="R37" s="14"/>
     </x:row>
     <x:row r="38" ht="22" customHeight="1">
       <x:c r="A38" s="17"/>
@@ -1121,8 +1201,10 @@
       <x:c r="L38" s="14"/>
       <x:c r="M38" s="14"/>
       <x:c r="N38" s="17"/>
-      <x:c r="O38" s="14"/>
-      <x:c r="P38" s="14"/>
+      <x:c r="O38" s="17"/>
+      <x:c r="P38" s="17"/>
+      <x:c r="Q38" s="14"/>
+      <x:c r="R38" s="14"/>
     </x:row>
     <x:row r="39" ht="22" customHeight="1">
       <x:c r="A39" s="17"/>
@@ -1139,8 +1221,10 @@
       <x:c r="L39" s="14"/>
       <x:c r="M39" s="14"/>
       <x:c r="N39" s="17"/>
-      <x:c r="O39" s="14"/>
-      <x:c r="P39" s="14"/>
+      <x:c r="O39" s="17"/>
+      <x:c r="P39" s="17"/>
+      <x:c r="Q39" s="14"/>
+      <x:c r="R39" s="14"/>
     </x:row>
     <x:row r="40" ht="22" customHeight="1">
       <x:c r="A40" s="17"/>
@@ -1157,8 +1241,10 @@
       <x:c r="L40" s="14"/>
       <x:c r="M40" s="14"/>
       <x:c r="N40" s="17"/>
-      <x:c r="O40" s="14"/>
-      <x:c r="P40" s="14"/>
+      <x:c r="O40" s="17"/>
+      <x:c r="P40" s="17"/>
+      <x:c r="Q40" s="14"/>
+      <x:c r="R40" s="14"/>
     </x:row>
     <x:row r="41" ht="22" customHeight="1">
       <x:c r="A41" s="17"/>
@@ -1175,8 +1261,10 @@
       <x:c r="L41" s="14"/>
       <x:c r="M41" s="14"/>
       <x:c r="N41" s="17"/>
-      <x:c r="O41" s="14"/>
-      <x:c r="P41" s="14"/>
+      <x:c r="O41" s="17"/>
+      <x:c r="P41" s="17"/>
+      <x:c r="Q41" s="14"/>
+      <x:c r="R41" s="14"/>
     </x:row>
     <x:row r="42" ht="22" customHeight="1">
       <x:c r="A42" s="17"/>
@@ -1193,8 +1281,10 @@
       <x:c r="L42" s="14"/>
       <x:c r="M42" s="14"/>
       <x:c r="N42" s="17"/>
-      <x:c r="O42" s="14"/>
-      <x:c r="P42" s="14"/>
+      <x:c r="O42" s="17"/>
+      <x:c r="P42" s="17"/>
+      <x:c r="Q42" s="14"/>
+      <x:c r="R42" s="14"/>
     </x:row>
     <x:row r="43" ht="22" customHeight="1">
       <x:c r="A43" s="17"/>
@@ -1211,8 +1301,10 @@
       <x:c r="L43" s="14"/>
       <x:c r="M43" s="14"/>
       <x:c r="N43" s="17"/>
-      <x:c r="O43" s="14"/>
-      <x:c r="P43" s="14"/>
+      <x:c r="O43" s="17"/>
+      <x:c r="P43" s="17"/>
+      <x:c r="Q43" s="14"/>
+      <x:c r="R43" s="14"/>
     </x:row>
     <x:row r="44" ht="22" customHeight="1">
       <x:c r="A44" s="17"/>
@@ -1229,8 +1321,10 @@
       <x:c r="L44" s="14"/>
       <x:c r="M44" s="14"/>
       <x:c r="N44" s="17"/>
-      <x:c r="O44" s="14"/>
-      <x:c r="P44" s="14"/>
+      <x:c r="O44" s="17"/>
+      <x:c r="P44" s="17"/>
+      <x:c r="Q44" s="14"/>
+      <x:c r="R44" s="14"/>
     </x:row>
     <x:row r="45" ht="22" customHeight="1">
       <x:c r="A45" s="17"/>
@@ -1247,8 +1341,10 @@
       <x:c r="L45" s="14"/>
       <x:c r="M45" s="14"/>
       <x:c r="N45" s="17"/>
-      <x:c r="O45" s="14"/>
-      <x:c r="P45" s="14"/>
+      <x:c r="O45" s="17"/>
+      <x:c r="P45" s="17"/>
+      <x:c r="Q45" s="14"/>
+      <x:c r="R45" s="14"/>
     </x:row>
     <x:row r="46" ht="22" customHeight="1">
       <x:c r="A46" s="17"/>
@@ -1265,8 +1361,10 @@
       <x:c r="L46" s="14"/>
       <x:c r="M46" s="14"/>
       <x:c r="N46" s="17"/>
-      <x:c r="O46" s="14"/>
-      <x:c r="P46" s="14"/>
+      <x:c r="O46" s="17"/>
+      <x:c r="P46" s="17"/>
+      <x:c r="Q46" s="14"/>
+      <x:c r="R46" s="14"/>
     </x:row>
     <x:row r="47" ht="22" customHeight="1">
       <x:c r="A47" s="17"/>
@@ -1283,8 +1381,10 @@
       <x:c r="L47" s="14"/>
       <x:c r="M47" s="14"/>
       <x:c r="N47" s="17"/>
-      <x:c r="O47" s="14"/>
-      <x:c r="P47" s="14"/>
+      <x:c r="O47" s="17"/>
+      <x:c r="P47" s="17"/>
+      <x:c r="Q47" s="14"/>
+      <x:c r="R47" s="14"/>
     </x:row>
     <x:row r="48" ht="22" customHeight="1">
       <x:c r="A48" s="17"/>
@@ -1301,8 +1401,10 @@
       <x:c r="L48" s="14"/>
       <x:c r="M48" s="14"/>
       <x:c r="N48" s="17"/>
-      <x:c r="O48" s="14"/>
-      <x:c r="P48" s="14"/>
+      <x:c r="O48" s="17"/>
+      <x:c r="P48" s="17"/>
+      <x:c r="Q48" s="14"/>
+      <x:c r="R48" s="14"/>
     </x:row>
     <x:row r="49" ht="22" customHeight="1">
       <x:c r="A49" s="17"/>
@@ -1319,8 +1421,10 @@
       <x:c r="L49" s="14"/>
       <x:c r="M49" s="14"/>
       <x:c r="N49" s="17"/>
-      <x:c r="O49" s="14"/>
-      <x:c r="P49" s="14"/>
+      <x:c r="O49" s="17"/>
+      <x:c r="P49" s="17"/>
+      <x:c r="Q49" s="14"/>
+      <x:c r="R49" s="14"/>
     </x:row>
     <x:row r="50" ht="22" customHeight="1">
       <x:c r="A50" s="17"/>
@@ -1337,8 +1441,10 @@
       <x:c r="L50" s="14"/>
       <x:c r="M50" s="14"/>
       <x:c r="N50" s="17"/>
-      <x:c r="O50" s="14"/>
-      <x:c r="P50" s="14"/>
+      <x:c r="O50" s="17"/>
+      <x:c r="P50" s="17"/>
+      <x:c r="Q50" s="14"/>
+      <x:c r="R50" s="14"/>
     </x:row>
     <x:row r="51" ht="22" customHeight="1">
       <x:c r="A51" s="17"/>
@@ -1355,8 +1461,10 @@
       <x:c r="L51" s="14"/>
       <x:c r="M51" s="14"/>
       <x:c r="N51" s="17"/>
-      <x:c r="O51" s="14"/>
-      <x:c r="P51" s="14"/>
+      <x:c r="O51" s="17"/>
+      <x:c r="P51" s="17"/>
+      <x:c r="Q51" s="14"/>
+      <x:c r="R51" s="14"/>
     </x:row>
     <x:row r="52" ht="22" customHeight="1">
       <x:c r="A52" s="17"/>
@@ -1373,8 +1481,10 @@
       <x:c r="L52" s="14"/>
       <x:c r="M52" s="14"/>
       <x:c r="N52" s="17"/>
-      <x:c r="O52" s="14"/>
-      <x:c r="P52" s="14"/>
+      <x:c r="O52" s="17"/>
+      <x:c r="P52" s="17"/>
+      <x:c r="Q52" s="14"/>
+      <x:c r="R52" s="14"/>
     </x:row>
     <x:row r="53" ht="22" customHeight="1">
       <x:c r="A53" s="17"/>
@@ -1391,8 +1501,10 @@
       <x:c r="L53" s="14"/>
       <x:c r="M53" s="14"/>
       <x:c r="N53" s="17"/>
-      <x:c r="O53" s="14"/>
-      <x:c r="P53" s="14"/>
+      <x:c r="O53" s="17"/>
+      <x:c r="P53" s="17"/>
+      <x:c r="Q53" s="14"/>
+      <x:c r="R53" s="14"/>
     </x:row>
     <x:row r="54" ht="22" customHeight="1">
       <x:c r="A54" s="17"/>
@@ -1409,8 +1521,10 @@
       <x:c r="L54" s="14"/>
       <x:c r="M54" s="14"/>
       <x:c r="N54" s="17"/>
-      <x:c r="O54" s="14"/>
-      <x:c r="P54" s="14"/>
+      <x:c r="O54" s="17"/>
+      <x:c r="P54" s="17"/>
+      <x:c r="Q54" s="14"/>
+      <x:c r="R54" s="14"/>
     </x:row>
     <x:row r="55" ht="22" customHeight="1">
       <x:c r="A55" s="17"/>
@@ -1427,8 +1541,10 @@
       <x:c r="L55" s="14"/>
       <x:c r="M55" s="14"/>
       <x:c r="N55" s="17"/>
-      <x:c r="O55" s="14"/>
-      <x:c r="P55" s="14"/>
+      <x:c r="O55" s="17"/>
+      <x:c r="P55" s="17"/>
+      <x:c r="Q55" s="14"/>
+      <x:c r="R55" s="14"/>
     </x:row>
     <x:row r="56" ht="22" customHeight="1">
       <x:c r="A56" s="17"/>
@@ -1445,8 +1561,10 @@
       <x:c r="L56" s="14"/>
       <x:c r="M56" s="14"/>
       <x:c r="N56" s="17"/>
-      <x:c r="O56" s="14"/>
-      <x:c r="P56" s="14"/>
+      <x:c r="O56" s="17"/>
+      <x:c r="P56" s="17"/>
+      <x:c r="Q56" s="14"/>
+      <x:c r="R56" s="14"/>
     </x:row>
     <x:row r="57" ht="22" customHeight="1">
       <x:c r="A57" s="17"/>
@@ -1463,8 +1581,10 @@
       <x:c r="L57" s="14"/>
       <x:c r="M57" s="14"/>
       <x:c r="N57" s="17"/>
-      <x:c r="O57" s="14"/>
-      <x:c r="P57" s="14"/>
+      <x:c r="O57" s="17"/>
+      <x:c r="P57" s="17"/>
+      <x:c r="Q57" s="14"/>
+      <x:c r="R57" s="14"/>
     </x:row>
     <x:row r="58" ht="22" customHeight="1">
       <x:c r="A58" s="17"/>
@@ -1481,8 +1601,10 @@
       <x:c r="L58" s="14"/>
       <x:c r="M58" s="14"/>
       <x:c r="N58" s="17"/>
-      <x:c r="O58" s="14"/>
-      <x:c r="P58" s="14"/>
+      <x:c r="O58" s="17"/>
+      <x:c r="P58" s="17"/>
+      <x:c r="Q58" s="14"/>
+      <x:c r="R58" s="14"/>
     </x:row>
     <x:row r="59" ht="22" customHeight="1">
       <x:c r="A59" s="17"/>
@@ -1499,8 +1621,10 @@
       <x:c r="L59" s="14"/>
       <x:c r="M59" s="14"/>
       <x:c r="N59" s="17"/>
-      <x:c r="O59" s="14"/>
-      <x:c r="P59" s="14"/>
+      <x:c r="O59" s="17"/>
+      <x:c r="P59" s="17"/>
+      <x:c r="Q59" s="14"/>
+      <x:c r="R59" s="14"/>
     </x:row>
     <x:row r="60" ht="22" customHeight="1">
       <x:c r="A60" s="17"/>
@@ -1517,8 +1641,10 @@
       <x:c r="L60" s="14"/>
       <x:c r="M60" s="14"/>
       <x:c r="N60" s="17"/>
-      <x:c r="O60" s="14"/>
-      <x:c r="P60" s="14"/>
+      <x:c r="O60" s="17"/>
+      <x:c r="P60" s="17"/>
+      <x:c r="Q60" s="14"/>
+      <x:c r="R60" s="14"/>
     </x:row>
     <x:row r="61" ht="22" customHeight="1">
       <x:c r="A61" s="17"/>
@@ -1535,8 +1661,10 @@
       <x:c r="L61" s="14"/>
       <x:c r="M61" s="14"/>
       <x:c r="N61" s="17"/>
-      <x:c r="O61" s="14"/>
-      <x:c r="P61" s="14"/>
+      <x:c r="O61" s="17"/>
+      <x:c r="P61" s="17"/>
+      <x:c r="Q61" s="14"/>
+      <x:c r="R61" s="14"/>
     </x:row>
     <x:row r="62" ht="22" customHeight="1">
       <x:c r="A62" s="17"/>
@@ -1553,8 +1681,10 @@
       <x:c r="L62" s="14"/>
       <x:c r="M62" s="14"/>
       <x:c r="N62" s="17"/>
-      <x:c r="O62" s="14"/>
-      <x:c r="P62" s="14"/>
+      <x:c r="O62" s="17"/>
+      <x:c r="P62" s="17"/>
+      <x:c r="Q62" s="14"/>
+      <x:c r="R62" s="14"/>
     </x:row>
     <x:row r="63" ht="22" customHeight="1">
       <x:c r="A63" s="17"/>
@@ -1571,8 +1701,10 @@
       <x:c r="L63" s="14"/>
       <x:c r="M63" s="14"/>
       <x:c r="N63" s="17"/>
-      <x:c r="O63" s="14"/>
-      <x:c r="P63" s="14"/>
+      <x:c r="O63" s="17"/>
+      <x:c r="P63" s="17"/>
+      <x:c r="Q63" s="14"/>
+      <x:c r="R63" s="14"/>
     </x:row>
     <x:row r="64" ht="22" customHeight="1">
       <x:c r="A64" s="17"/>
@@ -1589,8 +1721,10 @@
       <x:c r="L64" s="14"/>
       <x:c r="M64" s="14"/>
       <x:c r="N64" s="17"/>
-      <x:c r="O64" s="14"/>
-      <x:c r="P64" s="14"/>
+      <x:c r="O64" s="17"/>
+      <x:c r="P64" s="17"/>
+      <x:c r="Q64" s="14"/>
+      <x:c r="R64" s="14"/>
     </x:row>
     <x:row r="65" ht="22" customHeight="1">
       <x:c r="A65" s="17"/>
@@ -1607,8 +1741,10 @@
       <x:c r="L65" s="14"/>
       <x:c r="M65" s="14"/>
       <x:c r="N65" s="17"/>
-      <x:c r="O65" s="14"/>
-      <x:c r="P65" s="14"/>
+      <x:c r="O65" s="17"/>
+      <x:c r="P65" s="17"/>
+      <x:c r="Q65" s="14"/>
+      <x:c r="R65" s="14"/>
     </x:row>
     <x:row r="66" ht="22" customHeight="1">
       <x:c r="A66" s="17"/>
@@ -1625,8 +1761,10 @@
       <x:c r="L66" s="14"/>
       <x:c r="M66" s="14"/>
       <x:c r="N66" s="17"/>
-      <x:c r="O66" s="14"/>
-      <x:c r="P66" s="14"/>
+      <x:c r="O66" s="17"/>
+      <x:c r="P66" s="17"/>
+      <x:c r="Q66" s="14"/>
+      <x:c r="R66" s="14"/>
     </x:row>
     <x:row r="67" ht="22" customHeight="1">
       <x:c r="A67" s="17"/>
@@ -1643,8 +1781,10 @@
       <x:c r="L67" s="14"/>
       <x:c r="M67" s="14"/>
       <x:c r="N67" s="17"/>
-      <x:c r="O67" s="14"/>
-      <x:c r="P67" s="14"/>
+      <x:c r="O67" s="17"/>
+      <x:c r="P67" s="17"/>
+      <x:c r="Q67" s="14"/>
+      <x:c r="R67" s="14"/>
     </x:row>
     <x:row r="68" ht="22" customHeight="1">
       <x:c r="A68" s="17"/>
@@ -1661,8 +1801,10 @@
       <x:c r="L68" s="14"/>
       <x:c r="M68" s="14"/>
       <x:c r="N68" s="17"/>
-      <x:c r="O68" s="14"/>
-      <x:c r="P68" s="14"/>
+      <x:c r="O68" s="17"/>
+      <x:c r="P68" s="17"/>
+      <x:c r="Q68" s="14"/>
+      <x:c r="R68" s="14"/>
     </x:row>
     <x:row r="69" ht="22" customHeight="1">
       <x:c r="A69" s="17"/>
@@ -1679,8 +1821,10 @@
       <x:c r="L69" s="14"/>
       <x:c r="M69" s="14"/>
       <x:c r="N69" s="17"/>
-      <x:c r="O69" s="14"/>
-      <x:c r="P69" s="14"/>
+      <x:c r="O69" s="17"/>
+      <x:c r="P69" s="17"/>
+      <x:c r="Q69" s="14"/>
+      <x:c r="R69" s="14"/>
     </x:row>
     <x:row r="70" ht="22" customHeight="1">
       <x:c r="A70" s="17"/>
@@ -1697,8 +1841,10 @@
       <x:c r="L70" s="14"/>
       <x:c r="M70" s="14"/>
       <x:c r="N70" s="17"/>
-      <x:c r="O70" s="14"/>
-      <x:c r="P70" s="14"/>
+      <x:c r="O70" s="17"/>
+      <x:c r="P70" s="17"/>
+      <x:c r="Q70" s="14"/>
+      <x:c r="R70" s="14"/>
     </x:row>
     <x:row r="71" ht="22" customHeight="1">
       <x:c r="A71" s="17"/>
@@ -1715,8 +1861,10 @@
       <x:c r="L71" s="14"/>
       <x:c r="M71" s="14"/>
       <x:c r="N71" s="17"/>
-      <x:c r="O71" s="14"/>
-      <x:c r="P71" s="14"/>
+      <x:c r="O71" s="17"/>
+      <x:c r="P71" s="17"/>
+      <x:c r="Q71" s="14"/>
+      <x:c r="R71" s="14"/>
     </x:row>
     <x:row r="72" ht="22" customHeight="1">
       <x:c r="A72" s="17"/>
@@ -1733,8 +1881,10 @@
       <x:c r="L72" s="14"/>
       <x:c r="M72" s="14"/>
       <x:c r="N72" s="17"/>
-      <x:c r="O72" s="14"/>
-      <x:c r="P72" s="14"/>
+      <x:c r="O72" s="17"/>
+      <x:c r="P72" s="17"/>
+      <x:c r="Q72" s="14"/>
+      <x:c r="R72" s="14"/>
     </x:row>
     <x:row r="73" ht="22" customHeight="1">
       <x:c r="A73" s="17"/>
@@ -1751,8 +1901,10 @@
       <x:c r="L73" s="14"/>
       <x:c r="M73" s="14"/>
       <x:c r="N73" s="17"/>
-      <x:c r="O73" s="14"/>
-      <x:c r="P73" s="14"/>
+      <x:c r="O73" s="17"/>
+      <x:c r="P73" s="17"/>
+      <x:c r="Q73" s="14"/>
+      <x:c r="R73" s="14"/>
     </x:row>
     <x:row r="74" ht="22" customHeight="1">
       <x:c r="A74" s="17"/>
@@ -1769,8 +1921,10 @@
       <x:c r="L74" s="14"/>
       <x:c r="M74" s="14"/>
       <x:c r="N74" s="17"/>
-      <x:c r="O74" s="14"/>
-      <x:c r="P74" s="14"/>
+      <x:c r="O74" s="17"/>
+      <x:c r="P74" s="17"/>
+      <x:c r="Q74" s="14"/>
+      <x:c r="R74" s="14"/>
     </x:row>
     <x:row r="75" ht="22" customHeight="1">
       <x:c r="A75" s="17"/>
@@ -1787,8 +1941,10 @@
       <x:c r="L75" s="14"/>
       <x:c r="M75" s="14"/>
       <x:c r="N75" s="17"/>
-      <x:c r="O75" s="14"/>
-      <x:c r="P75" s="14"/>
+      <x:c r="O75" s="17"/>
+      <x:c r="P75" s="17"/>
+      <x:c r="Q75" s="14"/>
+      <x:c r="R75" s="14"/>
     </x:row>
     <x:row r="76" ht="22" customHeight="1">
       <x:c r="A76" s="17"/>
@@ -1805,8 +1961,10 @@
       <x:c r="L76" s="14"/>
       <x:c r="M76" s="14"/>
       <x:c r="N76" s="17"/>
-      <x:c r="O76" s="14"/>
-      <x:c r="P76" s="14"/>
+      <x:c r="O76" s="17"/>
+      <x:c r="P76" s="17"/>
+      <x:c r="Q76" s="14"/>
+      <x:c r="R76" s="14"/>
     </x:row>
     <x:row r="77" ht="22" customHeight="1">
       <x:c r="A77" s="17"/>
@@ -1823,8 +1981,10 @@
       <x:c r="L77" s="14"/>
       <x:c r="M77" s="14"/>
       <x:c r="N77" s="17"/>
-      <x:c r="O77" s="14"/>
-      <x:c r="P77" s="14"/>
+      <x:c r="O77" s="17"/>
+      <x:c r="P77" s="17"/>
+      <x:c r="Q77" s="14"/>
+      <x:c r="R77" s="14"/>
     </x:row>
     <x:row r="78" ht="22" customHeight="1">
       <x:c r="A78" s="17"/>
@@ -1841,8 +2001,10 @@
       <x:c r="L78" s="14"/>
       <x:c r="M78" s="14"/>
       <x:c r="N78" s="17"/>
-      <x:c r="O78" s="14"/>
-      <x:c r="P78" s="14"/>
+      <x:c r="O78" s="17"/>
+      <x:c r="P78" s="17"/>
+      <x:c r="Q78" s="14"/>
+      <x:c r="R78" s="14"/>
     </x:row>
     <x:row r="79" ht="22" customHeight="1">
       <x:c r="A79" s="17"/>
@@ -1859,8 +2021,10 @@
       <x:c r="L79" s="14"/>
       <x:c r="M79" s="14"/>
       <x:c r="N79" s="17"/>
-      <x:c r="O79" s="14"/>
-      <x:c r="P79" s="14"/>
+      <x:c r="O79" s="17"/>
+      <x:c r="P79" s="17"/>
+      <x:c r="Q79" s="14"/>
+      <x:c r="R79" s="14"/>
     </x:row>
     <x:row r="80" ht="22" customHeight="1">
       <x:c r="A80" s="17"/>
@@ -1877,8 +2041,10 @@
       <x:c r="L80" s="14"/>
       <x:c r="M80" s="14"/>
       <x:c r="N80" s="17"/>
-      <x:c r="O80" s="14"/>
-      <x:c r="P80" s="14"/>
+      <x:c r="O80" s="17"/>
+      <x:c r="P80" s="17"/>
+      <x:c r="Q80" s="14"/>
+      <x:c r="R80" s="14"/>
     </x:row>
     <x:row r="81" ht="22" customHeight="1">
       <x:c r="A81" s="17"/>
@@ -1895,8 +2061,10 @@
       <x:c r="L81" s="14"/>
       <x:c r="M81" s="14"/>
       <x:c r="N81" s="17"/>
-      <x:c r="O81" s="14"/>
-      <x:c r="P81" s="14"/>
+      <x:c r="O81" s="17"/>
+      <x:c r="P81" s="17"/>
+      <x:c r="Q81" s="14"/>
+      <x:c r="R81" s="14"/>
     </x:row>
     <x:row r="82" ht="22" customHeight="1">
       <x:c r="A82" s="17"/>
@@ -1913,8 +2081,10 @@
       <x:c r="L82" s="14"/>
       <x:c r="M82" s="14"/>
       <x:c r="N82" s="17"/>
-      <x:c r="O82" s="14"/>
-      <x:c r="P82" s="14"/>
+      <x:c r="O82" s="17"/>
+      <x:c r="P82" s="17"/>
+      <x:c r="Q82" s="14"/>
+      <x:c r="R82" s="14"/>
     </x:row>
     <x:row r="83" ht="22" customHeight="1">
       <x:c r="A83" s="17"/>
@@ -1931,8 +2101,10 @@
       <x:c r="L83" s="14"/>
       <x:c r="M83" s="14"/>
       <x:c r="N83" s="17"/>
-      <x:c r="O83" s="14"/>
-      <x:c r="P83" s="14"/>
+      <x:c r="O83" s="17"/>
+      <x:c r="P83" s="17"/>
+      <x:c r="Q83" s="14"/>
+      <x:c r="R83" s="14"/>
     </x:row>
     <x:row r="84" ht="22" customHeight="1">
       <x:c r="A84" s="17"/>
@@ -1949,8 +2121,10 @@
       <x:c r="L84" s="14"/>
       <x:c r="M84" s="14"/>
       <x:c r="N84" s="17"/>
-      <x:c r="O84" s="14"/>
-      <x:c r="P84" s="14"/>
+      <x:c r="O84" s="17"/>
+      <x:c r="P84" s="17"/>
+      <x:c r="Q84" s="14"/>
+      <x:c r="R84" s="14"/>
     </x:row>
     <x:row r="85" ht="22" customHeight="1">
       <x:c r="A85" s="17"/>
@@ -1967,8 +2141,10 @@
       <x:c r="L85" s="14"/>
       <x:c r="M85" s="14"/>
       <x:c r="N85" s="17"/>
-      <x:c r="O85" s="14"/>
-      <x:c r="P85" s="14"/>
+      <x:c r="O85" s="17"/>
+      <x:c r="P85" s="17"/>
+      <x:c r="Q85" s="14"/>
+      <x:c r="R85" s="14"/>
     </x:row>
     <x:row r="86" ht="22" customHeight="1">
       <x:c r="A86" s="17"/>
@@ -1985,8 +2161,10 @@
       <x:c r="L86" s="14"/>
       <x:c r="M86" s="14"/>
       <x:c r="N86" s="17"/>
-      <x:c r="O86" s="14"/>
-      <x:c r="P86" s="14"/>
+      <x:c r="O86" s="17"/>
+      <x:c r="P86" s="17"/>
+      <x:c r="Q86" s="14"/>
+      <x:c r="R86" s="14"/>
     </x:row>
     <x:row r="87" ht="22" customHeight="1">
       <x:c r="A87" s="17"/>
@@ -2003,8 +2181,10 @@
       <x:c r="L87" s="14"/>
       <x:c r="M87" s="14"/>
       <x:c r="N87" s="17"/>
-      <x:c r="O87" s="14"/>
-      <x:c r="P87" s="14"/>
+      <x:c r="O87" s="17"/>
+      <x:c r="P87" s="17"/>
+      <x:c r="Q87" s="14"/>
+      <x:c r="R87" s="14"/>
     </x:row>
     <x:row r="88" ht="22" customHeight="1">
       <x:c r="A88" s="17"/>
@@ -2021,8 +2201,10 @@
       <x:c r="L88" s="14"/>
       <x:c r="M88" s="14"/>
       <x:c r="N88" s="17"/>
-      <x:c r="O88" s="14"/>
-      <x:c r="P88" s="14"/>
+      <x:c r="O88" s="17"/>
+      <x:c r="P88" s="17"/>
+      <x:c r="Q88" s="14"/>
+      <x:c r="R88" s="14"/>
     </x:row>
     <x:row r="89" ht="22" customHeight="1">
       <x:c r="A89" s="17"/>
@@ -2039,8 +2221,10 @@
       <x:c r="L89" s="14"/>
       <x:c r="M89" s="14"/>
       <x:c r="N89" s="17"/>
-      <x:c r="O89" s="14"/>
-      <x:c r="P89" s="14"/>
+      <x:c r="O89" s="17"/>
+      <x:c r="P89" s="17"/>
+      <x:c r="Q89" s="14"/>
+      <x:c r="R89" s="14"/>
     </x:row>
     <x:row r="90" ht="22" customHeight="1">
       <x:c r="A90" s="17"/>
@@ -2057,8 +2241,10 @@
       <x:c r="L90" s="14"/>
       <x:c r="M90" s="14"/>
       <x:c r="N90" s="17"/>
-      <x:c r="O90" s="14"/>
-      <x:c r="P90" s="14"/>
+      <x:c r="O90" s="17"/>
+      <x:c r="P90" s="17"/>
+      <x:c r="Q90" s="14"/>
+      <x:c r="R90" s="14"/>
     </x:row>
     <x:row r="91" ht="22" customHeight="1">
       <x:c r="A91" s="17"/>
@@ -2075,8 +2261,10 @@
       <x:c r="L91" s="14"/>
       <x:c r="M91" s="14"/>
       <x:c r="N91" s="17"/>
-      <x:c r="O91" s="14"/>
-      <x:c r="P91" s="14"/>
+      <x:c r="O91" s="17"/>
+      <x:c r="P91" s="17"/>
+      <x:c r="Q91" s="14"/>
+      <x:c r="R91" s="14"/>
     </x:row>
     <x:row r="92" ht="22" customHeight="1">
       <x:c r="A92" s="17"/>
@@ -2093,8 +2281,10 @@
       <x:c r="L92" s="14"/>
       <x:c r="M92" s="14"/>
       <x:c r="N92" s="17"/>
-      <x:c r="O92" s="14"/>
-      <x:c r="P92" s="14"/>
+      <x:c r="O92" s="17"/>
+      <x:c r="P92" s="17"/>
+      <x:c r="Q92" s="14"/>
+      <x:c r="R92" s="14"/>
     </x:row>
     <x:row r="93" ht="22" customHeight="1">
       <x:c r="A93" s="17"/>
@@ -2111,8 +2301,10 @@
       <x:c r="L93" s="14"/>
       <x:c r="M93" s="14"/>
       <x:c r="N93" s="17"/>
-      <x:c r="O93" s="14"/>
-      <x:c r="P93" s="14"/>
+      <x:c r="O93" s="17"/>
+      <x:c r="P93" s="17"/>
+      <x:c r="Q93" s="14"/>
+      <x:c r="R93" s="14"/>
     </x:row>
     <x:row r="94" ht="22" customHeight="1">
       <x:c r="A94" s="17"/>
@@ -2129,8 +2321,10 @@
       <x:c r="L94" s="14"/>
       <x:c r="M94" s="14"/>
       <x:c r="N94" s="17"/>
-      <x:c r="O94" s="14"/>
-      <x:c r="P94" s="14"/>
+      <x:c r="O94" s="17"/>
+      <x:c r="P94" s="17"/>
+      <x:c r="Q94" s="14"/>
+      <x:c r="R94" s="14"/>
     </x:row>
     <x:row r="95" ht="22" customHeight="1">
       <x:c r="A95" s="17"/>
@@ -2147,8 +2341,10 @@
       <x:c r="L95" s="14"/>
       <x:c r="M95" s="14"/>
       <x:c r="N95" s="17"/>
-      <x:c r="O95" s="14"/>
-      <x:c r="P95" s="14"/>
+      <x:c r="O95" s="17"/>
+      <x:c r="P95" s="17"/>
+      <x:c r="Q95" s="14"/>
+      <x:c r="R95" s="14"/>
     </x:row>
     <x:row r="96" ht="22" customHeight="1">
       <x:c r="A96" s="17"/>
@@ -2165,8 +2361,10 @@
       <x:c r="L96" s="14"/>
       <x:c r="M96" s="14"/>
       <x:c r="N96" s="17"/>
-      <x:c r="O96" s="14"/>
-      <x:c r="P96" s="14"/>
+      <x:c r="O96" s="17"/>
+      <x:c r="P96" s="17"/>
+      <x:c r="Q96" s="14"/>
+      <x:c r="R96" s="14"/>
     </x:row>
     <x:row r="97" ht="22" customHeight="1">
       <x:c r="A97" s="17"/>
@@ -2183,8 +2381,10 @@
       <x:c r="L97" s="14"/>
       <x:c r="M97" s="14"/>
       <x:c r="N97" s="17"/>
-      <x:c r="O97" s="14"/>
-      <x:c r="P97" s="14"/>
+      <x:c r="O97" s="17"/>
+      <x:c r="P97" s="17"/>
+      <x:c r="Q97" s="14"/>
+      <x:c r="R97" s="14"/>
     </x:row>
     <x:row r="98" ht="22" customHeight="1">
       <x:c r="A98" s="17"/>
@@ -2201,8 +2401,10 @@
       <x:c r="L98" s="14"/>
       <x:c r="M98" s="14"/>
       <x:c r="N98" s="17"/>
-      <x:c r="O98" s="14"/>
-      <x:c r="P98" s="14"/>
+      <x:c r="O98" s="17"/>
+      <x:c r="P98" s="17"/>
+      <x:c r="Q98" s="14"/>
+      <x:c r="R98" s="14"/>
     </x:row>
     <x:row r="99" ht="22" customHeight="1">
       <x:c r="A99" s="17"/>
@@ -2219,8 +2421,10 @@
       <x:c r="L99" s="14"/>
       <x:c r="M99" s="14"/>
       <x:c r="N99" s="17"/>
-      <x:c r="O99" s="14"/>
-      <x:c r="P99" s="14"/>
+      <x:c r="O99" s="17"/>
+      <x:c r="P99" s="17"/>
+      <x:c r="Q99" s="14"/>
+      <x:c r="R99" s="14"/>
     </x:row>
     <x:row r="100" ht="22" customHeight="1">
       <x:c r="A100" s="17"/>
@@ -2237,8 +2441,10 @@
       <x:c r="L100" s="14"/>
       <x:c r="M100" s="14"/>
       <x:c r="N100" s="17"/>
-      <x:c r="O100" s="14"/>
-      <x:c r="P100" s="14"/>
+      <x:c r="O100" s="17"/>
+      <x:c r="P100" s="17"/>
+      <x:c r="Q100" s="14"/>
+      <x:c r="R100" s="14"/>
     </x:row>
     <x:row r="101" ht="22" customHeight="1">
       <x:c r="A101" s="17"/>
@@ -2255,8 +2461,10 @@
       <x:c r="L101" s="14"/>
       <x:c r="M101" s="14"/>
       <x:c r="N101" s="17"/>
-      <x:c r="O101" s="14"/>
-      <x:c r="P101" s="14"/>
+      <x:c r="O101" s="17"/>
+      <x:c r="P101" s="17"/>
+      <x:c r="Q101" s="14"/>
+      <x:c r="R101" s="14"/>
     </x:row>
     <x:row r="102" ht="22" customHeight="1">
       <x:c r="A102" s="17"/>
@@ -2273,8 +2481,10 @@
       <x:c r="L102" s="14"/>
       <x:c r="M102" s="14"/>
       <x:c r="N102" s="17"/>
-      <x:c r="O102" s="14"/>
-      <x:c r="P102" s="14"/>
+      <x:c r="O102" s="17"/>
+      <x:c r="P102" s="17"/>
+      <x:c r="Q102" s="14"/>
+      <x:c r="R102" s="14"/>
     </x:row>
     <x:row r="103" ht="22" customHeight="1">
       <x:c r="A103" s="17"/>
@@ -2291,8 +2501,10 @@
       <x:c r="L103" s="14"/>
       <x:c r="M103" s="14"/>
       <x:c r="N103" s="17"/>
-      <x:c r="O103" s="14"/>
-      <x:c r="P103" s="14"/>
+      <x:c r="O103" s="17"/>
+      <x:c r="P103" s="17"/>
+      <x:c r="Q103" s="14"/>
+      <x:c r="R103" s="14"/>
     </x:row>
     <x:row r="104" ht="22" customHeight="1">
       <x:c r="A104" s="17"/>
@@ -2309,8 +2521,10 @@
       <x:c r="L104" s="14"/>
       <x:c r="M104" s="14"/>
       <x:c r="N104" s="17"/>
-      <x:c r="O104" s="14"/>
-      <x:c r="P104" s="14"/>
+      <x:c r="O104" s="17"/>
+      <x:c r="P104" s="17"/>
+      <x:c r="Q104" s="14"/>
+      <x:c r="R104" s="14"/>
     </x:row>
     <x:row r="105" ht="22" customHeight="1">
       <x:c r="A105" s="17"/>
@@ -2327,8 +2541,10 @@
       <x:c r="L105" s="14"/>
       <x:c r="M105" s="14"/>
       <x:c r="N105" s="17"/>
-      <x:c r="O105" s="14"/>
-      <x:c r="P105" s="14"/>
+      <x:c r="O105" s="17"/>
+      <x:c r="P105" s="17"/>
+      <x:c r="Q105" s="14"/>
+      <x:c r="R105" s="14"/>
     </x:row>
     <x:row r="106" ht="22" customHeight="1">
       <x:c r="A106" s="17"/>
@@ -2345,8 +2561,10 @@
       <x:c r="L106" s="14"/>
       <x:c r="M106" s="14"/>
       <x:c r="N106" s="17"/>
-      <x:c r="O106" s="14"/>
-      <x:c r="P106" s="14"/>
+      <x:c r="O106" s="17"/>
+      <x:c r="P106" s="17"/>
+      <x:c r="Q106" s="14"/>
+      <x:c r="R106" s="14"/>
     </x:row>
     <x:row r="107" ht="22" customHeight="1">
       <x:c r="A107" s="17"/>
@@ -2363,8 +2581,10 @@
       <x:c r="L107" s="14"/>
       <x:c r="M107" s="14"/>
       <x:c r="N107" s="17"/>
-      <x:c r="O107" s="14"/>
-      <x:c r="P107" s="14"/>
+      <x:c r="O107" s="17"/>
+      <x:c r="P107" s="17"/>
+      <x:c r="Q107" s="14"/>
+      <x:c r="R107" s="14"/>
     </x:row>
     <x:row r="108" ht="22" customHeight="1">
       <x:c r="A108" s="17"/>
@@ -2381,8 +2601,10 @@
       <x:c r="L108" s="14"/>
       <x:c r="M108" s="14"/>
       <x:c r="N108" s="17"/>
-      <x:c r="O108" s="14"/>
-      <x:c r="P108" s="14"/>
+      <x:c r="O108" s="17"/>
+      <x:c r="P108" s="17"/>
+      <x:c r="Q108" s="14"/>
+      <x:c r="R108" s="14"/>
     </x:row>
     <x:row r="109" ht="22" customHeight="1">
       <x:c r="A109" s="17"/>
@@ -2399,8 +2621,10 @@
       <x:c r="L109" s="14"/>
       <x:c r="M109" s="14"/>
       <x:c r="N109" s="17"/>
-      <x:c r="O109" s="14"/>
-      <x:c r="P109" s="14"/>
+      <x:c r="O109" s="17"/>
+      <x:c r="P109" s="17"/>
+      <x:c r="Q109" s="14"/>
+      <x:c r="R109" s="14"/>
     </x:row>
     <x:row r="110" ht="22" customHeight="1">
       <x:c r="A110" s="17"/>
@@ -2417,8 +2641,10 @@
       <x:c r="L110" s="14"/>
       <x:c r="M110" s="14"/>
       <x:c r="N110" s="17"/>
-      <x:c r="O110" s="14"/>
-      <x:c r="P110" s="14"/>
+      <x:c r="O110" s="17"/>
+      <x:c r="P110" s="17"/>
+      <x:c r="Q110" s="14"/>
+      <x:c r="R110" s="14"/>
     </x:row>
     <x:row r="111" ht="22" customHeight="1">
       <x:c r="A111" s="17"/>
@@ -2435,8 +2661,10 @@
       <x:c r="L111" s="14"/>
       <x:c r="M111" s="14"/>
       <x:c r="N111" s="17"/>
-      <x:c r="O111" s="14"/>
-      <x:c r="P111" s="14"/>
+      <x:c r="O111" s="17"/>
+      <x:c r="P111" s="17"/>
+      <x:c r="Q111" s="14"/>
+      <x:c r="R111" s="14"/>
     </x:row>
     <x:row r="112" ht="22" customHeight="1">
       <x:c r="A112" s="17"/>
@@ -2453,8 +2681,10 @@
       <x:c r="L112" s="14"/>
       <x:c r="M112" s="14"/>
       <x:c r="N112" s="17"/>
-      <x:c r="O112" s="14"/>
-      <x:c r="P112" s="14"/>
+      <x:c r="O112" s="17"/>
+      <x:c r="P112" s="17"/>
+      <x:c r="Q112" s="14"/>
+      <x:c r="R112" s="14"/>
     </x:row>
     <x:row r="113" ht="22" customHeight="1">
       <x:c r="A113" s="17"/>
@@ -2471,8 +2701,10 @@
       <x:c r="L113" s="14"/>
       <x:c r="M113" s="14"/>
       <x:c r="N113" s="17"/>
-      <x:c r="O113" s="14"/>
-      <x:c r="P113" s="14"/>
+      <x:c r="O113" s="17"/>
+      <x:c r="P113" s="17"/>
+      <x:c r="Q113" s="14"/>
+      <x:c r="R113" s="14"/>
     </x:row>
     <x:row r="114" ht="22" customHeight="1">
       <x:c r="A114" s="17"/>
@@ -2489,8 +2721,10 @@
       <x:c r="L114" s="14"/>
       <x:c r="M114" s="14"/>
       <x:c r="N114" s="17"/>
-      <x:c r="O114" s="14"/>
-      <x:c r="P114" s="14"/>
+      <x:c r="O114" s="17"/>
+      <x:c r="P114" s="17"/>
+      <x:c r="Q114" s="14"/>
+      <x:c r="R114" s="14"/>
     </x:row>
     <x:row r="115" ht="22" customHeight="1">
       <x:c r="A115" s="17"/>
@@ -2507,8 +2741,10 @@
       <x:c r="L115" s="14"/>
       <x:c r="M115" s="14"/>
       <x:c r="N115" s="17"/>
-      <x:c r="O115" s="14"/>
-      <x:c r="P115" s="14"/>
+      <x:c r="O115" s="17"/>
+      <x:c r="P115" s="17"/>
+      <x:c r="Q115" s="14"/>
+      <x:c r="R115" s="14"/>
     </x:row>
     <x:row r="116" ht="22" customHeight="1">
       <x:c r="A116" s="17"/>
@@ -2525,8 +2761,10 @@
       <x:c r="L116" s="14"/>
       <x:c r="M116" s="14"/>
       <x:c r="N116" s="17"/>
-      <x:c r="O116" s="14"/>
-      <x:c r="P116" s="14"/>
+      <x:c r="O116" s="17"/>
+      <x:c r="P116" s="17"/>
+      <x:c r="Q116" s="14"/>
+      <x:c r="R116" s="14"/>
     </x:row>
     <x:row r="117" ht="22" customHeight="1">
       <x:c r="A117" s="17"/>
@@ -2543,8 +2781,10 @@
       <x:c r="L117" s="14"/>
       <x:c r="M117" s="14"/>
       <x:c r="N117" s="17"/>
-      <x:c r="O117" s="14"/>
-      <x:c r="P117" s="14"/>
+      <x:c r="O117" s="17"/>
+      <x:c r="P117" s="17"/>
+      <x:c r="Q117" s="14"/>
+      <x:c r="R117" s="14"/>
     </x:row>
     <x:row r="118" ht="22" customHeight="1">
       <x:c r="A118" s="17"/>
@@ -2561,8 +2801,10 @@
       <x:c r="L118" s="14"/>
       <x:c r="M118" s="14"/>
       <x:c r="N118" s="17"/>
-      <x:c r="O118" s="14"/>
-      <x:c r="P118" s="14"/>
+      <x:c r="O118" s="17"/>
+      <x:c r="P118" s="17"/>
+      <x:c r="Q118" s="14"/>
+      <x:c r="R118" s="14"/>
     </x:row>
     <x:row r="119" ht="22" customHeight="1">
       <x:c r="A119" s="17"/>
@@ -2579,8 +2821,10 @@
       <x:c r="L119" s="14"/>
       <x:c r="M119" s="14"/>
       <x:c r="N119" s="17"/>
-      <x:c r="O119" s="14"/>
-      <x:c r="P119" s="14"/>
+      <x:c r="O119" s="17"/>
+      <x:c r="P119" s="17"/>
+      <x:c r="Q119" s="14"/>
+      <x:c r="R119" s="14"/>
     </x:row>
     <x:row r="120" ht="22" customHeight="1">
       <x:c r="A120" s="17"/>
@@ -2597,8 +2841,10 @@
       <x:c r="L120" s="14"/>
       <x:c r="M120" s="14"/>
       <x:c r="N120" s="17"/>
-      <x:c r="O120" s="14"/>
-      <x:c r="P120" s="14"/>
+      <x:c r="O120" s="17"/>
+      <x:c r="P120" s="17"/>
+      <x:c r="Q120" s="14"/>
+      <x:c r="R120" s="14"/>
     </x:row>
     <x:row r="121" ht="22" customHeight="1">
       <x:c r="A121" s="17"/>
@@ -2615,8 +2861,10 @@
       <x:c r="L121" s="14"/>
       <x:c r="M121" s="14"/>
       <x:c r="N121" s="17"/>
-      <x:c r="O121" s="14"/>
-      <x:c r="P121" s="14"/>
+      <x:c r="O121" s="17"/>
+      <x:c r="P121" s="17"/>
+      <x:c r="Q121" s="14"/>
+      <x:c r="R121" s="14"/>
     </x:row>
     <x:row r="122" ht="22" customHeight="1">
       <x:c r="A122" s="17"/>
@@ -2633,8 +2881,10 @@
       <x:c r="L122" s="14"/>
       <x:c r="M122" s="14"/>
       <x:c r="N122" s="17"/>
-      <x:c r="O122" s="14"/>
-      <x:c r="P122" s="14"/>
+      <x:c r="O122" s="17"/>
+      <x:c r="P122" s="17"/>
+      <x:c r="Q122" s="14"/>
+      <x:c r="R122" s="14"/>
     </x:row>
     <x:row r="123" ht="22" customHeight="1">
       <x:c r="A123" s="17"/>
@@ -2651,8 +2901,10 @@
       <x:c r="L123" s="14"/>
       <x:c r="M123" s="14"/>
       <x:c r="N123" s="17"/>
-      <x:c r="O123" s="14"/>
-      <x:c r="P123" s="14"/>
+      <x:c r="O123" s="17"/>
+      <x:c r="P123" s="17"/>
+      <x:c r="Q123" s="14"/>
+      <x:c r="R123" s="14"/>
     </x:row>
     <x:row r="124" ht="22" customHeight="1">
       <x:c r="A124" s="17"/>
@@ -2669,8 +2921,10 @@
       <x:c r="L124" s="14"/>
       <x:c r="M124" s="14"/>
       <x:c r="N124" s="17"/>
-      <x:c r="O124" s="14"/>
-      <x:c r="P124" s="14"/>
+      <x:c r="O124" s="17"/>
+      <x:c r="P124" s="17"/>
+      <x:c r="Q124" s="14"/>
+      <x:c r="R124" s="14"/>
     </x:row>
     <x:row r="125" ht="22" customHeight="1">
       <x:c r="A125" s="17"/>
@@ -2687,8 +2941,10 @@
       <x:c r="L125" s="14"/>
       <x:c r="M125" s="14"/>
       <x:c r="N125" s="17"/>
-      <x:c r="O125" s="14"/>
-      <x:c r="P125" s="14"/>
+      <x:c r="O125" s="17"/>
+      <x:c r="P125" s="17"/>
+      <x:c r="Q125" s="14"/>
+      <x:c r="R125" s="14"/>
     </x:row>
     <x:row r="126" ht="22" customHeight="1">
       <x:c r="A126" s="17"/>
@@ -2705,8 +2961,10 @@
       <x:c r="L126" s="14"/>
       <x:c r="M126" s="14"/>
       <x:c r="N126" s="17"/>
-      <x:c r="O126" s="14"/>
-      <x:c r="P126" s="14"/>
+      <x:c r="O126" s="17"/>
+      <x:c r="P126" s="17"/>
+      <x:c r="Q126" s="14"/>
+      <x:c r="R126" s="14"/>
     </x:row>
     <x:row r="127" ht="22" customHeight="1">
       <x:c r="A127" s="17"/>
@@ -2723,8 +2981,10 @@
       <x:c r="L127" s="14"/>
       <x:c r="M127" s="14"/>
       <x:c r="N127" s="17"/>
-      <x:c r="O127" s="14"/>
-      <x:c r="P127" s="14"/>
+      <x:c r="O127" s="17"/>
+      <x:c r="P127" s="17"/>
+      <x:c r="Q127" s="14"/>
+      <x:c r="R127" s="14"/>
     </x:row>
     <x:row r="128" ht="22" customHeight="1">
       <x:c r="A128" s="17"/>
@@ -2741,8 +3001,10 @@
       <x:c r="L128" s="14"/>
       <x:c r="M128" s="14"/>
       <x:c r="N128" s="17"/>
-      <x:c r="O128" s="14"/>
-      <x:c r="P128" s="14"/>
+      <x:c r="O128" s="17"/>
+      <x:c r="P128" s="17"/>
+      <x:c r="Q128" s="14"/>
+      <x:c r="R128" s="14"/>
     </x:row>
     <x:row r="129" ht="22" customHeight="1">
       <x:c r="A129" s="17"/>
@@ -2759,8 +3021,10 @@
       <x:c r="L129" s="14"/>
       <x:c r="M129" s="14"/>
       <x:c r="N129" s="17"/>
-      <x:c r="O129" s="14"/>
-      <x:c r="P129" s="14"/>
+      <x:c r="O129" s="17"/>
+      <x:c r="P129" s="17"/>
+      <x:c r="Q129" s="14"/>
+      <x:c r="R129" s="14"/>
     </x:row>
     <x:row r="130" ht="22" customHeight="1">
       <x:c r="A130" s="17"/>
@@ -2777,8 +3041,10 @@
       <x:c r="L130" s="14"/>
       <x:c r="M130" s="14"/>
       <x:c r="N130" s="17"/>
-      <x:c r="O130" s="14"/>
-      <x:c r="P130" s="14"/>
+      <x:c r="O130" s="17"/>
+      <x:c r="P130" s="17"/>
+      <x:c r="Q130" s="14"/>
+      <x:c r="R130" s="14"/>
     </x:row>
     <x:row r="131" ht="22" customHeight="1">
       <x:c r="A131" s="17"/>
@@ -2795,8 +3061,10 @@
       <x:c r="L131" s="14"/>
       <x:c r="M131" s="14"/>
       <x:c r="N131" s="17"/>
-      <x:c r="O131" s="14"/>
-      <x:c r="P131" s="14"/>
+      <x:c r="O131" s="17"/>
+      <x:c r="P131" s="17"/>
+      <x:c r="Q131" s="14"/>
+      <x:c r="R131" s="14"/>
     </x:row>
     <x:row r="132" ht="22" customHeight="1">
       <x:c r="A132" s="17"/>
@@ -2813,8 +3081,10 @@
       <x:c r="L132" s="14"/>
       <x:c r="M132" s="14"/>
       <x:c r="N132" s="17"/>
-      <x:c r="O132" s="14"/>
-      <x:c r="P132" s="14"/>
+      <x:c r="O132" s="17"/>
+      <x:c r="P132" s="17"/>
+      <x:c r="Q132" s="14"/>
+      <x:c r="R132" s="14"/>
     </x:row>
     <x:row r="133" ht="22" customHeight="1">
       <x:c r="A133" s="17"/>
@@ -2831,8 +3101,10 @@
       <x:c r="L133" s="14"/>
       <x:c r="M133" s="14"/>
       <x:c r="N133" s="17"/>
-      <x:c r="O133" s="14"/>
-      <x:c r="P133" s="14"/>
+      <x:c r="O133" s="17"/>
+      <x:c r="P133" s="17"/>
+      <x:c r="Q133" s="14"/>
+      <x:c r="R133" s="14"/>
     </x:row>
     <x:row r="134" ht="22" customHeight="1">
       <x:c r="A134" s="17"/>
@@ -2849,8 +3121,10 @@
       <x:c r="L134" s="14"/>
       <x:c r="M134" s="14"/>
       <x:c r="N134" s="17"/>
-      <x:c r="O134" s="14"/>
-      <x:c r="P134" s="14"/>
+      <x:c r="O134" s="17"/>
+      <x:c r="P134" s="17"/>
+      <x:c r="Q134" s="14"/>
+      <x:c r="R134" s="14"/>
     </x:row>
     <x:row r="135" ht="22" customHeight="1">
       <x:c r="A135" s="17"/>
@@ -2867,8 +3141,10 @@
       <x:c r="L135" s="14"/>
       <x:c r="M135" s="14"/>
       <x:c r="N135" s="17"/>
-      <x:c r="O135" s="14"/>
-      <x:c r="P135" s="14"/>
+      <x:c r="O135" s="17"/>
+      <x:c r="P135" s="17"/>
+      <x:c r="Q135" s="14"/>
+      <x:c r="R135" s="14"/>
     </x:row>
     <x:row r="136" ht="22" customHeight="1">
       <x:c r="A136" s="17"/>
@@ -2885,8 +3161,10 @@
       <x:c r="L136" s="14"/>
       <x:c r="M136" s="14"/>
       <x:c r="N136" s="17"/>
-      <x:c r="O136" s="14"/>
-      <x:c r="P136" s="14"/>
+      <x:c r="O136" s="17"/>
+      <x:c r="P136" s="17"/>
+      <x:c r="Q136" s="14"/>
+      <x:c r="R136" s="14"/>
     </x:row>
     <x:row r="137" ht="22" customHeight="1">
       <x:c r="A137" s="17"/>
@@ -2903,8 +3181,10 @@
       <x:c r="L137" s="14"/>
       <x:c r="M137" s="14"/>
       <x:c r="N137" s="17"/>
-      <x:c r="O137" s="14"/>
-      <x:c r="P137" s="14"/>
+      <x:c r="O137" s="17"/>
+      <x:c r="P137" s="17"/>
+      <x:c r="Q137" s="14"/>
+      <x:c r="R137" s="14"/>
     </x:row>
     <x:row r="138" ht="22" customHeight="1">
       <x:c r="A138" s="17"/>
@@ -2921,8 +3201,10 @@
       <x:c r="L138" s="14"/>
       <x:c r="M138" s="14"/>
       <x:c r="N138" s="17"/>
-      <x:c r="O138" s="14"/>
-      <x:c r="P138" s="14"/>
+      <x:c r="O138" s="17"/>
+      <x:c r="P138" s="17"/>
+      <x:c r="Q138" s="14"/>
+      <x:c r="R138" s="14"/>
     </x:row>
     <x:row r="139" ht="22" customHeight="1">
       <x:c r="A139" s="17"/>
@@ -2939,8 +3221,10 @@
       <x:c r="L139" s="14"/>
       <x:c r="M139" s="14"/>
       <x:c r="N139" s="17"/>
-      <x:c r="O139" s="14"/>
-      <x:c r="P139" s="14"/>
+      <x:c r="O139" s="17"/>
+      <x:c r="P139" s="17"/>
+      <x:c r="Q139" s="14"/>
+      <x:c r="R139" s="14"/>
     </x:row>
     <x:row r="140" ht="22" customHeight="1">
       <x:c r="A140" s="17"/>
@@ -2957,8 +3241,10 @@
       <x:c r="L140" s="14"/>
       <x:c r="M140" s="14"/>
       <x:c r="N140" s="17"/>
-      <x:c r="O140" s="14"/>
-      <x:c r="P140" s="14"/>
+      <x:c r="O140" s="17"/>
+      <x:c r="P140" s="17"/>
+      <x:c r="Q140" s="14"/>
+      <x:c r="R140" s="14"/>
     </x:row>
     <x:row r="141" ht="22" customHeight="1">
       <x:c r="A141" s="17"/>
@@ -2975,8 +3261,10 @@
       <x:c r="L141" s="14"/>
       <x:c r="M141" s="14"/>
       <x:c r="N141" s="17"/>
-      <x:c r="O141" s="14"/>
-      <x:c r="P141" s="14"/>
+      <x:c r="O141" s="17"/>
+      <x:c r="P141" s="17"/>
+      <x:c r="Q141" s="14"/>
+      <x:c r="R141" s="14"/>
     </x:row>
     <x:row r="142" ht="22" customHeight="1">
       <x:c r="A142" s="17"/>
@@ -2993,8 +3281,10 @@
       <x:c r="L142" s="14"/>
       <x:c r="M142" s="14"/>
       <x:c r="N142" s="17"/>
-      <x:c r="O142" s="14"/>
-      <x:c r="P142" s="14"/>
+      <x:c r="O142" s="17"/>
+      <x:c r="P142" s="17"/>
+      <x:c r="Q142" s="14"/>
+      <x:c r="R142" s="14"/>
     </x:row>
     <x:row r="143" ht="22" customHeight="1">
       <x:c r="A143" s="17"/>
@@ -3011,8 +3301,10 @@
       <x:c r="L143" s="14"/>
       <x:c r="M143" s="14"/>
       <x:c r="N143" s="17"/>
-      <x:c r="O143" s="14"/>
-      <x:c r="P143" s="14"/>
+      <x:c r="O143" s="17"/>
+      <x:c r="P143" s="17"/>
+      <x:c r="Q143" s="14"/>
+      <x:c r="R143" s="14"/>
     </x:row>
     <x:row r="144" ht="22" customHeight="1">
       <x:c r="A144" s="17"/>
@@ -3029,8 +3321,10 @@
       <x:c r="L144" s="14"/>
       <x:c r="M144" s="14"/>
       <x:c r="N144" s="17"/>
-      <x:c r="O144" s="14"/>
-      <x:c r="P144" s="14"/>
+      <x:c r="O144" s="17"/>
+      <x:c r="P144" s="17"/>
+      <x:c r="Q144" s="14"/>
+      <x:c r="R144" s="14"/>
     </x:row>
     <x:row r="145" ht="22" customHeight="1">
       <x:c r="A145" s="17"/>
@@ -3047,8 +3341,10 @@
       <x:c r="L145" s="14"/>
       <x:c r="M145" s="14"/>
       <x:c r="N145" s="17"/>
-      <x:c r="O145" s="14"/>
-      <x:c r="P145" s="14"/>
+      <x:c r="O145" s="17"/>
+      <x:c r="P145" s="17"/>
+      <x:c r="Q145" s="14"/>
+      <x:c r="R145" s="14"/>
     </x:row>
     <x:row r="146" ht="22" customHeight="1">
       <x:c r="A146" s="17"/>
@@ -3065,8 +3361,10 @@
       <x:c r="L146" s="14"/>
       <x:c r="M146" s="14"/>
       <x:c r="N146" s="17"/>
-      <x:c r="O146" s="14"/>
-      <x:c r="P146" s="14"/>
+      <x:c r="O146" s="17"/>
+      <x:c r="P146" s="17"/>
+      <x:c r="Q146" s="14"/>
+      <x:c r="R146" s="14"/>
     </x:row>
     <x:row r="147" ht="22" customHeight="1">
       <x:c r="A147" s="17"/>
@@ -3083,8 +3381,10 @@
       <x:c r="L147" s="14"/>
       <x:c r="M147" s="14"/>
       <x:c r="N147" s="17"/>
-      <x:c r="O147" s="14"/>
-      <x:c r="P147" s="14"/>
+      <x:c r="O147" s="17"/>
+      <x:c r="P147" s="17"/>
+      <x:c r="Q147" s="14"/>
+      <x:c r="R147" s="14"/>
     </x:row>
     <x:row r="148" ht="22" customHeight="1">
       <x:c r="A148" s="17"/>
@@ -3101,8 +3401,10 @@
       <x:c r="L148" s="14"/>
       <x:c r="M148" s="14"/>
       <x:c r="N148" s="17"/>
-      <x:c r="O148" s="14"/>
-      <x:c r="P148" s="14"/>
+      <x:c r="O148" s="17"/>
+      <x:c r="P148" s="17"/>
+      <x:c r="Q148" s="14"/>
+      <x:c r="R148" s="14"/>
     </x:row>
     <x:row r="149" ht="22" customHeight="1">
       <x:c r="A149" s="17"/>
@@ -3119,8 +3421,10 @@
       <x:c r="L149" s="14"/>
       <x:c r="M149" s="14"/>
       <x:c r="N149" s="17"/>
-      <x:c r="O149" s="14"/>
-      <x:c r="P149" s="14"/>
+      <x:c r="O149" s="17"/>
+      <x:c r="P149" s="17"/>
+      <x:c r="Q149" s="14"/>
+      <x:c r="R149" s="14"/>
     </x:row>
     <x:row r="150" ht="22" customHeight="1">
       <x:c r="A150" s="17"/>
@@ -3137,8 +3441,10 @@
       <x:c r="L150" s="14"/>
       <x:c r="M150" s="14"/>
       <x:c r="N150" s="17"/>
-      <x:c r="O150" s="14"/>
-      <x:c r="P150" s="14"/>
+      <x:c r="O150" s="17"/>
+      <x:c r="P150" s="17"/>
+      <x:c r="Q150" s="14"/>
+      <x:c r="R150" s="14"/>
     </x:row>
     <x:row r="151" ht="22" customHeight="1">
       <x:c r="A151" s="17"/>
@@ -3155,8 +3461,10 @@
       <x:c r="L151" s="14"/>
       <x:c r="M151" s="14"/>
       <x:c r="N151" s="17"/>
-      <x:c r="O151" s="14"/>
-      <x:c r="P151" s="14"/>
+      <x:c r="O151" s="17"/>
+      <x:c r="P151" s="17"/>
+      <x:c r="Q151" s="14"/>
+      <x:c r="R151" s="14"/>
     </x:row>
     <x:row r="152" ht="22" customHeight="1">
       <x:c r="A152" s="17"/>
@@ -3173,8 +3481,10 @@
       <x:c r="L152" s="14"/>
       <x:c r="M152" s="14"/>
       <x:c r="N152" s="17"/>
-      <x:c r="O152" s="14"/>
-      <x:c r="P152" s="14"/>
+      <x:c r="O152" s="17"/>
+      <x:c r="P152" s="17"/>
+      <x:c r="Q152" s="14"/>
+      <x:c r="R152" s="14"/>
     </x:row>
     <x:row r="153" ht="22" customHeight="1">
       <x:c r="A153" s="17"/>
@@ -3191,8 +3501,10 @@
       <x:c r="L153" s="14"/>
       <x:c r="M153" s="14"/>
       <x:c r="N153" s="17"/>
-      <x:c r="O153" s="14"/>
-      <x:c r="P153" s="14"/>
+      <x:c r="O153" s="17"/>
+      <x:c r="P153" s="17"/>
+      <x:c r="Q153" s="14"/>
+      <x:c r="R153" s="14"/>
     </x:row>
     <x:row r="154" ht="22" customHeight="1">
       <x:c r="A154" s="17"/>
@@ -3209,8 +3521,10 @@
       <x:c r="L154" s="14"/>
       <x:c r="M154" s="14"/>
       <x:c r="N154" s="17"/>
-      <x:c r="O154" s="14"/>
-      <x:c r="P154" s="14"/>
+      <x:c r="O154" s="17"/>
+      <x:c r="P154" s="17"/>
+      <x:c r="Q154" s="14"/>
+      <x:c r="R154" s="14"/>
     </x:row>
     <x:row r="155" ht="22" customHeight="1">
       <x:c r="A155" s="17"/>
@@ -3227,8 +3541,10 @@
       <x:c r="L155" s="14"/>
       <x:c r="M155" s="14"/>
       <x:c r="N155" s="17"/>
-      <x:c r="O155" s="14"/>
-      <x:c r="P155" s="14"/>
+      <x:c r="O155" s="17"/>
+      <x:c r="P155" s="17"/>
+      <x:c r="Q155" s="14"/>
+      <x:c r="R155" s="14"/>
     </x:row>
     <x:row r="156" ht="22" customHeight="1">
       <x:c r="A156" s="17"/>
@@ -3245,8 +3561,10 @@
       <x:c r="L156" s="14"/>
       <x:c r="M156" s="14"/>
       <x:c r="N156" s="17"/>
-      <x:c r="O156" s="14"/>
-      <x:c r="P156" s="14"/>
+      <x:c r="O156" s="17"/>
+      <x:c r="P156" s="17"/>
+      <x:c r="Q156" s="14"/>
+      <x:c r="R156" s="14"/>
     </x:row>
     <x:row r="157" ht="22" customHeight="1">
       <x:c r="A157" s="17"/>
@@ -3263,8 +3581,10 @@
       <x:c r="L157" s="14"/>
       <x:c r="M157" s="14"/>
       <x:c r="N157" s="17"/>
-      <x:c r="O157" s="14"/>
-      <x:c r="P157" s="14"/>
+      <x:c r="O157" s="17"/>
+      <x:c r="P157" s="17"/>
+      <x:c r="Q157" s="14"/>
+      <x:c r="R157" s="14"/>
     </x:row>
     <x:row r="158" ht="22" customHeight="1">
       <x:c r="A158" s="17"/>
@@ -3281,8 +3601,10 @@
       <x:c r="L158" s="14"/>
       <x:c r="M158" s="14"/>
       <x:c r="N158" s="17"/>
-      <x:c r="O158" s="14"/>
-      <x:c r="P158" s="14"/>
+      <x:c r="O158" s="17"/>
+      <x:c r="P158" s="17"/>
+      <x:c r="Q158" s="14"/>
+      <x:c r="R158" s="14"/>
     </x:row>
     <x:row r="159" ht="22" customHeight="1">
       <x:c r="A159" s="17"/>
@@ -3299,8 +3621,10 @@
       <x:c r="L159" s="14"/>
       <x:c r="M159" s="14"/>
       <x:c r="N159" s="17"/>
-      <x:c r="O159" s="14"/>
-      <x:c r="P159" s="14"/>
+      <x:c r="O159" s="17"/>
+      <x:c r="P159" s="17"/>
+      <x:c r="Q159" s="14"/>
+      <x:c r="R159" s="14"/>
     </x:row>
     <x:row r="160" ht="22" customHeight="1">
       <x:c r="A160" s="17"/>
@@ -3317,8 +3641,10 @@
       <x:c r="L160" s="14"/>
       <x:c r="M160" s="14"/>
       <x:c r="N160" s="17"/>
-      <x:c r="O160" s="14"/>
-      <x:c r="P160" s="14"/>
+      <x:c r="O160" s="17"/>
+      <x:c r="P160" s="17"/>
+      <x:c r="Q160" s="14"/>
+      <x:c r="R160" s="14"/>
     </x:row>
     <x:row r="161" ht="22" customHeight="1">
       <x:c r="A161" s="17"/>
@@ -3335,8 +3661,10 @@
       <x:c r="L161" s="14"/>
       <x:c r="M161" s="14"/>
       <x:c r="N161" s="17"/>
-      <x:c r="O161" s="14"/>
-      <x:c r="P161" s="14"/>
+      <x:c r="O161" s="17"/>
+      <x:c r="P161" s="17"/>
+      <x:c r="Q161" s="14"/>
+      <x:c r="R161" s="14"/>
     </x:row>
     <x:row r="162" ht="22" customHeight="1">
       <x:c r="A162" s="17"/>
@@ -3353,8 +3681,10 @@
       <x:c r="L162" s="14"/>
       <x:c r="M162" s="14"/>
       <x:c r="N162" s="17"/>
-      <x:c r="O162" s="14"/>
-      <x:c r="P162" s="14"/>
+      <x:c r="O162" s="17"/>
+      <x:c r="P162" s="17"/>
+      <x:c r="Q162" s="14"/>
+      <x:c r="R162" s="14"/>
     </x:row>
     <x:row r="163" ht="22" customHeight="1">
       <x:c r="A163" s="17"/>
@@ -3371,8 +3701,10 @@
       <x:c r="L163" s="14"/>
       <x:c r="M163" s="14"/>
       <x:c r="N163" s="17"/>
-      <x:c r="O163" s="14"/>
-      <x:c r="P163" s="14"/>
+      <x:c r="O163" s="17"/>
+      <x:c r="P163" s="17"/>
+      <x:c r="Q163" s="14"/>
+      <x:c r="R163" s="14"/>
     </x:row>
     <x:row r="164" ht="22" customHeight="1">
       <x:c r="A164" s="17"/>
@@ -3389,8 +3721,10 @@
       <x:c r="L164" s="14"/>
       <x:c r="M164" s="14"/>
       <x:c r="N164" s="17"/>
-      <x:c r="O164" s="14"/>
-      <x:c r="P164" s="14"/>
+      <x:c r="O164" s="17"/>
+      <x:c r="P164" s="17"/>
+      <x:c r="Q164" s="14"/>
+      <x:c r="R164" s="14"/>
     </x:row>
     <x:row r="165" ht="22" customHeight="1">
       <x:c r="A165" s="17"/>
@@ -3407,8 +3741,10 @@
       <x:c r="L165" s="14"/>
       <x:c r="M165" s="14"/>
       <x:c r="N165" s="17"/>
-      <x:c r="O165" s="14"/>
-      <x:c r="P165" s="14"/>
+      <x:c r="O165" s="17"/>
+      <x:c r="P165" s="17"/>
+      <x:c r="Q165" s="14"/>
+      <x:c r="R165" s="14"/>
     </x:row>
     <x:row r="166" ht="22" customHeight="1">
       <x:c r="A166" s="17"/>
@@ -3425,8 +3761,10 @@
       <x:c r="L166" s="14"/>
       <x:c r="M166" s="14"/>
       <x:c r="N166" s="17"/>
-      <x:c r="O166" s="14"/>
-      <x:c r="P166" s="14"/>
+      <x:c r="O166" s="17"/>
+      <x:c r="P166" s="17"/>
+      <x:c r="Q166" s="14"/>
+      <x:c r="R166" s="14"/>
     </x:row>
     <x:row r="167" ht="22" customHeight="1">
       <x:c r="A167" s="17"/>
@@ -3443,8 +3781,10 @@
       <x:c r="L167" s="14"/>
       <x:c r="M167" s="14"/>
       <x:c r="N167" s="17"/>
-      <x:c r="O167" s="14"/>
-      <x:c r="P167" s="14"/>
+      <x:c r="O167" s="17"/>
+      <x:c r="P167" s="17"/>
+      <x:c r="Q167" s="14"/>
+      <x:c r="R167" s="14"/>
     </x:row>
     <x:row r="168" ht="22" customHeight="1">
       <x:c r="A168" s="17"/>
@@ -3461,8 +3801,10 @@
       <x:c r="L168" s="14"/>
       <x:c r="M168" s="14"/>
       <x:c r="N168" s="17"/>
-      <x:c r="O168" s="14"/>
-      <x:c r="P168" s="14"/>
+      <x:c r="O168" s="17"/>
+      <x:c r="P168" s="17"/>
+      <x:c r="Q168" s="14"/>
+      <x:c r="R168" s="14"/>
     </x:row>
     <x:row r="169" ht="22" customHeight="1">
       <x:c r="A169" s="17"/>
@@ -3479,8 +3821,10 @@
       <x:c r="L169" s="14"/>
       <x:c r="M169" s="14"/>
       <x:c r="N169" s="17"/>
-      <x:c r="O169" s="14"/>
-      <x:c r="P169" s="14"/>
+      <x:c r="O169" s="17"/>
+      <x:c r="P169" s="17"/>
+      <x:c r="Q169" s="14"/>
+      <x:c r="R169" s="14"/>
     </x:row>
     <x:row r="170" ht="22" customHeight="1">
       <x:c r="A170" s="17"/>
@@ -3497,8 +3841,10 @@
       <x:c r="L170" s="14"/>
       <x:c r="M170" s="14"/>
       <x:c r="N170" s="17"/>
-      <x:c r="O170" s="14"/>
-      <x:c r="P170" s="14"/>
+      <x:c r="O170" s="17"/>
+      <x:c r="P170" s="17"/>
+      <x:c r="Q170" s="14"/>
+      <x:c r="R170" s="14"/>
     </x:row>
     <x:row r="171" ht="22" customHeight="1">
       <x:c r="A171" s="17"/>
@@ -3515,8 +3861,10 @@
       <x:c r="L171" s="14"/>
       <x:c r="M171" s="14"/>
       <x:c r="N171" s="17"/>
-      <x:c r="O171" s="14"/>
-      <x:c r="P171" s="14"/>
+      <x:c r="O171" s="17"/>
+      <x:c r="P171" s="17"/>
+      <x:c r="Q171" s="14"/>
+      <x:c r="R171" s="14"/>
     </x:row>
     <x:row r="172" ht="22" customHeight="1">
       <x:c r="A172" s="17"/>
@@ -3533,8 +3881,10 @@
       <x:c r="L172" s="14"/>
       <x:c r="M172" s="14"/>
       <x:c r="N172" s="17"/>
-      <x:c r="O172" s="14"/>
-      <x:c r="P172" s="14"/>
+      <x:c r="O172" s="17"/>
+      <x:c r="P172" s="17"/>
+      <x:c r="Q172" s="14"/>
+      <x:c r="R172" s="14"/>
     </x:row>
     <x:row r="173" ht="22" customHeight="1">
       <x:c r="A173" s="17"/>
@@ -3551,8 +3901,10 @@
       <x:c r="L173" s="14"/>
       <x:c r="M173" s="14"/>
       <x:c r="N173" s="17"/>
-      <x:c r="O173" s="14"/>
-      <x:c r="P173" s="14"/>
+      <x:c r="O173" s="17"/>
+      <x:c r="P173" s="17"/>
+      <x:c r="Q173" s="14"/>
+      <x:c r="R173" s="14"/>
     </x:row>
     <x:row r="174" ht="22" customHeight="1">
       <x:c r="A174" s="17"/>
@@ -3569,8 +3921,10 @@
       <x:c r="L174" s="14"/>
       <x:c r="M174" s="14"/>
       <x:c r="N174" s="17"/>
-      <x:c r="O174" s="14"/>
-      <x:c r="P174" s="14"/>
+      <x:c r="O174" s="17"/>
+      <x:c r="P174" s="17"/>
+      <x:c r="Q174" s="14"/>
+      <x:c r="R174" s="14"/>
     </x:row>
     <x:row r="175" ht="22" customHeight="1">
       <x:c r="A175" s="17"/>
@@ -3587,8 +3941,10 @@
       <x:c r="L175" s="14"/>
       <x:c r="M175" s="14"/>
       <x:c r="N175" s="17"/>
-      <x:c r="O175" s="14"/>
-      <x:c r="P175" s="14"/>
+      <x:c r="O175" s="17"/>
+      <x:c r="P175" s="17"/>
+      <x:c r="Q175" s="14"/>
+      <x:c r="R175" s="14"/>
     </x:row>
     <x:row r="176" ht="22" customHeight="1">
       <x:c r="A176" s="17"/>
@@ -3605,8 +3961,10 @@
       <x:c r="L176" s="14"/>
       <x:c r="M176" s="14"/>
       <x:c r="N176" s="17"/>
-      <x:c r="O176" s="14"/>
-      <x:c r="P176" s="14"/>
+      <x:c r="O176" s="17"/>
+      <x:c r="P176" s="17"/>
+      <x:c r="Q176" s="14"/>
+      <x:c r="R176" s="14"/>
     </x:row>
     <x:row r="177" ht="22" customHeight="1">
       <x:c r="A177" s="17"/>
@@ -3623,8 +3981,10 @@
       <x:c r="L177" s="14"/>
       <x:c r="M177" s="14"/>
       <x:c r="N177" s="17"/>
-      <x:c r="O177" s="14"/>
-      <x:c r="P177" s="14"/>
+      <x:c r="O177" s="17"/>
+      <x:c r="P177" s="17"/>
+      <x:c r="Q177" s="14"/>
+      <x:c r="R177" s="14"/>
     </x:row>
     <x:row r="178" ht="22" customHeight="1">
       <x:c r="A178" s="17"/>
@@ -3641,8 +4001,10 @@
       <x:c r="L178" s="14"/>
       <x:c r="M178" s="14"/>
       <x:c r="N178" s="17"/>
-      <x:c r="O178" s="14"/>
-      <x:c r="P178" s="14"/>
+      <x:c r="O178" s="17"/>
+      <x:c r="P178" s="17"/>
+      <x:c r="Q178" s="14"/>
+      <x:c r="R178" s="14"/>
     </x:row>
     <x:row r="179" ht="22" customHeight="1">
       <x:c r="A179" s="17"/>
@@ -3659,8 +4021,10 @@
       <x:c r="L179" s="14"/>
       <x:c r="M179" s="14"/>
       <x:c r="N179" s="17"/>
-      <x:c r="O179" s="14"/>
-      <x:c r="P179" s="14"/>
+      <x:c r="O179" s="17"/>
+      <x:c r="P179" s="17"/>
+      <x:c r="Q179" s="14"/>
+      <x:c r="R179" s="14"/>
     </x:row>
     <x:row r="180" ht="22" customHeight="1">
       <x:c r="A180" s="17"/>
@@ -3677,8 +4041,10 @@
       <x:c r="L180" s="14"/>
       <x:c r="M180" s="14"/>
       <x:c r="N180" s="17"/>
-      <x:c r="O180" s="14"/>
-      <x:c r="P180" s="14"/>
+      <x:c r="O180" s="17"/>
+      <x:c r="P180" s="17"/>
+      <x:c r="Q180" s="14"/>
+      <x:c r="R180" s="14"/>
     </x:row>
     <x:row r="181" ht="22" customHeight="1">
       <x:c r="A181" s="17"/>
@@ -3695,8 +4061,10 @@
       <x:c r="L181" s="14"/>
       <x:c r="M181" s="14"/>
       <x:c r="N181" s="17"/>
-      <x:c r="O181" s="14"/>
-      <x:c r="P181" s="14"/>
+      <x:c r="O181" s="17"/>
+      <x:c r="P181" s="17"/>
+      <x:c r="Q181" s="14"/>
+      <x:c r="R181" s="14"/>
     </x:row>
     <x:row r="182" ht="22" customHeight="1">
       <x:c r="A182" s="17"/>
@@ -3713,8 +4081,10 @@
       <x:c r="L182" s="14"/>
       <x:c r="M182" s="14"/>
       <x:c r="N182" s="17"/>
-      <x:c r="O182" s="14"/>
-      <x:c r="P182" s="14"/>
+      <x:c r="O182" s="17"/>
+      <x:c r="P182" s="17"/>
+      <x:c r="Q182" s="14"/>
+      <x:c r="R182" s="14"/>
     </x:row>
     <x:row r="183" ht="22" customHeight="1">
       <x:c r="A183" s="17"/>
@@ -3731,8 +4101,10 @@
       <x:c r="L183" s="14"/>
       <x:c r="M183" s="14"/>
       <x:c r="N183" s="17"/>
-      <x:c r="O183" s="14"/>
-      <x:c r="P183" s="14"/>
+      <x:c r="O183" s="17"/>
+      <x:c r="P183" s="17"/>
+      <x:c r="Q183" s="14"/>
+      <x:c r="R183" s="14"/>
     </x:row>
     <x:row r="184" ht="22" customHeight="1">
       <x:c r="A184" s="17"/>
@@ -3749,8 +4121,10 @@
       <x:c r="L184" s="14"/>
       <x:c r="M184" s="14"/>
       <x:c r="N184" s="17"/>
-      <x:c r="O184" s="14"/>
-      <x:c r="P184" s="14"/>
+      <x:c r="O184" s="17"/>
+      <x:c r="P184" s="17"/>
+      <x:c r="Q184" s="14"/>
+      <x:c r="R184" s="14"/>
     </x:row>
     <x:row r="185" ht="22" customHeight="1">
       <x:c r="A185" s="17"/>
@@ -3767,8 +4141,10 @@
       <x:c r="L185" s="14"/>
       <x:c r="M185" s="14"/>
       <x:c r="N185" s="17"/>
-      <x:c r="O185" s="14"/>
-      <x:c r="P185" s="14"/>
+      <x:c r="O185" s="17"/>
+      <x:c r="P185" s="17"/>
+      <x:c r="Q185" s="14"/>
+      <x:c r="R185" s="14"/>
     </x:row>
     <x:row r="186" ht="22" customHeight="1">
       <x:c r="A186" s="17"/>
@@ -3785,8 +4161,10 @@
       <x:c r="L186" s="14"/>
       <x:c r="M186" s="14"/>
       <x:c r="N186" s="17"/>
-      <x:c r="O186" s="14"/>
-      <x:c r="P186" s="14"/>
+      <x:c r="O186" s="17"/>
+      <x:c r="P186" s="17"/>
+      <x:c r="Q186" s="14"/>
+      <x:c r="R186" s="14"/>
     </x:row>
     <x:row r="187" ht="22" customHeight="1">
       <x:c r="A187" s="17"/>
@@ -3803,8 +4181,10 @@
       <x:c r="L187" s="14"/>
       <x:c r="M187" s="14"/>
       <x:c r="N187" s="17"/>
-      <x:c r="O187" s="14"/>
-      <x:c r="P187" s="14"/>
+      <x:c r="O187" s="17"/>
+      <x:c r="P187" s="17"/>
+      <x:c r="Q187" s="14"/>
+      <x:c r="R187" s="14"/>
     </x:row>
     <x:row r="188" ht="22" customHeight="1">
       <x:c r="A188" s="17"/>
@@ -3821,8 +4201,10 @@
       <x:c r="L188" s="14"/>
       <x:c r="M188" s="14"/>
       <x:c r="N188" s="17"/>
-      <x:c r="O188" s="14"/>
-      <x:c r="P188" s="14"/>
+      <x:c r="O188" s="17"/>
+      <x:c r="P188" s="17"/>
+      <x:c r="Q188" s="14"/>
+      <x:c r="R188" s="14"/>
     </x:row>
     <x:row r="189" ht="22" customHeight="1">
       <x:c r="A189" s="17"/>
@@ -3839,8 +4221,10 @@
       <x:c r="L189" s="14"/>
       <x:c r="M189" s="14"/>
       <x:c r="N189" s="17"/>
-      <x:c r="O189" s="14"/>
-      <x:c r="P189" s="14"/>
+      <x:c r="O189" s="17"/>
+      <x:c r="P189" s="17"/>
+      <x:c r="Q189" s="14"/>
+      <x:c r="R189" s="14"/>
     </x:row>
     <x:row r="190" ht="22" customHeight="1">
       <x:c r="A190" s="17"/>
@@ -3857,8 +4241,10 @@
       <x:c r="L190" s="14"/>
       <x:c r="M190" s="14"/>
       <x:c r="N190" s="17"/>
-      <x:c r="O190" s="14"/>
-      <x:c r="P190" s="14"/>
+      <x:c r="O190" s="17"/>
+      <x:c r="P190" s="17"/>
+      <x:c r="Q190" s="14"/>
+      <x:c r="R190" s="14"/>
     </x:row>
     <x:row r="191" ht="22" customHeight="1">
       <x:c r="A191" s="17"/>
@@ -3875,8 +4261,10 @@
       <x:c r="L191" s="14"/>
       <x:c r="M191" s="14"/>
       <x:c r="N191" s="17"/>
-      <x:c r="O191" s="14"/>
-      <x:c r="P191" s="14"/>
+      <x:c r="O191" s="17"/>
+      <x:c r="P191" s="17"/>
+      <x:c r="Q191" s="14"/>
+      <x:c r="R191" s="14"/>
     </x:row>
     <x:row r="192" ht="22" customHeight="1">
       <x:c r="A192" s="17"/>
@@ -3893,8 +4281,10 @@
       <x:c r="L192" s="14"/>
       <x:c r="M192" s="14"/>
       <x:c r="N192" s="17"/>
-      <x:c r="O192" s="14"/>
-      <x:c r="P192" s="14"/>
+      <x:c r="O192" s="17"/>
+      <x:c r="P192" s="17"/>
+      <x:c r="Q192" s="14"/>
+      <x:c r="R192" s="14"/>
     </x:row>
     <x:row r="193" ht="22" customHeight="1">
       <x:c r="A193" s="17"/>
@@ -3911,8 +4301,10 @@
       <x:c r="L193" s="14"/>
       <x:c r="M193" s="14"/>
       <x:c r="N193" s="17"/>
-      <x:c r="O193" s="14"/>
-      <x:c r="P193" s="14"/>
+      <x:c r="O193" s="17"/>
+      <x:c r="P193" s="17"/>
+      <x:c r="Q193" s="14"/>
+      <x:c r="R193" s="14"/>
     </x:row>
     <x:row r="194" ht="22" customHeight="1">
       <x:c r="A194" s="17"/>
@@ -3929,8 +4321,10 @@
       <x:c r="L194" s="14"/>
       <x:c r="M194" s="14"/>
       <x:c r="N194" s="17"/>
-      <x:c r="O194" s="14"/>
-      <x:c r="P194" s="14"/>
+      <x:c r="O194" s="17"/>
+      <x:c r="P194" s="17"/>
+      <x:c r="Q194" s="14"/>
+      <x:c r="R194" s="14"/>
     </x:row>
     <x:row r="195" ht="22" customHeight="1">
       <x:c r="A195" s="17"/>
@@ -3947,8 +4341,10 @@
       <x:c r="L195" s="14"/>
       <x:c r="M195" s="14"/>
       <x:c r="N195" s="17"/>
-      <x:c r="O195" s="14"/>
-      <x:c r="P195" s="14"/>
+      <x:c r="O195" s="17"/>
+      <x:c r="P195" s="17"/>
+      <x:c r="Q195" s="14"/>
+      <x:c r="R195" s="14"/>
     </x:row>
     <x:row r="196" ht="22" customHeight="1">
       <x:c r="A196" s="17"/>
@@ -3965,8 +4361,10 @@
       <x:c r="L196" s="14"/>
       <x:c r="M196" s="14"/>
       <x:c r="N196" s="17"/>
-      <x:c r="O196" s="14"/>
-      <x:c r="P196" s="14"/>
+      <x:c r="O196" s="17"/>
+      <x:c r="P196" s="17"/>
+      <x:c r="Q196" s="14"/>
+      <x:c r="R196" s="14"/>
     </x:row>
     <x:row r="197" ht="22" customHeight="1">
       <x:c r="A197" s="17"/>
@@ -3983,8 +4381,10 @@
       <x:c r="L197" s="14"/>
       <x:c r="M197" s="14"/>
       <x:c r="N197" s="17"/>
-      <x:c r="O197" s="14"/>
-      <x:c r="P197" s="14"/>
+      <x:c r="O197" s="17"/>
+      <x:c r="P197" s="17"/>
+      <x:c r="Q197" s="14"/>
+      <x:c r="R197" s="14"/>
     </x:row>
     <x:row r="198" ht="22" customHeight="1">
       <x:c r="A198" s="17"/>
@@ -4001,8 +4401,10 @@
       <x:c r="L198" s="14"/>
       <x:c r="M198" s="14"/>
       <x:c r="N198" s="17"/>
-      <x:c r="O198" s="14"/>
-      <x:c r="P198" s="14"/>
+      <x:c r="O198" s="17"/>
+      <x:c r="P198" s="17"/>
+      <x:c r="Q198" s="14"/>
+      <x:c r="R198" s="14"/>
     </x:row>
     <x:row r="199" ht="22" customHeight="1">
       <x:c r="A199" s="17"/>
@@ -4019,8 +4421,10 @@
       <x:c r="L199" s="14"/>
       <x:c r="M199" s="14"/>
       <x:c r="N199" s="17"/>
-      <x:c r="O199" s="14"/>
-      <x:c r="P199" s="14"/>
+      <x:c r="O199" s="17"/>
+      <x:c r="P199" s="17"/>
+      <x:c r="Q199" s="14"/>
+      <x:c r="R199" s="14"/>
     </x:row>
     <x:row r="200" ht="22" customHeight="1">
       <x:c r="A200" s="17"/>
@@ -4037,8 +4441,10 @@
       <x:c r="L200" s="14"/>
       <x:c r="M200" s="14"/>
       <x:c r="N200" s="17"/>
-      <x:c r="O200" s="14"/>
-      <x:c r="P200" s="14"/>
+      <x:c r="O200" s="17"/>
+      <x:c r="P200" s="17"/>
+      <x:c r="Q200" s="14"/>
+      <x:c r="R200" s="14"/>
     </x:row>
     <x:row r="201" ht="22" customHeight="1">
       <x:c r="A201" s="17"/>
@@ -4055,8 +4461,10 @@
       <x:c r="L201" s="14"/>
       <x:c r="M201" s="14"/>
       <x:c r="N201" s="17"/>
-      <x:c r="O201" s="14"/>
-      <x:c r="P201" s="14"/>
+      <x:c r="O201" s="17"/>
+      <x:c r="P201" s="17"/>
+      <x:c r="Q201" s="14"/>
+      <x:c r="R201" s="14"/>
     </x:row>
     <x:row r="202" ht="22" customHeight="1">
       <x:c r="A202" s="17"/>
@@ -4073,8 +4481,10 @@
       <x:c r="L202" s="14"/>
       <x:c r="M202" s="14"/>
       <x:c r="N202" s="17"/>
-      <x:c r="O202" s="14"/>
-      <x:c r="P202" s="14"/>
+      <x:c r="O202" s="17"/>
+      <x:c r="P202" s="17"/>
+      <x:c r="Q202" s="14"/>
+      <x:c r="R202" s="14"/>
     </x:row>
     <x:row r="203" ht="22" customHeight="1">
       <x:c r="A203" s="17"/>
@@ -4091,8 +4501,10 @@
       <x:c r="L203" s="14"/>
       <x:c r="M203" s="14"/>
       <x:c r="N203" s="17"/>
-      <x:c r="O203" s="14"/>
-      <x:c r="P203" s="14"/>
+      <x:c r="O203" s="17"/>
+      <x:c r="P203" s="17"/>
+      <x:c r="Q203" s="14"/>
+      <x:c r="R203" s="14"/>
     </x:row>
     <x:row r="204" ht="22" customHeight="1">
       <x:c r="A204" s="17"/>
@@ -4109,8 +4521,10 @@
       <x:c r="L204" s="14"/>
       <x:c r="M204" s="14"/>
       <x:c r="N204" s="17"/>
-      <x:c r="O204" s="14"/>
-      <x:c r="P204" s="14"/>
+      <x:c r="O204" s="17"/>
+      <x:c r="P204" s="17"/>
+      <x:c r="Q204" s="14"/>
+      <x:c r="R204" s="14"/>
     </x:row>
     <x:row r="205" ht="22" customHeight="1">
       <x:c r="A205" s="17"/>
@@ -4127,8 +4541,10 @@
       <x:c r="L205" s="14"/>
       <x:c r="M205" s="14"/>
       <x:c r="N205" s="17"/>
-      <x:c r="O205" s="14"/>
-      <x:c r="P205" s="14"/>
+      <x:c r="O205" s="17"/>
+      <x:c r="P205" s="17"/>
+      <x:c r="Q205" s="14"/>
+      <x:c r="R205" s="14"/>
     </x:row>
     <x:row r="206" ht="22" customHeight="1">
       <x:c r="A206" s="17"/>
@@ -4145,8 +4561,10 @@
       <x:c r="L206" s="14"/>
       <x:c r="M206" s="14"/>
       <x:c r="N206" s="17"/>
-      <x:c r="O206" s="14"/>
-      <x:c r="P206" s="14"/>
+      <x:c r="O206" s="17"/>
+      <x:c r="P206" s="17"/>
+      <x:c r="Q206" s="14"/>
+      <x:c r="R206" s="14"/>
     </x:row>
     <x:row r="207" ht="22" customHeight="1">
       <x:c r="A207" s="17"/>
@@ -4163,8 +4581,10 @@
       <x:c r="L207" s="14"/>
       <x:c r="M207" s="14"/>
       <x:c r="N207" s="17"/>
-      <x:c r="O207" s="14"/>
-      <x:c r="P207" s="14"/>
+      <x:c r="O207" s="17"/>
+      <x:c r="P207" s="17"/>
+      <x:c r="Q207" s="14"/>
+      <x:c r="R207" s="14"/>
     </x:row>
     <x:row r="208" ht="22" customHeight="1">
       <x:c r="A208" s="17"/>
@@ -4181,8 +4601,10 @@
       <x:c r="L208" s="14"/>
       <x:c r="M208" s="14"/>
       <x:c r="N208" s="17"/>
-      <x:c r="O208" s="14"/>
-      <x:c r="P208" s="14"/>
+      <x:c r="O208" s="17"/>
+      <x:c r="P208" s="17"/>
+      <x:c r="Q208" s="14"/>
+      <x:c r="R208" s="14"/>
     </x:row>
     <x:row r="209" ht="22" customHeight="1">
       <x:c r="A209" s="17"/>
@@ -4199,8 +4621,10 @@
       <x:c r="L209" s="14"/>
       <x:c r="M209" s="14"/>
       <x:c r="N209" s="17"/>
-      <x:c r="O209" s="14"/>
-      <x:c r="P209" s="14"/>
+      <x:c r="O209" s="17"/>
+      <x:c r="P209" s="17"/>
+      <x:c r="Q209" s="14"/>
+      <x:c r="R209" s="14"/>
     </x:row>
     <x:row r="210" ht="22" customHeight="1">
       <x:c r="A210" s="17"/>
@@ -4217,8 +4641,10 @@
       <x:c r="L210" s="14"/>
       <x:c r="M210" s="14"/>
       <x:c r="N210" s="17"/>
-      <x:c r="O210" s="14"/>
-      <x:c r="P210" s="14"/>
+      <x:c r="O210" s="17"/>
+      <x:c r="P210" s="17"/>
+      <x:c r="Q210" s="14"/>
+      <x:c r="R210" s="14"/>
     </x:row>
     <x:row r="211" ht="22" customHeight="1">
       <x:c r="A211" s="17"/>
@@ -4235,8 +4661,10 @@
       <x:c r="L211" s="14"/>
       <x:c r="M211" s="14"/>
       <x:c r="N211" s="17"/>
-      <x:c r="O211" s="14"/>
-      <x:c r="P211" s="14"/>
+      <x:c r="O211" s="17"/>
+      <x:c r="P211" s="17"/>
+      <x:c r="Q211" s="14"/>
+      <x:c r="R211" s="14"/>
     </x:row>
     <x:row r="212" ht="22" customHeight="1">
       <x:c r="A212" s="17"/>
@@ -4253,8 +4681,10 @@
       <x:c r="L212" s="14"/>
       <x:c r="M212" s="14"/>
       <x:c r="N212" s="17"/>
-      <x:c r="O212" s="14"/>
-      <x:c r="P212" s="14"/>
+      <x:c r="O212" s="17"/>
+      <x:c r="P212" s="17"/>
+      <x:c r="Q212" s="14"/>
+      <x:c r="R212" s="14"/>
     </x:row>
     <x:row r="213" ht="22" customHeight="1">
       <x:c r="A213" s="17"/>
@@ -4271,8 +4701,10 @@
       <x:c r="L213" s="14"/>
       <x:c r="M213" s="14"/>
       <x:c r="N213" s="17"/>
-      <x:c r="O213" s="14"/>
-      <x:c r="P213" s="14"/>
+      <x:c r="O213" s="17"/>
+      <x:c r="P213" s="17"/>
+      <x:c r="Q213" s="14"/>
+      <x:c r="R213" s="14"/>
     </x:row>
     <x:row r="214" ht="22" customHeight="1">
       <x:c r="A214" s="17"/>
@@ -4289,8 +4721,10 @@
       <x:c r="L214" s="14"/>
       <x:c r="M214" s="14"/>
       <x:c r="N214" s="17"/>
-      <x:c r="O214" s="14"/>
-      <x:c r="P214" s="14"/>
+      <x:c r="O214" s="17"/>
+      <x:c r="P214" s="17"/>
+      <x:c r="Q214" s="14"/>
+      <x:c r="R214" s="14"/>
     </x:row>
     <x:row r="215" ht="22" customHeight="1">
       <x:c r="A215" s="17"/>
@@ -4307,8 +4741,10 @@
       <x:c r="L215" s="14"/>
       <x:c r="M215" s="14"/>
       <x:c r="N215" s="17"/>
-      <x:c r="O215" s="14"/>
-      <x:c r="P215" s="14"/>
+      <x:c r="O215" s="17"/>
+      <x:c r="P215" s="17"/>
+      <x:c r="Q215" s="14"/>
+      <x:c r="R215" s="14"/>
     </x:row>
     <x:row r="216" ht="22" customHeight="1">
       <x:c r="A216" s="17"/>
@@ -4325,8 +4761,10 @@
       <x:c r="L216" s="14"/>
       <x:c r="M216" s="14"/>
       <x:c r="N216" s="17"/>
-      <x:c r="O216" s="14"/>
-      <x:c r="P216" s="14"/>
+      <x:c r="O216" s="17"/>
+      <x:c r="P216" s="17"/>
+      <x:c r="Q216" s="14"/>
+      <x:c r="R216" s="14"/>
     </x:row>
     <x:row r="217" ht="22" customHeight="1">
       <x:c r="A217" s="17"/>
@@ -4343,8 +4781,10 @@
       <x:c r="L217" s="14"/>
       <x:c r="M217" s="14"/>
       <x:c r="N217" s="17"/>
-      <x:c r="O217" s="14"/>
-      <x:c r="P217" s="14"/>
+      <x:c r="O217" s="17"/>
+      <x:c r="P217" s="17"/>
+      <x:c r="Q217" s="14"/>
+      <x:c r="R217" s="14"/>
     </x:row>
     <x:row r="218" ht="22" customHeight="1">
       <x:c r="A218" s="17"/>
@@ -4361,8 +4801,10 @@
       <x:c r="L218" s="14"/>
       <x:c r="M218" s="14"/>
       <x:c r="N218" s="17"/>
-      <x:c r="O218" s="14"/>
-      <x:c r="P218" s="14"/>
+      <x:c r="O218" s="17"/>
+      <x:c r="P218" s="17"/>
+      <x:c r="Q218" s="14"/>
+      <x:c r="R218" s="14"/>
     </x:row>
     <x:row r="219" ht="22" customHeight="1">
       <x:c r="A219" s="17"/>
@@ -4379,8 +4821,10 @@
       <x:c r="L219" s="14"/>
       <x:c r="M219" s="14"/>
       <x:c r="N219" s="17"/>
-      <x:c r="O219" s="14"/>
-      <x:c r="P219" s="14"/>
+      <x:c r="O219" s="17"/>
+      <x:c r="P219" s="17"/>
+      <x:c r="Q219" s="14"/>
+      <x:c r="R219" s="14"/>
     </x:row>
     <x:row r="220" ht="22" customHeight="1">
       <x:c r="A220" s="17"/>
@@ -4397,8 +4841,10 @@
       <x:c r="L220" s="14"/>
       <x:c r="M220" s="14"/>
       <x:c r="N220" s="17"/>
-      <x:c r="O220" s="14"/>
-      <x:c r="P220" s="14"/>
+      <x:c r="O220" s="17"/>
+      <x:c r="P220" s="17"/>
+      <x:c r="Q220" s="14"/>
+      <x:c r="R220" s="14"/>
     </x:row>
     <x:row r="221" ht="22" customHeight="1">
       <x:c r="A221" s="17"/>
@@ -4415,8 +4861,10 @@
       <x:c r="L221" s="14"/>
       <x:c r="M221" s="14"/>
       <x:c r="N221" s="17"/>
-      <x:c r="O221" s="14"/>
-      <x:c r="P221" s="14"/>
+      <x:c r="O221" s="17"/>
+      <x:c r="P221" s="17"/>
+      <x:c r="Q221" s="14"/>
+      <x:c r="R221" s="14"/>
     </x:row>
     <x:row r="222" ht="22" customHeight="1">
       <x:c r="A222" s="17"/>
@@ -4433,8 +4881,10 @@
       <x:c r="L222" s="14"/>
       <x:c r="M222" s="14"/>
       <x:c r="N222" s="17"/>
-      <x:c r="O222" s="14"/>
-      <x:c r="P222" s="14"/>
+      <x:c r="O222" s="17"/>
+      <x:c r="P222" s="17"/>
+      <x:c r="Q222" s="14"/>
+      <x:c r="R222" s="14"/>
     </x:row>
     <x:row r="223" ht="22" customHeight="1">
       <x:c r="A223" s="17"/>
@@ -4451,8 +4901,10 @@
       <x:c r="L223" s="14"/>
       <x:c r="M223" s="14"/>
       <x:c r="N223" s="17"/>
-      <x:c r="O223" s="14"/>
-      <x:c r="P223" s="14"/>
+      <x:c r="O223" s="17"/>
+      <x:c r="P223" s="17"/>
+      <x:c r="Q223" s="14"/>
+      <x:c r="R223" s="14"/>
     </x:row>
     <x:row r="224" ht="22" customHeight="1">
       <x:c r="A224" s="17"/>
@@ -4469,8 +4921,10 @@
       <x:c r="L224" s="14"/>
       <x:c r="M224" s="14"/>
       <x:c r="N224" s="17"/>
-      <x:c r="O224" s="14"/>
-      <x:c r="P224" s="14"/>
+      <x:c r="O224" s="17"/>
+      <x:c r="P224" s="17"/>
+      <x:c r="Q224" s="14"/>
+      <x:c r="R224" s="14"/>
     </x:row>
     <x:row r="225" ht="22" customHeight="1">
       <x:c r="A225" s="17"/>
@@ -4487,8 +4941,10 @@
       <x:c r="L225" s="14"/>
       <x:c r="M225" s="14"/>
       <x:c r="N225" s="17"/>
-      <x:c r="O225" s="14"/>
-      <x:c r="P225" s="14"/>
+      <x:c r="O225" s="17"/>
+      <x:c r="P225" s="17"/>
+      <x:c r="Q225" s="14"/>
+      <x:c r="R225" s="14"/>
     </x:row>
     <x:row r="226" ht="22" customHeight="1">
       <x:c r="A226" s="17"/>
@@ -4505,8 +4961,10 @@
       <x:c r="L226" s="14"/>
       <x:c r="M226" s="14"/>
       <x:c r="N226" s="17"/>
-      <x:c r="O226" s="14"/>
-      <x:c r="P226" s="14"/>
+      <x:c r="O226" s="17"/>
+      <x:c r="P226" s="17"/>
+      <x:c r="Q226" s="14"/>
+      <x:c r="R226" s="14"/>
     </x:row>
     <x:row r="227" ht="22" customHeight="1">
       <x:c r="A227" s="17"/>
@@ -4523,8 +4981,10 @@
       <x:c r="L227" s="14"/>
       <x:c r="M227" s="14"/>
       <x:c r="N227" s="17"/>
-      <x:c r="O227" s="14"/>
-      <x:c r="P227" s="14"/>
+      <x:c r="O227" s="17"/>
+      <x:c r="P227" s="17"/>
+      <x:c r="Q227" s="14"/>
+      <x:c r="R227" s="14"/>
     </x:row>
     <x:row r="228" ht="22" customHeight="1">
       <x:c r="A228" s="17"/>
@@ -4541,8 +5001,10 @@
       <x:c r="L228" s="14"/>
       <x:c r="M228" s="14"/>
       <x:c r="N228" s="17"/>
-      <x:c r="O228" s="14"/>
-      <x:c r="P228" s="14"/>
+      <x:c r="O228" s="17"/>
+      <x:c r="P228" s="17"/>
+      <x:c r="Q228" s="14"/>
+      <x:c r="R228" s="14"/>
     </x:row>
     <x:row r="229" ht="22" customHeight="1">
       <x:c r="A229" s="17"/>
@@ -4559,8 +5021,10 @@
       <x:c r="L229" s="14"/>
       <x:c r="M229" s="14"/>
       <x:c r="N229" s="17"/>
-      <x:c r="O229" s="14"/>
-      <x:c r="P229" s="14"/>
+      <x:c r="O229" s="17"/>
+      <x:c r="P229" s="17"/>
+      <x:c r="Q229" s="14"/>
+      <x:c r="R229" s="14"/>
     </x:row>
     <x:row r="230" ht="22" customHeight="1">
       <x:c r="A230" s="17"/>
@@ -4577,8 +5041,10 @@
       <x:c r="L230" s="14"/>
       <x:c r="M230" s="14"/>
       <x:c r="N230" s="17"/>
-      <x:c r="O230" s="14"/>
-      <x:c r="P230" s="14"/>
+      <x:c r="O230" s="17"/>
+      <x:c r="P230" s="17"/>
+      <x:c r="Q230" s="14"/>
+      <x:c r="R230" s="14"/>
     </x:row>
     <x:row r="231" ht="22" customHeight="1">
       <x:c r="A231" s="17"/>
@@ -4595,8 +5061,10 @@
       <x:c r="L231" s="14"/>
       <x:c r="M231" s="14"/>
       <x:c r="N231" s="17"/>
-      <x:c r="O231" s="14"/>
-      <x:c r="P231" s="14"/>
+      <x:c r="O231" s="17"/>
+      <x:c r="P231" s="17"/>
+      <x:c r="Q231" s="14"/>
+      <x:c r="R231" s="14"/>
     </x:row>
     <x:row r="232" ht="22" customHeight="1">
       <x:c r="A232" s="17"/>
@@ -4613,8 +5081,10 @@
       <x:c r="L232" s="14"/>
       <x:c r="M232" s="14"/>
       <x:c r="N232" s="17"/>
-      <x:c r="O232" s="14"/>
-      <x:c r="P232" s="14"/>
+      <x:c r="O232" s="17"/>
+      <x:c r="P232" s="17"/>
+      <x:c r="Q232" s="14"/>
+      <x:c r="R232" s="14"/>
     </x:row>
     <x:row r="233" ht="22" customHeight="1">
       <x:c r="A233" s="17"/>
@@ -4631,8 +5101,10 @@
       <x:c r="L233" s="14"/>
       <x:c r="M233" s="14"/>
       <x:c r="N233" s="17"/>
-      <x:c r="O233" s="14"/>
-      <x:c r="P233" s="14"/>
+      <x:c r="O233" s="17"/>
+      <x:c r="P233" s="17"/>
+      <x:c r="Q233" s="14"/>
+      <x:c r="R233" s="14"/>
     </x:row>
     <x:row r="234" ht="22" customHeight="1">
       <x:c r="A234" s="17"/>
@@ -4649,8 +5121,10 @@
       <x:c r="L234" s="14"/>
       <x:c r="M234" s="14"/>
       <x:c r="N234" s="17"/>
-      <x:c r="O234" s="14"/>
-      <x:c r="P234" s="14"/>
+      <x:c r="O234" s="17"/>
+      <x:c r="P234" s="17"/>
+      <x:c r="Q234" s="14"/>
+      <x:c r="R234" s="14"/>
     </x:row>
     <x:row r="235" ht="22" customHeight="1">
       <x:c r="A235" s="17"/>
@@ -4667,8 +5141,10 @@
       <x:c r="L235" s="14"/>
       <x:c r="M235" s="14"/>
       <x:c r="N235" s="17"/>
-      <x:c r="O235" s="14"/>
-      <x:c r="P235" s="14"/>
+      <x:c r="O235" s="17"/>
+      <x:c r="P235" s="17"/>
+      <x:c r="Q235" s="14"/>
+      <x:c r="R235" s="14"/>
     </x:row>
     <x:row r="236" ht="22" customHeight="1">
       <x:c r="A236" s="17"/>
@@ -4685,8 +5161,10 @@
       <x:c r="L236" s="14"/>
       <x:c r="M236" s="14"/>
       <x:c r="N236" s="17"/>
-      <x:c r="O236" s="14"/>
-      <x:c r="P236" s="14"/>
+      <x:c r="O236" s="17"/>
+      <x:c r="P236" s="17"/>
+      <x:c r="Q236" s="14"/>
+      <x:c r="R236" s="14"/>
     </x:row>
     <x:row r="237" ht="22" customHeight="1">
       <x:c r="A237" s="17"/>
@@ -4703,8 +5181,10 @@
       <x:c r="L237" s="14"/>
       <x:c r="M237" s="14"/>
       <x:c r="N237" s="17"/>
-      <x:c r="O237" s="14"/>
-      <x:c r="P237" s="14"/>
+      <x:c r="O237" s="17"/>
+      <x:c r="P237" s="17"/>
+      <x:c r="Q237" s="14"/>
+      <x:c r="R237" s="14"/>
     </x:row>
     <x:row r="238" ht="22" customHeight="1">
       <x:c r="A238" s="17"/>
@@ -4721,8 +5201,10 @@
       <x:c r="L238" s="14"/>
       <x:c r="M238" s="14"/>
       <x:c r="N238" s="17"/>
-      <x:c r="O238" s="14"/>
-      <x:c r="P238" s="14"/>
+      <x:c r="O238" s="17"/>
+      <x:c r="P238" s="17"/>
+      <x:c r="Q238" s="14"/>
+      <x:c r="R238" s="14"/>
     </x:row>
     <x:row r="239" ht="22" customHeight="1">
       <x:c r="A239" s="17"/>
@@ -4739,8 +5221,10 @@
       <x:c r="L239" s="14"/>
       <x:c r="M239" s="14"/>
       <x:c r="N239" s="17"/>
-      <x:c r="O239" s="14"/>
-      <x:c r="P239" s="14"/>
+      <x:c r="O239" s="17"/>
+      <x:c r="P239" s="17"/>
+      <x:c r="Q239" s="14"/>
+      <x:c r="R239" s="14"/>
     </x:row>
     <x:row r="240" ht="22" customHeight="1">
       <x:c r="A240" s="17"/>
@@ -4757,8 +5241,10 @@
       <x:c r="L240" s="14"/>
       <x:c r="M240" s="14"/>
       <x:c r="N240" s="17"/>
-      <x:c r="O240" s="14"/>
-      <x:c r="P240" s="14"/>
+      <x:c r="O240" s="17"/>
+      <x:c r="P240" s="17"/>
+      <x:c r="Q240" s="14"/>
+      <x:c r="R240" s="14"/>
     </x:row>
     <x:row r="241" ht="22" customHeight="1">
       <x:c r="A241" s="17"/>
@@ -4775,8 +5261,10 @@
       <x:c r="L241" s="14"/>
       <x:c r="M241" s="14"/>
       <x:c r="N241" s="17"/>
-      <x:c r="O241" s="14"/>
-      <x:c r="P241" s="14"/>
+      <x:c r="O241" s="17"/>
+      <x:c r="P241" s="17"/>
+      <x:c r="Q241" s="14"/>
+      <x:c r="R241" s="14"/>
     </x:row>
     <x:row r="242" ht="22" customHeight="1">
       <x:c r="A242" s="17"/>
@@ -4793,8 +5281,10 @@
       <x:c r="L242" s="14"/>
       <x:c r="M242" s="14"/>
       <x:c r="N242" s="17"/>
-      <x:c r="O242" s="14"/>
-      <x:c r="P242" s="14"/>
+      <x:c r="O242" s="17"/>
+      <x:c r="P242" s="17"/>
+      <x:c r="Q242" s="14"/>
+      <x:c r="R242" s="14"/>
     </x:row>
     <x:row r="243" ht="22" customHeight="1">
       <x:c r="A243" s="17"/>
@@ -4811,8 +5301,10 @@
       <x:c r="L243" s="14"/>
       <x:c r="M243" s="14"/>
       <x:c r="N243" s="17"/>
-      <x:c r="O243" s="14"/>
-      <x:c r="P243" s="14"/>
+      <x:c r="O243" s="17"/>
+      <x:c r="P243" s="17"/>
+      <x:c r="Q243" s="14"/>
+      <x:c r="R243" s="14"/>
     </x:row>
     <x:row r="244" ht="22" customHeight="1">
       <x:c r="A244" s="17"/>
@@ -4829,8 +5321,10 @@
       <x:c r="L244" s="14"/>
       <x:c r="M244" s="14"/>
       <x:c r="N244" s="17"/>
-      <x:c r="O244" s="14"/>
-      <x:c r="P244" s="14"/>
+      <x:c r="O244" s="17"/>
+      <x:c r="P244" s="17"/>
+      <x:c r="Q244" s="14"/>
+      <x:c r="R244" s="14"/>
     </x:row>
     <x:row r="245" ht="22" customHeight="1">
       <x:c r="A245" s="17"/>
@@ -4847,8 +5341,10 @@
       <x:c r="L245" s="14"/>
       <x:c r="M245" s="14"/>
       <x:c r="N245" s="17"/>
-      <x:c r="O245" s="14"/>
-      <x:c r="P245" s="14"/>
+      <x:c r="O245" s="17"/>
+      <x:c r="P245" s="17"/>
+      <x:c r="Q245" s="14"/>
+      <x:c r="R245" s="14"/>
     </x:row>
     <x:row r="246" ht="22" customHeight="1">
       <x:c r="A246" s="17"/>
@@ -4865,8 +5361,10 @@
       <x:c r="L246" s="14"/>
       <x:c r="M246" s="14"/>
       <x:c r="N246" s="17"/>
-      <x:c r="O246" s="14"/>
-      <x:c r="P246" s="14"/>
+      <x:c r="O246" s="17"/>
+      <x:c r="P246" s="17"/>
+      <x:c r="Q246" s="14"/>
+      <x:c r="R246" s="14"/>
     </x:row>
     <x:row r="247" ht="22" customHeight="1">
       <x:c r="A247" s="17"/>
@@ -4883,8 +5381,10 @@
       <x:c r="L247" s="14"/>
       <x:c r="M247" s="14"/>
       <x:c r="N247" s="17"/>
-      <x:c r="O247" s="14"/>
-      <x:c r="P247" s="14"/>
+      <x:c r="O247" s="17"/>
+      <x:c r="P247" s="17"/>
+      <x:c r="Q247" s="14"/>
+      <x:c r="R247" s="14"/>
     </x:row>
     <x:row r="248" ht="22" customHeight="1">
       <x:c r="A248" s="17"/>
@@ -4901,8 +5401,10 @@
       <x:c r="L248" s="14"/>
       <x:c r="M248" s="14"/>
       <x:c r="N248" s="17"/>
-      <x:c r="O248" s="14"/>
-      <x:c r="P248" s="14"/>
+      <x:c r="O248" s="17"/>
+      <x:c r="P248" s="17"/>
+      <x:c r="Q248" s="14"/>
+      <x:c r="R248" s="14"/>
     </x:row>
     <x:row r="249" ht="22" customHeight="1">
       <x:c r="A249" s="17"/>
@@ -4919,8 +5421,10 @@
       <x:c r="L249" s="14"/>
       <x:c r="M249" s="14"/>
       <x:c r="N249" s="17"/>
-      <x:c r="O249" s="14"/>
-      <x:c r="P249" s="14"/>
+      <x:c r="O249" s="17"/>
+      <x:c r="P249" s="17"/>
+      <x:c r="Q249" s="14"/>
+      <x:c r="R249" s="14"/>
     </x:row>
     <x:row r="250" ht="22" customHeight="1">
       <x:c r="A250" s="17"/>
@@ -4937,8 +5441,10 @@
       <x:c r="L250" s="14"/>
       <x:c r="M250" s="14"/>
       <x:c r="N250" s="17"/>
-      <x:c r="O250" s="14"/>
-      <x:c r="P250" s="14"/>
+      <x:c r="O250" s="17"/>
+      <x:c r="P250" s="17"/>
+      <x:c r="Q250" s="14"/>
+      <x:c r="R250" s="14"/>
     </x:row>
     <x:row r="251" ht="22" customHeight="1">
       <x:c r="A251" s="17"/>
@@ -4955,8 +5461,10 @@
       <x:c r="L251" s="14"/>
       <x:c r="M251" s="14"/>
       <x:c r="N251" s="17"/>
-      <x:c r="O251" s="14"/>
-      <x:c r="P251" s="14"/>
+      <x:c r="O251" s="17"/>
+      <x:c r="P251" s="17"/>
+      <x:c r="Q251" s="14"/>
+      <x:c r="R251" s="14"/>
     </x:row>
     <x:row r="252" ht="22" customHeight="1">
       <x:c r="A252" s="17"/>
@@ -4973,8 +5481,10 @@
       <x:c r="L252" s="14"/>
       <x:c r="M252" s="14"/>
       <x:c r="N252" s="17"/>
-      <x:c r="O252" s="14"/>
-      <x:c r="P252" s="14"/>
+      <x:c r="O252" s="17"/>
+      <x:c r="P252" s="17"/>
+      <x:c r="Q252" s="14"/>
+      <x:c r="R252" s="14"/>
     </x:row>
     <x:row r="253" ht="22" customHeight="1">
       <x:c r="A253" s="17"/>
@@ -4991,8 +5501,10 @@
       <x:c r="L253" s="14"/>
       <x:c r="M253" s="14"/>
       <x:c r="N253" s="17"/>
-      <x:c r="O253" s="14"/>
-      <x:c r="P253" s="14"/>
+      <x:c r="O253" s="17"/>
+      <x:c r="P253" s="17"/>
+      <x:c r="Q253" s="14"/>
+      <x:c r="R253" s="14"/>
     </x:row>
     <x:row r="254" ht="22" customHeight="1">
       <x:c r="A254" s="17"/>
@@ -5009,8 +5521,10 @@
       <x:c r="L254" s="14"/>
       <x:c r="M254" s="14"/>
       <x:c r="N254" s="17"/>
-      <x:c r="O254" s="14"/>
-      <x:c r="P254" s="14"/>
+      <x:c r="O254" s="17"/>
+      <x:c r="P254" s="17"/>
+      <x:c r="Q254" s="14"/>
+      <x:c r="R254" s="14"/>
     </x:row>
     <x:row r="255" ht="22" customHeight="1">
       <x:c r="A255" s="17"/>
@@ -5027,8 +5541,10 @@
       <x:c r="L255" s="14"/>
       <x:c r="M255" s="14"/>
       <x:c r="N255" s="17"/>
-      <x:c r="O255" s="14"/>
-      <x:c r="P255" s="14"/>
+      <x:c r="O255" s="17"/>
+      <x:c r="P255" s="17"/>
+      <x:c r="Q255" s="14"/>
+      <x:c r="R255" s="14"/>
     </x:row>
     <x:row r="256" ht="22" customHeight="1">
       <x:c r="A256" s="17"/>
@@ -5045,8 +5561,10 @@
       <x:c r="L256" s="14"/>
       <x:c r="M256" s="14"/>
       <x:c r="N256" s="17"/>
-      <x:c r="O256" s="14"/>
-      <x:c r="P256" s="14"/>
+      <x:c r="O256" s="17"/>
+      <x:c r="P256" s="17"/>
+      <x:c r="Q256" s="14"/>
+      <x:c r="R256" s="14"/>
     </x:row>
     <x:row r="257" ht="22" customHeight="1">
       <x:c r="A257" s="17"/>
@@ -5063,8 +5581,10 @@
       <x:c r="L257" s="14"/>
       <x:c r="M257" s="14"/>
       <x:c r="N257" s="17"/>
-      <x:c r="O257" s="14"/>
-      <x:c r="P257" s="14"/>
+      <x:c r="O257" s="17"/>
+      <x:c r="P257" s="17"/>
+      <x:c r="Q257" s="14"/>
+      <x:c r="R257" s="14"/>
     </x:row>
     <x:row r="258" ht="22" customHeight="1">
       <x:c r="A258" s="17"/>
@@ -5081,8 +5601,10 @@
       <x:c r="L258" s="14"/>
       <x:c r="M258" s="14"/>
       <x:c r="N258" s="17"/>
-      <x:c r="O258" s="14"/>
-      <x:c r="P258" s="14"/>
+      <x:c r="O258" s="17"/>
+      <x:c r="P258" s="17"/>
+      <x:c r="Q258" s="14"/>
+      <x:c r="R258" s="14"/>
     </x:row>
     <x:row r="259" ht="22" customHeight="1">
       <x:c r="A259" s="17"/>
@@ -5099,8 +5621,10 @@
       <x:c r="L259" s="14"/>
       <x:c r="M259" s="14"/>
       <x:c r="N259" s="17"/>
-      <x:c r="O259" s="14"/>
-      <x:c r="P259" s="14"/>
+      <x:c r="O259" s="17"/>
+      <x:c r="P259" s="17"/>
+      <x:c r="Q259" s="14"/>
+      <x:c r="R259" s="14"/>
     </x:row>
     <x:row r="260" ht="22" customHeight="1">
       <x:c r="A260" s="17"/>
@@ -5117,8 +5641,10 @@
       <x:c r="L260" s="14"/>
       <x:c r="M260" s="14"/>
       <x:c r="N260" s="17"/>
-      <x:c r="O260" s="14"/>
-      <x:c r="P260" s="14"/>
+      <x:c r="O260" s="17"/>
+      <x:c r="P260" s="17"/>
+      <x:c r="Q260" s="14"/>
+      <x:c r="R260" s="14"/>
     </x:row>
     <x:row r="261" ht="22" customHeight="1">
       <x:c r="A261" s="17"/>
@@ -5135,8 +5661,10 @@
       <x:c r="L261" s="14"/>
       <x:c r="M261" s="14"/>
       <x:c r="N261" s="17"/>
-      <x:c r="O261" s="14"/>
-      <x:c r="P261" s="14"/>
+      <x:c r="O261" s="17"/>
+      <x:c r="P261" s="17"/>
+      <x:c r="Q261" s="14"/>
+      <x:c r="R261" s="14"/>
     </x:row>
     <x:row r="262" ht="22" customHeight="1">
       <x:c r="A262" s="17"/>
@@ -5153,8 +5681,10 @@
       <x:c r="L262" s="14"/>
       <x:c r="M262" s="14"/>
       <x:c r="N262" s="17"/>
-      <x:c r="O262" s="14"/>
-      <x:c r="P262" s="14"/>
+      <x:c r="O262" s="17"/>
+      <x:c r="P262" s="17"/>
+      <x:c r="Q262" s="14"/>
+      <x:c r="R262" s="14"/>
     </x:row>
     <x:row r="263" ht="22" customHeight="1">
       <x:c r="A263" s="17"/>
@@ -5171,8 +5701,10 @@
       <x:c r="L263" s="14"/>
       <x:c r="M263" s="14"/>
       <x:c r="N263" s="17"/>
-      <x:c r="O263" s="14"/>
-      <x:c r="P263" s="14"/>
+      <x:c r="O263" s="17"/>
+      <x:c r="P263" s="17"/>
+      <x:c r="Q263" s="14"/>
+      <x:c r="R263" s="14"/>
     </x:row>
     <x:row r="264" ht="22" customHeight="1">
       <x:c r="A264" s="17"/>
@@ -5189,8 +5721,10 @@
       <x:c r="L264" s="14"/>
       <x:c r="M264" s="14"/>
       <x:c r="N264" s="17"/>
-      <x:c r="O264" s="14"/>
-      <x:c r="P264" s="14"/>
+      <x:c r="O264" s="17"/>
+      <x:c r="P264" s="17"/>
+      <x:c r="Q264" s="14"/>
+      <x:c r="R264" s="14"/>
     </x:row>
     <x:row r="265" ht="22" customHeight="1">
       <x:c r="A265" s="17"/>
@@ -5207,8 +5741,10 @@
       <x:c r="L265" s="14"/>
       <x:c r="M265" s="14"/>
       <x:c r="N265" s="17"/>
-      <x:c r="O265" s="14"/>
-      <x:c r="P265" s="14"/>
+      <x:c r="O265" s="17"/>
+      <x:c r="P265" s="17"/>
+      <x:c r="Q265" s="14"/>
+      <x:c r="R265" s="14"/>
     </x:row>
     <x:row r="266" ht="22" customHeight="1">
       <x:c r="A266" s="17"/>
@@ -5225,8 +5761,10 @@
       <x:c r="L266" s="14"/>
       <x:c r="M266" s="14"/>
       <x:c r="N266" s="17"/>
-      <x:c r="O266" s="14"/>
-      <x:c r="P266" s="14"/>
+      <x:c r="O266" s="17"/>
+      <x:c r="P266" s="17"/>
+      <x:c r="Q266" s="14"/>
+      <x:c r="R266" s="14"/>
     </x:row>
     <x:row r="267" ht="22" customHeight="1">
       <x:c r="A267" s="17"/>
@@ -5243,8 +5781,10 @@
       <x:c r="L267" s="14"/>
       <x:c r="M267" s="14"/>
       <x:c r="N267" s="17"/>
-      <x:c r="O267" s="14"/>
-      <x:c r="P267" s="14"/>
+      <x:c r="O267" s="17"/>
+      <x:c r="P267" s="17"/>
+      <x:c r="Q267" s="14"/>
+      <x:c r="R267" s="14"/>
     </x:row>
     <x:row r="268" ht="22" customHeight="1">
       <x:c r="A268" s="17"/>
@@ -5261,8 +5801,10 @@
       <x:c r="L268" s="14"/>
       <x:c r="M268" s="14"/>
       <x:c r="N268" s="17"/>
-      <x:c r="O268" s="14"/>
-      <x:c r="P268" s="14"/>
+      <x:c r="O268" s="17"/>
+      <x:c r="P268" s="17"/>
+      <x:c r="Q268" s="14"/>
+      <x:c r="R268" s="14"/>
     </x:row>
     <x:row r="269" ht="22" customHeight="1">
       <x:c r="A269" s="17"/>
@@ -5279,8 +5821,10 @@
       <x:c r="L269" s="14"/>
       <x:c r="M269" s="14"/>
       <x:c r="N269" s="17"/>
-      <x:c r="O269" s="14"/>
-      <x:c r="P269" s="14"/>
+      <x:c r="O269" s="17"/>
+      <x:c r="P269" s="17"/>
+      <x:c r="Q269" s="14"/>
+      <x:c r="R269" s="14"/>
     </x:row>
     <x:row r="270" ht="22" customHeight="1">
       <x:c r="A270" s="17"/>
@@ -5297,8 +5841,10 @@
       <x:c r="L270" s="14"/>
       <x:c r="M270" s="14"/>
       <x:c r="N270" s="17"/>
-      <x:c r="O270" s="14"/>
-      <x:c r="P270" s="14"/>
+      <x:c r="O270" s="17"/>
+      <x:c r="P270" s="17"/>
+      <x:c r="Q270" s="14"/>
+      <x:c r="R270" s="14"/>
     </x:row>
     <x:row r="271" ht="22" customHeight="1">
       <x:c r="A271" s="17"/>
@@ -5315,8 +5861,10 @@
       <x:c r="L271" s="14"/>
       <x:c r="M271" s="14"/>
       <x:c r="N271" s="17"/>
-      <x:c r="O271" s="14"/>
-      <x:c r="P271" s="14"/>
+      <x:c r="O271" s="17"/>
+      <x:c r="P271" s="17"/>
+      <x:c r="Q271" s="14"/>
+      <x:c r="R271" s="14"/>
     </x:row>
     <x:row r="272" ht="22" customHeight="1">
       <x:c r="A272" s="17"/>
@@ -5333,8 +5881,10 @@
       <x:c r="L272" s="14"/>
       <x:c r="M272" s="14"/>
       <x:c r="N272" s="17"/>
-      <x:c r="O272" s="14"/>
-      <x:c r="P272" s="14"/>
+      <x:c r="O272" s="17"/>
+      <x:c r="P272" s="17"/>
+      <x:c r="Q272" s="14"/>
+      <x:c r="R272" s="14"/>
     </x:row>
     <x:row r="273" ht="22" customHeight="1">
       <x:c r="A273" s="17"/>
@@ -5351,8 +5901,10 @@
       <x:c r="L273" s="14"/>
       <x:c r="M273" s="14"/>
       <x:c r="N273" s="17"/>
-      <x:c r="O273" s="14"/>
-      <x:c r="P273" s="14"/>
+      <x:c r="O273" s="17"/>
+      <x:c r="P273" s="17"/>
+      <x:c r="Q273" s="14"/>
+      <x:c r="R273" s="14"/>
     </x:row>
     <x:row r="274" ht="22" customHeight="1">
       <x:c r="A274" s="17"/>
@@ -5369,8 +5921,10 @@
       <x:c r="L274" s="14"/>
       <x:c r="M274" s="14"/>
       <x:c r="N274" s="17"/>
-      <x:c r="O274" s="14"/>
-      <x:c r="P274" s="14"/>
+      <x:c r="O274" s="17"/>
+      <x:c r="P274" s="17"/>
+      <x:c r="Q274" s="14"/>
+      <x:c r="R274" s="14"/>
     </x:row>
     <x:row r="275" ht="22" customHeight="1">
       <x:c r="A275" s="17"/>
@@ -5387,8 +5941,10 @@
       <x:c r="L275" s="14"/>
       <x:c r="M275" s="14"/>
       <x:c r="N275" s="17"/>
-      <x:c r="O275" s="14"/>
-      <x:c r="P275" s="14"/>
+      <x:c r="O275" s="17"/>
+      <x:c r="P275" s="17"/>
+      <x:c r="Q275" s="14"/>
+      <x:c r="R275" s="14"/>
     </x:row>
     <x:row r="276" ht="22" customHeight="1">
       <x:c r="A276" s="17"/>
@@ -5405,8 +5961,10 @@
       <x:c r="L276" s="14"/>
       <x:c r="M276" s="14"/>
       <x:c r="N276" s="17"/>
-      <x:c r="O276" s="14"/>
-      <x:c r="P276" s="14"/>
+      <x:c r="O276" s="17"/>
+      <x:c r="P276" s="17"/>
+      <x:c r="Q276" s="14"/>
+      <x:c r="R276" s="14"/>
     </x:row>
     <x:row r="277" ht="22" customHeight="1">
       <x:c r="A277" s="17"/>
@@ -5423,8 +5981,10 @@
       <x:c r="L277" s="14"/>
       <x:c r="M277" s="14"/>
       <x:c r="N277" s="17"/>
-      <x:c r="O277" s="14"/>
-      <x:c r="P277" s="14"/>
+      <x:c r="O277" s="17"/>
+      <x:c r="P277" s="17"/>
+      <x:c r="Q277" s="14"/>
+      <x:c r="R277" s="14"/>
     </x:row>
     <x:row r="278" ht="22" customHeight="1">
       <x:c r="A278" s="17"/>
@@ -5441,8 +6001,10 @@
       <x:c r="L278" s="14"/>
       <x:c r="M278" s="14"/>
       <x:c r="N278" s="17"/>
-      <x:c r="O278" s="14"/>
-      <x:c r="P278" s="14"/>
+      <x:c r="O278" s="17"/>
+      <x:c r="P278" s="17"/>
+      <x:c r="Q278" s="14"/>
+      <x:c r="R278" s="14"/>
     </x:row>
     <x:row r="279" ht="22" customHeight="1">
       <x:c r="A279" s="17"/>
@@ -5459,8 +6021,10 @@
       <x:c r="L279" s="14"/>
       <x:c r="M279" s="14"/>
       <x:c r="N279" s="17"/>
-      <x:c r="O279" s="14"/>
-      <x:c r="P279" s="14"/>
+      <x:c r="O279" s="17"/>
+      <x:c r="P279" s="17"/>
+      <x:c r="Q279" s="14"/>
+      <x:c r="R279" s="14"/>
     </x:row>
     <x:row r="280" ht="22" customHeight="1">
       <x:c r="A280" s="17"/>
@@ -5477,8 +6041,10 @@
       <x:c r="L280" s="14"/>
       <x:c r="M280" s="14"/>
       <x:c r="N280" s="17"/>
-      <x:c r="O280" s="14"/>
-      <x:c r="P280" s="14"/>
+      <x:c r="O280" s="17"/>
+      <x:c r="P280" s="17"/>
+      <x:c r="Q280" s="14"/>
+      <x:c r="R280" s="14"/>
     </x:row>
     <x:row r="281" ht="22" customHeight="1">
       <x:c r="A281" s="17"/>
@@ -5495,8 +6061,10 @@
       <x:c r="L281" s="14"/>
       <x:c r="M281" s="14"/>
       <x:c r="N281" s="17"/>
-      <x:c r="O281" s="14"/>
-      <x:c r="P281" s="14"/>
+      <x:c r="O281" s="17"/>
+      <x:c r="P281" s="17"/>
+      <x:c r="Q281" s="14"/>
+      <x:c r="R281" s="14"/>
     </x:row>
     <x:row r="282" ht="22" customHeight="1">
       <x:c r="A282" s="17"/>
@@ -5513,8 +6081,10 @@
       <x:c r="L282" s="14"/>
       <x:c r="M282" s="14"/>
       <x:c r="N282" s="17"/>
-      <x:c r="O282" s="14"/>
-      <x:c r="P282" s="14"/>
+      <x:c r="O282" s="17"/>
+      <x:c r="P282" s="17"/>
+      <x:c r="Q282" s="14"/>
+      <x:c r="R282" s="14"/>
     </x:row>
     <x:row r="283" ht="22" customHeight="1">
       <x:c r="A283" s="17"/>
@@ -5531,8 +6101,10 @@
       <x:c r="L283" s="14"/>
       <x:c r="M283" s="14"/>
       <x:c r="N283" s="17"/>
-      <x:c r="O283" s="14"/>
-      <x:c r="P283" s="14"/>
+      <x:c r="O283" s="17"/>
+      <x:c r="P283" s="17"/>
+      <x:c r="Q283" s="14"/>
+      <x:c r="R283" s="14"/>
     </x:row>
     <x:row r="284" ht="22" customHeight="1">
       <x:c r="A284" s="17"/>
@@ -5549,8 +6121,10 @@
       <x:c r="L284" s="14"/>
       <x:c r="M284" s="14"/>
       <x:c r="N284" s="17"/>
-      <x:c r="O284" s="14"/>
-      <x:c r="P284" s="14"/>
+      <x:c r="O284" s="17"/>
+      <x:c r="P284" s="17"/>
+      <x:c r="Q284" s="14"/>
+      <x:c r="R284" s="14"/>
     </x:row>
     <x:row r="285" ht="22" customHeight="1">
       <x:c r="A285" s="17"/>
@@ -5567,8 +6141,10 @@
       <x:c r="L285" s="14"/>
       <x:c r="M285" s="14"/>
       <x:c r="N285" s="17"/>
-      <x:c r="O285" s="14"/>
-      <x:c r="P285" s="14"/>
+      <x:c r="O285" s="17"/>
+      <x:c r="P285" s="17"/>
+      <x:c r="Q285" s="14"/>
+      <x:c r="R285" s="14"/>
     </x:row>
     <x:row r="286" ht="22" customHeight="1">
       <x:c r="A286" s="17"/>
@@ -5585,8 +6161,10 @@
       <x:c r="L286" s="14"/>
       <x:c r="M286" s="14"/>
       <x:c r="N286" s="17"/>
-      <x:c r="O286" s="14"/>
-      <x:c r="P286" s="14"/>
+      <x:c r="O286" s="17"/>
+      <x:c r="P286" s="17"/>
+      <x:c r="Q286" s="14"/>
+      <x:c r="R286" s="14"/>
     </x:row>
     <x:row r="287" ht="22" customHeight="1">
       <x:c r="A287" s="17"/>
@@ -5603,8 +6181,10 @@
       <x:c r="L287" s="14"/>
       <x:c r="M287" s="14"/>
       <x:c r="N287" s="17"/>
-      <x:c r="O287" s="14"/>
-      <x:c r="P287" s="14"/>
+      <x:c r="O287" s="17"/>
+      <x:c r="P287" s="17"/>
+      <x:c r="Q287" s="14"/>
+      <x:c r="R287" s="14"/>
     </x:row>
     <x:row r="288" ht="22" customHeight="1">
       <x:c r="A288" s="17"/>
@@ -5621,8 +6201,10 @@
       <x:c r="L288" s="14"/>
       <x:c r="M288" s="14"/>
       <x:c r="N288" s="17"/>
-      <x:c r="O288" s="14"/>
-      <x:c r="P288" s="14"/>
+      <x:c r="O288" s="17"/>
+      <x:c r="P288" s="17"/>
+      <x:c r="Q288" s="14"/>
+      <x:c r="R288" s="14"/>
     </x:row>
     <x:row r="289" ht="22" customHeight="1">
       <x:c r="A289" s="17"/>
@@ -5639,8 +6221,10 @@
       <x:c r="L289" s="14"/>
       <x:c r="M289" s="14"/>
       <x:c r="N289" s="17"/>
-      <x:c r="O289" s="14"/>
-      <x:c r="P289" s="14"/>
+      <x:c r="O289" s="17"/>
+      <x:c r="P289" s="17"/>
+      <x:c r="Q289" s="14"/>
+      <x:c r="R289" s="14"/>
     </x:row>
     <x:row r="290" ht="22" customHeight="1">
       <x:c r="A290" s="17"/>
@@ -5657,8 +6241,10 @@
       <x:c r="L290" s="14"/>
       <x:c r="M290" s="14"/>
       <x:c r="N290" s="17"/>
-      <x:c r="O290" s="14"/>
-      <x:c r="P290" s="14"/>
+      <x:c r="O290" s="17"/>
+      <x:c r="P290" s="17"/>
+      <x:c r="Q290" s="14"/>
+      <x:c r="R290" s="14"/>
     </x:row>
     <x:row r="291" ht="22" customHeight="1">
       <x:c r="A291" s="17"/>
@@ -5675,8 +6261,10 @@
       <x:c r="L291" s="14"/>
       <x:c r="M291" s="14"/>
       <x:c r="N291" s="17"/>
-      <x:c r="O291" s="14"/>
-      <x:c r="P291" s="14"/>
+      <x:c r="O291" s="17"/>
+      <x:c r="P291" s="17"/>
+      <x:c r="Q291" s="14"/>
+      <x:c r="R291" s="14"/>
     </x:row>
     <x:row r="292" ht="22" customHeight="1">
       <x:c r="A292" s="17"/>
@@ -5693,8 +6281,10 @@
       <x:c r="L292" s="14"/>
       <x:c r="M292" s="14"/>
       <x:c r="N292" s="17"/>
-      <x:c r="O292" s="14"/>
-      <x:c r="P292" s="14"/>
+      <x:c r="O292" s="17"/>
+      <x:c r="P292" s="17"/>
+      <x:c r="Q292" s="14"/>
+      <x:c r="R292" s="14"/>
     </x:row>
     <x:row r="293" ht="22" customHeight="1">
       <x:c r="A293" s="17"/>
@@ -5711,8 +6301,10 @@
       <x:c r="L293" s="14"/>
       <x:c r="M293" s="14"/>
       <x:c r="N293" s="17"/>
-      <x:c r="O293" s="14"/>
-      <x:c r="P293" s="14"/>
+      <x:c r="O293" s="17"/>
+      <x:c r="P293" s="17"/>
+      <x:c r="Q293" s="14"/>
+      <x:c r="R293" s="14"/>
     </x:row>
     <x:row r="294" ht="22" customHeight="1">
       <x:c r="A294" s="17"/>
@@ -5729,8 +6321,10 @@
       <x:c r="L294" s="14"/>
       <x:c r="M294" s="14"/>
       <x:c r="N294" s="17"/>
-      <x:c r="O294" s="14"/>
-      <x:c r="P294" s="14"/>
+      <x:c r="O294" s="17"/>
+      <x:c r="P294" s="17"/>
+      <x:c r="Q294" s="14"/>
+      <x:c r="R294" s="14"/>
     </x:row>
     <x:row r="295" ht="22" customHeight="1">
       <x:c r="A295" s="17"/>
@@ -5747,8 +6341,10 @@
       <x:c r="L295" s="14"/>
       <x:c r="M295" s="14"/>
       <x:c r="N295" s="17"/>
-      <x:c r="O295" s="14"/>
-      <x:c r="P295" s="14"/>
+      <x:c r="O295" s="17"/>
+      <x:c r="P295" s="17"/>
+      <x:c r="Q295" s="14"/>
+      <x:c r="R295" s="14"/>
     </x:row>
     <x:row r="296" ht="22" customHeight="1">
       <x:c r="A296" s="17"/>
@@ -5765,8 +6361,10 @@
       <x:c r="L296" s="14"/>
       <x:c r="M296" s="14"/>
       <x:c r="N296" s="17"/>
-      <x:c r="O296" s="14"/>
-      <x:c r="P296" s="14"/>
+      <x:c r="O296" s="17"/>
+      <x:c r="P296" s="17"/>
+      <x:c r="Q296" s="14"/>
+      <x:c r="R296" s="14"/>
     </x:row>
     <x:row r="297" ht="22" customHeight="1">
       <x:c r="A297" s="17"/>
@@ -5783,8 +6381,10 @@
       <x:c r="L297" s="14"/>
       <x:c r="M297" s="14"/>
       <x:c r="N297" s="17"/>
-      <x:c r="O297" s="14"/>
-      <x:c r="P297" s="14"/>
+      <x:c r="O297" s="17"/>
+      <x:c r="P297" s="17"/>
+      <x:c r="Q297" s="14"/>
+      <x:c r="R297" s="14"/>
     </x:row>
     <x:row r="298" ht="22" customHeight="1">
       <x:c r="A298" s="17"/>
@@ -5801,8 +6401,10 @@
       <x:c r="L298" s="14"/>
       <x:c r="M298" s="14"/>
       <x:c r="N298" s="17"/>
-      <x:c r="O298" s="14"/>
-      <x:c r="P298" s="14"/>
+      <x:c r="O298" s="17"/>
+      <x:c r="P298" s="17"/>
+      <x:c r="Q298" s="14"/>
+      <x:c r="R298" s="14"/>
     </x:row>
     <x:row r="299" ht="22" customHeight="1">
       <x:c r="A299" s="17"/>
@@ -5819,8 +6421,10 @@
       <x:c r="L299" s="14"/>
       <x:c r="M299" s="14"/>
       <x:c r="N299" s="17"/>
-      <x:c r="O299" s="14"/>
-      <x:c r="P299" s="14"/>
+      <x:c r="O299" s="17"/>
+      <x:c r="P299" s="17"/>
+      <x:c r="Q299" s="14"/>
+      <x:c r="R299" s="14"/>
     </x:row>
     <x:row r="300" ht="22" customHeight="1">
       <x:c r="A300" s="17"/>
@@ -5837,8 +6441,10 @@
       <x:c r="L300" s="14"/>
       <x:c r="M300" s="14"/>
       <x:c r="N300" s="17"/>
-      <x:c r="O300" s="14"/>
-      <x:c r="P300" s="14"/>
+      <x:c r="O300" s="17"/>
+      <x:c r="P300" s="17"/>
+      <x:c r="Q300" s="14"/>
+      <x:c r="R300" s="14"/>
     </x:row>
     <x:row r="301" ht="22" customHeight="1">
       <x:c r="A301" s="18"/>
@@ -5855,11 +6461,13 @@
       <x:c r="L301" s="15"/>
       <x:c r="M301" s="15"/>
       <x:c r="N301" s="18"/>
-      <x:c r="O301" s="15"/>
-      <x:c r="P301" s="15"/>
+      <x:c r="O301" s="18"/>
+      <x:c r="P301" s="18"/>
+      <x:c r="Q301" s="15"/>
+      <x:c r="R301" s="15"/>
     </x:row>
   </x:sheetData>
-  <x:dataValidations count="3">
+  <x:dataValidations count="5">
     <x:dataValidation type="list" sqref="A2:A301">
       <x:formula1>"DNI,CE"</x:formula1>
     </x:dataValidation>
@@ -5867,6 +6475,12 @@
       <x:formula1>"SIN REI,01,02,03,04,05,06,07,08,09,10,11,12,13,14,15,16,17,18,19"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="P2:P301">
+      <x:formula1>"EBR,EBE,EBA,PRONOEI"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="Q2:Q301">
+      <x:formula1>"director_iiee,user,jefe_area,director,responsable_cdd,admin"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="R2:R301">
       <x:formula1>"SI,NO"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -5975,7 +6589,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B7" s="31" t="str">
-        <x:v>Nombres, apellidos y datos descriptivos se normalizan a MAYÚSCULAS. El correo debe ser @ugel06.gob.pe y se conserva en minúsculas.</x:v>
+        <x:v>Nombres, apellidos y datos descriptivos se normalizan a MAYÚSCULAS.</x:v>
       </x:c>
       <x:c r="C7" s="31"/>
       <x:c r="D7" s="31"/>
@@ -6011,7 +6625,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="B10" s="31" t="str">
-        <x:v>Rol: usa el código del rol, por ejemplo user o director_iiee. También se aceptan roles activos creados en el sistema.</x:v>
+        <x:v>Antes de cargar Directores IIEE, el administrador debe sincronizar las plazas desde Usuarios &gt; Plazas Director IIEE.</x:v>
       </x:c>
       <x:c r="C10" s="31"/>
       <x:c r="D10" s="31"/>
@@ -6023,7 +6637,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="B11" s="31" t="str">
-        <x:v>Código institucional: exactamente 8 dígitos, por ejemplo 25642929. Es obligatorio solo para director_iiee y se conserva como texto si inicia con 0.</x:v>
+        <x:v>Para director_iiee: código institucional (8 dígitos), nombre del colegio como referencia y modalidad son obligatorios.</x:v>
       </x:c>
       <x:c r="C11" s="31"/>
       <x:c r="D11" s="31"/>
@@ -6035,7 +6649,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="B12" s="31" t="str">
-        <x:v>REI: usa 01, 02, 03... hasta 19, o SIN REI. can_create_monitoreo: escribe SI o NO.</x:v>
+        <x:v>Para director_iiee deja correo y REI vacíos: el sistema usa el alias y la REI oficial de la plaza. can_create_monitoreo siempre será NO.</x:v>
       </x:c>
       <x:c r="C12" s="31"/>
       <x:c r="D12" s="31"/>
@@ -6047,52 +6661,86 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="B13" s="31" t="str">
-        <x:v>No agregues una columna de contraseña. El sistema la genera desde el apellido paterno (QUISPE → Quispe123@@) y exige cambiarla en el primer ingreso.</x:v>
+        <x:v>Para otros roles: correo @ugel06.gob.pe y rol son obligatorios; no llenes código institucional, nombre del colegio ni modalidad.</x:v>
       </x:c>
       <x:c r="C13" s="31"/>
       <x:c r="D13" s="31"/>
       <x:c r="E13" s="31"/>
       <x:c r="F13" s="31"/>
     </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="25" t="str">
+    <x:row r="14" ht="34" customHeight="1">
+      <x:c r="A14" s="28" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B14" s="31" t="str">
+        <x:v>REI usa 01, 02, 03... hasta 19 o SIN REI. El código institucional se conserva como texto si empieza con 0.</x:v>
+      </x:c>
+      <x:c r="C14" s="31"/>
+      <x:c r="D14" s="31"/>
+      <x:c r="E14" s="31"/>
+      <x:c r="F14" s="31"/>
+    </x:row>
+    <x:row r="15" ht="34" customHeight="1">
+      <x:c r="A15" s="28" t="str">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B15" s="31" t="str">
+        <x:v>No agregues contraseña. El sistema la genera desde el apellido paterno (QUISPE → Quispe123@@) y exige cambiarla en el primer ingreso.</x:v>
+      </x:c>
+      <x:c r="C15" s="31"/>
+      <x:c r="D15" s="31"/>
+      <x:c r="E15" s="31"/>
+      <x:c r="F15" s="31"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="25" t="str">
         <x:v>Campos obligatorios</x:v>
       </x:c>
-      <x:c r="B15" s="25" t="str">
+      <x:c r="B17" s="25" t="str">
         <x:v>Campos obligatorios</x:v>
       </x:c>
-      <x:c r="C15" s="25" t="str">
+      <x:c r="C17" s="25" t="str">
         <x:v>Campos obligatorios</x:v>
       </x:c>
-      <x:c r="D15" s="25" t="str">
+      <x:c r="D17" s="25" t="str">
         <x:v>Campos obligatorios</x:v>
       </x:c>
-      <x:c r="E15" s="25" t="str">
+      <x:c r="E17" s="25" t="str">
         <x:v>Campos obligatorios</x:v>
       </x:c>
-      <x:c r="F15" s="25" t="str">
+      <x:c r="F17" s="25" t="str">
         <x:v>Campos obligatorios</x:v>
       </x:c>
     </x:row>
-    <x:row r="16" ht="32" customHeight="1">
-      <x:c r="A16" s="30" t="str">
-        <x:v>tipo_documento, numero_documento, apellido_paterno, apellido_materno, nombres, correo y rol</x:v>
+    <x:row r="18" ht="32" customHeight="1">
+      <x:c r="A18" s="30" t="str">
+        <x:v>Todos: tipo_documento, numero_documento, apellido_paterno, apellido_materno, nombres y rol.</x:v>
       </x:c>
-      <x:c r="B16" s="30"/>
-      <x:c r="C16" s="30"/>
-      <x:c r="D16" s="30"/>
-      <x:c r="E16" s="30"/>
-      <x:c r="F16" s="30"/>
-    </x:row>
-    <x:row r="17" ht="32" customHeight="1">
-      <x:c r="A17" s="30" t="str">
-        <x:v>codigo_institucional es obligatorio únicamente para director_iiee. Los demás campos son opcionales; UGEL se completa como UGEL 06 y REI como SIN REI.</x:v>
+      <x:c r="B18" s="30"/>
+      <x:c r="C18" s="30"/>
+      <x:c r="D18" s="30"/>
+      <x:c r="E18" s="30"/>
+      <x:c r="F18" s="30"/>
+    </x:row>
+    <x:row r="19" ht="32" customHeight="1">
+      <x:c r="A19" s="30" t="str">
+        <x:v>Director IIEE: codigo_institucional, nombre_colegio_referencia y modalidad. Correo, REI y permisos se obtienen de la plaza.</x:v>
       </x:c>
-      <x:c r="B17" s="30"/>
-      <x:c r="C17" s="30"/>
-      <x:c r="D17" s="30"/>
-      <x:c r="E17" s="30"/>
-      <x:c r="F17" s="30"/>
+      <x:c r="B19" s="30"/>
+      <x:c r="C19" s="30"/>
+      <x:c r="D19" s="30"/>
+      <x:c r="E19" s="30"/>
+      <x:c r="F19" s="30"/>
+    </x:row>
+    <x:row r="20" ht="32" customHeight="1">
+      <x:c r="A20" s="30" t="str">
+        <x:v>Otros roles: correo. Los demás campos son opcionales; UGEL se completa como UGEL 06.</x:v>
+      </x:c>
+      <x:c r="B20" s="30"/>
+      <x:c r="C20" s="30"/>
+      <x:c r="D20" s="30"/>
+      <x:c r="E20" s="30"/>
+      <x:c r="F20" s="30"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -6107,9 +6755,12 @@
     <x:mergeCell ref="B11:F11"/>
     <x:mergeCell ref="B12:F12"/>
     <x:mergeCell ref="B13:F13"/>
-    <x:mergeCell ref="A15:F15"/>
-    <x:mergeCell ref="A16:F16"/>
+    <x:mergeCell ref="B14:F14"/>
+    <x:mergeCell ref="B15:F15"/>
     <x:mergeCell ref="A17:F17"/>
+    <x:mergeCell ref="A18:F18"/>
+    <x:mergeCell ref="A19:F19"/>
+    <x:mergeCell ref="A20:F20"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>